<commit_message>
bot session end 2026-10-13 16:02
</commit_message>
<xml_diff>
--- a/reports/Paper Bot Live.xlsx
+++ b/reports/Paper Bot Live.xlsx
@@ -1270,7 +1270,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BA22"/>
+  <dimension ref="A1:BA23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4761,8 +4761,14 @@
           <t>off</t>
         </is>
       </c>
-      <c r="H21" s="2" t="n"/>
-      <c r="I21" s="2" t="n"/>
+      <c r="H21" s="2" t="n">
+        <v>-1.762</v>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
           <t>eod_squeeze</t>
@@ -4816,8 +4822,12 @@
       <c r="Z21" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA21" s="2" t="n"/>
-      <c r="AB21" s="2" t="n"/>
+      <c r="AA21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB21" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="AC21" s="2" t="n"/>
       <c r="AD21" s="2" t="n"/>
       <c r="AE21" s="2" t="n"/>
@@ -4842,7 +4852,9 @@
       <c r="AX21" s="2" t="n"/>
       <c r="AY21" s="2" t="n"/>
       <c r="AZ21" s="2" t="n"/>
-      <c r="BA21" s="2" t="n"/>
+      <c r="BA21" s="2" t="n">
+        <v>0.00346</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -4874,8 +4886,14 @@
           <t>off</t>
         </is>
       </c>
-      <c r="H22" s="2" t="n"/>
-      <c r="I22" s="2" t="n"/>
+      <c r="H22" s="2" t="n">
+        <v>-1.138</v>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
           <t>eod_squeeze</t>
@@ -4929,33 +4947,200 @@
       <c r="Z22" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA22" s="2" t="n"/>
-      <c r="AB22" s="2" t="n"/>
-      <c r="AC22" s="2" t="n"/>
-      <c r="AD22" s="2" t="n"/>
-      <c r="AE22" s="2" t="n"/>
-      <c r="AF22" s="2" t="n"/>
-      <c r="AG22" s="2" t="n"/>
-      <c r="AH22" s="2" t="n"/>
-      <c r="AI22" s="2" t="n"/>
-      <c r="AJ22" s="2" t="n"/>
-      <c r="AK22" s="2" t="n"/>
-      <c r="AL22" s="2" t="n"/>
-      <c r="AM22" s="2" t="n"/>
-      <c r="AN22" s="2" t="n"/>
-      <c r="AO22" s="2" t="n"/>
-      <c r="AP22" s="2" t="n"/>
-      <c r="AQ22" s="2" t="n"/>
-      <c r="AR22" s="2" t="n"/>
-      <c r="AS22" s="2" t="n"/>
-      <c r="AT22" s="2" t="n"/>
-      <c r="AU22" s="2" t="n"/>
-      <c r="AV22" s="2" t="n"/>
-      <c r="AW22" s="2" t="n"/>
-      <c r="AX22" s="2" t="n"/>
-      <c r="AY22" s="2" t="n"/>
-      <c r="AZ22" s="2" t="n"/>
-      <c r="BA22" s="2" t="n"/>
+      <c r="AA22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC22" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AD22" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE22" s="2" t="n">
+        <v>8.225</v>
+      </c>
+      <c r="AF22" s="2" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="AG22" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AH22" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI22" s="2" t="n">
+        <v>8.225</v>
+      </c>
+      <c r="AJ22" s="2" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="AK22" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AL22" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM22" s="2" t="n">
+        <v>8.225</v>
+      </c>
+      <c r="AN22" s="2" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="AO22" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AP22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ22" s="2" t="n">
+        <v>8.225</v>
+      </c>
+      <c r="AR22" s="2" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="AS22" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AT22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU22" s="2" t="n">
+        <v>8.225</v>
+      </c>
+      <c r="AV22" s="2" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="AW22" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AX22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY22" s="2" t="n">
+        <v>8.225</v>
+      </c>
+      <c r="AZ22" s="2" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="BA22" s="2" t="n">
+        <v>0.00122</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>15:37</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>GFR</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="n">
+        <v>6.73</v>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13 15:36:00-04:00</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="n"/>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="n"/>
+      <c r="I23" s="2" t="n"/>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>eod_squeeze</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="n">
+        <v>367</v>
+      </c>
+      <c r="L23" s="2" t="n">
+        <v>0.0654574056569432</v>
+      </c>
+      <c r="M23" s="2" t="n">
+        <v>0.0078863900148797</v>
+      </c>
+      <c r="N23" s="2" t="n">
+        <v>1.498700262832116</v>
+      </c>
+      <c r="O23" s="2" t="n">
+        <v>0.009098990004164901</v>
+      </c>
+      <c r="P23" s="2" t="n">
+        <v>0.0037009791291449</v>
+      </c>
+      <c r="Q23" s="2" t="n">
+        <v>-0.006617658092901</v>
+      </c>
+      <c r="R23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S23" s="2" t="n">
+        <v>1.910282988353823</v>
+      </c>
+      <c r="T23" s="2" t="n">
+        <v>0.0003085095451269</v>
+      </c>
+      <c r="U23" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA23" s="2" t="n"/>
+      <c r="AB23" s="2" t="n"/>
+      <c r="AC23" s="2" t="n"/>
+      <c r="AD23" s="2" t="n"/>
+      <c r="AE23" s="2" t="n"/>
+      <c r="AF23" s="2" t="n"/>
+      <c r="AG23" s="2" t="n"/>
+      <c r="AH23" s="2" t="n"/>
+      <c r="AI23" s="2" t="n"/>
+      <c r="AJ23" s="2" t="n"/>
+      <c r="AK23" s="2" t="n"/>
+      <c r="AL23" s="2" t="n"/>
+      <c r="AM23" s="2" t="n"/>
+      <c r="AN23" s="2" t="n"/>
+      <c r="AO23" s="2" t="n"/>
+      <c r="AP23" s="2" t="n"/>
+      <c r="AQ23" s="2" t="n"/>
+      <c r="AR23" s="2" t="n"/>
+      <c r="AS23" s="2" t="n"/>
+      <c r="AT23" s="2" t="n"/>
+      <c r="AU23" s="2" t="n"/>
+      <c r="AV23" s="2" t="n"/>
+      <c r="AW23" s="2" t="n"/>
+      <c r="AX23" s="2" t="n"/>
+      <c r="AY23" s="2" t="n"/>
+      <c r="AZ23" s="2" t="n"/>
+      <c r="BA23" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
bot session end 2026-10-14 16:02
</commit_message>
<xml_diff>
--- a/reports/Paper Bot Live.xlsx
+++ b/reports/Paper Bot Live.xlsx
@@ -864,7 +864,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q6"/>
+  <dimension ref="A1:Q11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1256,6 +1256,311 @@
       <c r="Q6" s="2" t="inlineStr">
         <is>
           <t>Bull flag: 3.7% pole, 0.9% flag on light vol, broke 8.07 | news: [Google News] Is Alignment Healthcare (ALHC) Cheap Following</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>eod_squeeze</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>GFR</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>6.78</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>6.73</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>6.83</v>
+      </c>
+      <c r="I7" s="2" t="n">
+        <v>6.88</v>
+      </c>
+      <c r="J7" s="2" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>next open</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="M7" s="2" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="N7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O7" s="2" t="n"/>
+      <c r="P7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EOD squeeze: +6.5%, within 1% of HOD 6.80, hold to next open | news: [Newswire] SCIENTURE Reports Approximately $1.22 Million in </t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>350</v>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>eod_squeeze</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>GFR</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>51</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>6.78</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>6.73</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>6.83</v>
+      </c>
+      <c r="I8" s="2" t="n">
+        <v>6.88</v>
+      </c>
+      <c r="J8" s="2" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>next open</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="M8" s="2" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="N8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O8" s="2" t="n"/>
+      <c r="P8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EOD squeeze: +6.5%, within 1% of HOD 6.80, hold to next open | news: [Newswire] SCIENTURE Reports Approximately $1.22 Million in </t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>250</v>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>ema_bounce</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>IBRX</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>10.34</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>10.23</v>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>10.45</v>
+      </c>
+      <c r="I9" s="2" t="n">
+        <v>10.56</v>
+      </c>
+      <c r="J9" s="2" t="n">
+        <v>10.32</v>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>breakeven</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="M9" s="2" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="N9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O9" s="2" t="n"/>
+      <c r="P9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q9" s="2" t="inlineStr">
+        <is>
+          <t>9/21 EMA bounce: tagged 21 EMA 10.29, closed back over 9 EMA | news: [Benzinga] FDA Approves ImmunityBio's Anktiva To Treat Adult</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>550</v>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>bull_flag</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>IBRX</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>10.42</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>10.23</v>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>10.61</v>
+      </c>
+      <c r="I10" s="2" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="J10" s="2" t="n">
+        <v>10.21</v>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="n">
+        <v>-5.88</v>
+      </c>
+      <c r="M10" s="2" t="n">
+        <v>-1.07</v>
+      </c>
+      <c r="N10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O10" s="2" t="n"/>
+      <c r="P10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q10" s="2" t="inlineStr">
+        <is>
+          <t>Bull flag: 3.0% pole, 1.2% flag on light vol, broke 10.36 | news: [Benzinga] FDA Approves ImmunityBio's Anktiva To Treat Adult</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>vwap_pullback</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>MXCT</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>79</v>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="H11" s="2" t="n">
+        <v>1.34</v>
+      </c>
+      <c r="I11" s="2" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="J11" s="2" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="n">
+        <v>-5.53</v>
+      </c>
+      <c r="M11" s="2" t="n">
+        <v>-1.38</v>
+      </c>
+      <c r="N11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O11" s="2" t="n"/>
+      <c r="P11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q11" s="2" t="inlineStr">
+        <is>
+          <t>VWAP pullback: +31.7%, dipped to VWAP 1.26, reclaimed with green bar | news: [Benzinga] MaxCyte Reports Preliminary Q3 Core Revenue Of ~$</t>
         </is>
       </c>
     </row>
@@ -1270,7 +1575,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BA23"/>
+  <dimension ref="A1:BA34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5059,8 +5364,14 @@
           <t>off</t>
         </is>
       </c>
-      <c r="H23" s="2" t="n"/>
-      <c r="I23" s="2" t="n"/>
+      <c r="H23" s="2" t="n">
+        <v>0.444</v>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>next open</t>
+        </is>
+      </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
           <t>eod_squeeze</t>
@@ -5114,33 +5425,1846 @@
       <c r="Z23" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA23" s="2" t="n"/>
-      <c r="AB23" s="2" t="n"/>
-      <c r="AC23" s="2" t="n"/>
-      <c r="AD23" s="2" t="n"/>
-      <c r="AE23" s="2" t="n"/>
-      <c r="AF23" s="2" t="n"/>
-      <c r="AG23" s="2" t="n"/>
-      <c r="AH23" s="2" t="n"/>
-      <c r="AI23" s="2" t="n"/>
-      <c r="AJ23" s="2" t="n"/>
-      <c r="AK23" s="2" t="n"/>
-      <c r="AL23" s="2" t="n"/>
-      <c r="AM23" s="2" t="n"/>
-      <c r="AN23" s="2" t="n"/>
-      <c r="AO23" s="2" t="n"/>
-      <c r="AP23" s="2" t="n"/>
-      <c r="AQ23" s="2" t="n"/>
-      <c r="AR23" s="2" t="n"/>
-      <c r="AS23" s="2" t="n"/>
-      <c r="AT23" s="2" t="n"/>
-      <c r="AU23" s="2" t="n"/>
-      <c r="AV23" s="2" t="n"/>
-      <c r="AW23" s="2" t="n"/>
-      <c r="AX23" s="2" t="n"/>
-      <c r="AY23" s="2" t="n"/>
-      <c r="AZ23" s="2" t="n"/>
-      <c r="BA23" s="2" t="n"/>
+      <c r="AA23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC23" s="2" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="AD23" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AE23" s="2" t="n">
+        <v>6.755</v>
+      </c>
+      <c r="AF23" s="2" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="AG23" s="2" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="AH23" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI23" s="2" t="n">
+        <v>6.755</v>
+      </c>
+      <c r="AJ23" s="2" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="AK23" s="2" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AL23" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AM23" s="2" t="n">
+        <v>6.755</v>
+      </c>
+      <c r="AN23" s="2" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="AO23" s="2" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="AP23" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AQ23" s="2" t="n">
+        <v>6.755</v>
+      </c>
+      <c r="AR23" s="2" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="AS23" s="2" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="AT23" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU23" s="2" t="n">
+        <v>6.755</v>
+      </c>
+      <c r="AV23" s="2" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="AW23" s="2" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AX23" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AY23" s="2" t="n">
+        <v>6.755</v>
+      </c>
+      <c r="AZ23" s="2" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="BA23" s="2" t="n">
+        <v>0.00148</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>13:33</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>MXCT</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 13:32:00-04:00</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="n"/>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="n">
+        <v>-1.364</v>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>vwap_pullback</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="n">
+        <v>243</v>
+      </c>
+      <c r="L24" s="2" t="n">
+        <v>0.3174273843527664</v>
+      </c>
+      <c r="M24" s="2" t="n">
+        <v>0.2707469302989209</v>
+      </c>
+      <c r="N24" s="2" t="n">
+        <v>3.998392262277589</v>
+      </c>
+      <c r="O24" s="2" t="n">
+        <v>0.0049784209318419</v>
+      </c>
+      <c r="P24" s="2" t="n">
+        <v>0.0236220325803686</v>
+      </c>
+      <c r="Q24" s="2" t="n">
+        <v>-0.0451128271073669</v>
+      </c>
+      <c r="R24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S24" s="2" t="n">
+        <v>0.2390168854520066</v>
+      </c>
+      <c r="T24" s="2" t="n">
+        <v>-0.0122235056699204</v>
+      </c>
+      <c r="U24" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V24" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="W24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB24" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC24" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AD24" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE24" s="2" t="n">
+        <v>1.275</v>
+      </c>
+      <c r="AF24" s="2" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="AG24" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AH24" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI24" s="2" t="n">
+        <v>1.275</v>
+      </c>
+      <c r="AJ24" s="2" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="AK24" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AL24" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM24" s="2" t="n">
+        <v>1.275</v>
+      </c>
+      <c r="AN24" s="2" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="AO24" s="2" t="n"/>
+      <c r="AP24" s="2" t="n"/>
+      <c r="AQ24" s="2" t="n"/>
+      <c r="AR24" s="2" t="n"/>
+      <c r="AS24" s="2" t="n"/>
+      <c r="AT24" s="2" t="n"/>
+      <c r="AU24" s="2" t="n"/>
+      <c r="AV24" s="2" t="n"/>
+      <c r="AW24" s="2" t="n"/>
+      <c r="AX24" s="2" t="n"/>
+      <c r="AY24" s="2" t="n"/>
+      <c r="AZ24" s="2" t="n"/>
+      <c r="BA24" s="2" t="n">
+        <v>0.00784</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>13:39</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>GFS</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="n">
+        <v>48.7</v>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 13:38:00-04:00</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="n"/>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="n">
+        <v>-1.368</v>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>vwap_pullback</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="n">
+        <v>249</v>
+      </c>
+      <c r="L25" s="2" t="n">
+        <v>0.0456103004993004</v>
+      </c>
+      <c r="M25" s="2" t="n">
+        <v>0.0246252182525501</v>
+      </c>
+      <c r="N25" s="2" t="n">
+        <v>1.359333642620841</v>
+      </c>
+      <c r="O25" s="2" t="n">
+        <v>0.0006247880014953</v>
+      </c>
+      <c r="P25" s="2" t="n">
+        <v>0.0026623351664919</v>
+      </c>
+      <c r="Q25" s="2" t="n">
+        <v>-0.0194778598567527</v>
+      </c>
+      <c r="R25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S25" s="2" t="n">
+        <v>3.888344915572128</v>
+      </c>
+      <c r="T25" s="2" t="n">
+        <v>-0.0124484228185076</v>
+      </c>
+      <c r="U25" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC25" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AD25" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE25" s="2" t="n">
+        <v>48.82</v>
+      </c>
+      <c r="AF25" s="2" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="AG25" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AH25" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI25" s="2" t="n">
+        <v>48.82</v>
+      </c>
+      <c r="AJ25" s="2" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="AK25" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AL25" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM25" s="2" t="n">
+        <v>48.82</v>
+      </c>
+      <c r="AN25" s="2" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="AO25" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AP25" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ25" s="2" t="n">
+        <v>48.82</v>
+      </c>
+      <c r="AR25" s="2" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="AS25" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AT25" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU25" s="2" t="n">
+        <v>48.82</v>
+      </c>
+      <c r="AV25" s="2" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="AW25" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AX25" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY25" s="2" t="n">
+        <v>48.82</v>
+      </c>
+      <c r="AZ25" s="2" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="BA25" s="2" t="n">
+        <v>0.00061</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>13:39</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>IBRX</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="n">
+        <v>10.23</v>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 13:38:00-04:00</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="n"/>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="n">
+        <v>-1.174</v>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>ema_bounce</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="n">
+        <v>249</v>
+      </c>
+      <c r="L26" s="2" t="n">
+        <v>0.0535713886033002</v>
+      </c>
+      <c r="M26" s="2" t="n">
+        <v>-0.0112245518582294</v>
+      </c>
+      <c r="N26" s="2" t="n">
+        <v>1.062099175402153</v>
+      </c>
+      <c r="O26" s="2" t="n">
+        <v>0.0488767111425205</v>
+      </c>
+      <c r="P26" s="2" t="n">
+        <v>0.0092009502198623</v>
+      </c>
+      <c r="Q26" s="2" t="n">
+        <v>-0.0110059085437701</v>
+      </c>
+      <c r="R26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S26" s="2" t="n">
+        <v>2.334568120373986</v>
+      </c>
+      <c r="T26" s="2" t="n">
+        <v>-0.0124484228185076</v>
+      </c>
+      <c r="U26" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W26" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="X26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC26" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AD26" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AE26" s="2" t="n">
+        <v>10.325</v>
+      </c>
+      <c r="AF26" s="2" t="n">
+        <v>0.095</v>
+      </c>
+      <c r="AG26" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AH26" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI26" s="2" t="n">
+        <v>10.325</v>
+      </c>
+      <c r="AJ26" s="2" t="n">
+        <v>0.095</v>
+      </c>
+      <c r="AK26" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AL26" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AM26" s="2" t="n">
+        <v>10.325</v>
+      </c>
+      <c r="AN26" s="2" t="n">
+        <v>0.095</v>
+      </c>
+      <c r="AO26" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AP26" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AQ26" s="2" t="n">
+        <v>10.325</v>
+      </c>
+      <c r="AR26" s="2" t="n">
+        <v>0.095</v>
+      </c>
+      <c r="AS26" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AT26" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU26" s="2" t="n">
+        <v>10.325</v>
+      </c>
+      <c r="AV26" s="2" t="n">
+        <v>0.095</v>
+      </c>
+      <c r="AW26" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AX26" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AY26" s="2" t="n">
+        <v>10.325</v>
+      </c>
+      <c r="AZ26" s="2" t="n">
+        <v>0.095</v>
+      </c>
+      <c r="BA26" s="2" t="n">
+        <v>0.0009700000000000001</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>13:42</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>MXCT</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 13:41:00-04:00</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="n"/>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="n">
+        <v>-1.444</v>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>ema_bounce</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="n">
+        <v>252</v>
+      </c>
+      <c r="L27" s="2" t="n">
+        <v>0.3268671773539939</v>
+      </c>
+      <c r="M27" s="2" t="n">
+        <v>0.2707469302989209</v>
+      </c>
+      <c r="N27" s="2" t="n">
+        <v>3.967763547844457</v>
+      </c>
+      <c r="O27" s="2" t="n">
+        <v>0.0121365157692752</v>
+      </c>
+      <c r="P27" s="2" t="n">
+        <v>0.0227503264718634</v>
+      </c>
+      <c r="Q27" s="2" t="n">
+        <v>-0.0382707518941952</v>
+      </c>
+      <c r="R27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S27" s="2" t="n">
+        <v>0.2461566596953398</v>
+      </c>
+      <c r="T27" s="2" t="n">
+        <v>-0.0128533050661038</v>
+      </c>
+      <c r="U27" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V27" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="W27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC27" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AD27" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE27" s="2" t="n">
+        <v>1.275</v>
+      </c>
+      <c r="AF27" s="2" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="AG27" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AH27" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI27" s="2" t="n">
+        <v>1.275</v>
+      </c>
+      <c r="AJ27" s="2" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="AK27" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AL27" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM27" s="2" t="n">
+        <v>1.275</v>
+      </c>
+      <c r="AN27" s="2" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="AO27" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AP27" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ27" s="2" t="n">
+        <v>1.275</v>
+      </c>
+      <c r="AR27" s="2" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="AS27" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AT27" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU27" s="2" t="n">
+        <v>1.275</v>
+      </c>
+      <c r="AV27" s="2" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="AW27" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AX27" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY27" s="2" t="n">
+        <v>1.275</v>
+      </c>
+      <c r="AZ27" s="2" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="BA27" s="2" t="n">
+        <v>0.00784</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>13:45</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>IBRX</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="n">
+        <v>10.23</v>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 13:44:00-04:00</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="n"/>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="n">
+        <v>-1.118</v>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>bull_flag</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="n">
+        <v>255</v>
+      </c>
+      <c r="L28" s="2" t="n">
+        <v>0.0602040960311092</v>
+      </c>
+      <c r="M28" s="2" t="n">
+        <v>-0.0112245518582294</v>
+      </c>
+      <c r="N28" s="2" t="n">
+        <v>1.060583449946848</v>
+      </c>
+      <c r="O28" s="2" t="n">
+        <v>0.0543389980682877</v>
+      </c>
+      <c r="P28" s="2" t="n">
+        <v>0.0153994550563782</v>
+      </c>
+      <c r="Q28" s="2" t="n">
+        <v>-0.0047797443489004</v>
+      </c>
+      <c r="R28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S28" s="2" t="n">
+        <v>2.340843838154711</v>
+      </c>
+      <c r="T28" s="2" t="n">
+        <v>-0.0125191065823293</v>
+      </c>
+      <c r="U28" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W28" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="X28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC28" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AD28" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE28" s="2" t="n">
+        <v>10.38</v>
+      </c>
+      <c r="AF28" s="2" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="AG28" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AH28" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI28" s="2" t="n">
+        <v>10.38</v>
+      </c>
+      <c r="AJ28" s="2" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="AK28" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AL28" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM28" s="2" t="n">
+        <v>10.38</v>
+      </c>
+      <c r="AN28" s="2" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="AO28" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AP28" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ28" s="2" t="n">
+        <v>10.38</v>
+      </c>
+      <c r="AR28" s="2" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="AS28" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AT28" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU28" s="2" t="n">
+        <v>10.38</v>
+      </c>
+      <c r="AV28" s="2" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="AW28" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AX28" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY28" s="2" t="n">
+        <v>10.38</v>
+      </c>
+      <c r="AZ28" s="2" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="BA28" s="2" t="n">
+        <v>0.00096</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>14:13</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>CANG</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 14:12:00-04:00</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="n"/>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="n">
+        <v>-1.29</v>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>ema_bounce</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="n">
+        <v>283</v>
+      </c>
+      <c r="L29" s="2" t="n">
+        <v>0.0857142720903669</v>
+      </c>
+      <c r="M29" s="2" t="n">
+        <v>0.0171428407941545</v>
+      </c>
+      <c r="N29" s="2" t="n">
+        <v>2.806767859017679</v>
+      </c>
+      <c r="O29" s="2" t="n">
+        <v>0.025434212595651</v>
+      </c>
+      <c r="P29" s="2" t="n">
+        <v>0.0131578823536055</v>
+      </c>
+      <c r="Q29" s="2" t="n">
+        <v>-0.0142672027198642</v>
+      </c>
+      <c r="R29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S29" s="2" t="n">
+        <v>1.335001054183994</v>
+      </c>
+      <c r="T29" s="2" t="n">
+        <v>-0.0132324555994564</v>
+      </c>
+      <c r="U29" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC29" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AD29" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AE29" s="2" t="n">
+        <v>3.799</v>
+      </c>
+      <c r="AF29" s="2" t="n">
+        <v>0.049</v>
+      </c>
+      <c r="AG29" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AH29" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI29" s="2" t="n">
+        <v>3.799</v>
+      </c>
+      <c r="AJ29" s="2" t="n">
+        <v>0.049</v>
+      </c>
+      <c r="AK29" s="2" t="n">
+        <v>0.6122</v>
+      </c>
+      <c r="AL29" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AM29" s="2" t="n">
+        <v>3.799</v>
+      </c>
+      <c r="AN29" s="2" t="n">
+        <v>0.049</v>
+      </c>
+      <c r="AO29" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AP29" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AQ29" s="2" t="n">
+        <v>3.799</v>
+      </c>
+      <c r="AR29" s="2" t="n">
+        <v>0.049</v>
+      </c>
+      <c r="AS29" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AT29" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU29" s="2" t="n">
+        <v>3.799</v>
+      </c>
+      <c r="AV29" s="2" t="n">
+        <v>0.049</v>
+      </c>
+      <c r="AW29" s="2" t="n">
+        <v>0.6122</v>
+      </c>
+      <c r="AX29" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AY29" s="2" t="n">
+        <v>3.799</v>
+      </c>
+      <c r="AZ29" s="2" t="n">
+        <v>0.049</v>
+      </c>
+      <c r="BA29" s="2" t="n">
+        <v>0.00528</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>14:21</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>GFS</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="n">
+        <v>48.43</v>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 14:20:00-04:00</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="n"/>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="n">
+        <v>-1.146</v>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>ema_bounce</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="n">
+        <v>291</v>
+      </c>
+      <c r="L30" s="2" t="n">
+        <v>0.0458243973166423</v>
+      </c>
+      <c r="M30" s="2" t="n">
+        <v>0.0246252182525501</v>
+      </c>
+      <c r="N30" s="2" t="n">
+        <v>1.319878607715998</v>
+      </c>
+      <c r="O30" s="2" t="n">
+        <v>0.0014688340818449</v>
+      </c>
+      <c r="P30" s="2" t="n">
+        <v>0.0083947614927713</v>
+      </c>
+      <c r="Q30" s="2" t="n">
+        <v>-0.019277090344978</v>
+      </c>
+      <c r="R30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S30" s="2" t="n">
+        <v>3.888549652366744</v>
+      </c>
+      <c r="T30" s="2" t="n">
+        <v>-0.0125191065823293</v>
+      </c>
+      <c r="U30" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC30" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AD30" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE30" s="2" t="n">
+        <v>48.84</v>
+      </c>
+      <c r="AF30" s="2" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="AG30" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AH30" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI30" s="2" t="n">
+        <v>48.84</v>
+      </c>
+      <c r="AJ30" s="2" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="AK30" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AL30" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM30" s="2" t="n">
+        <v>48.84</v>
+      </c>
+      <c r="AN30" s="2" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="AO30" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AP30" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ30" s="2" t="n">
+        <v>48.84</v>
+      </c>
+      <c r="AR30" s="2" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="AS30" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AT30" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU30" s="2" t="n">
+        <v>48.84</v>
+      </c>
+      <c r="AV30" s="2" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="AW30" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AX30" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY30" s="2" t="n">
+        <v>48.84</v>
+      </c>
+      <c r="AZ30" s="2" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="BA30" s="2" t="n">
+        <v>0.00041</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>14:29</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>BSP</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="n">
+        <v>53.11</v>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 14:28:00-04:00</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="n"/>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="n">
+        <v>0.382</v>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>breakeven</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>vwap_pullback</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="n">
+        <v>299</v>
+      </c>
+      <c r="L31" s="2" t="n">
+        <v>0.4125726011640367</v>
+      </c>
+      <c r="M31" s="2" t="n">
+        <v>0.3280506595012964</v>
+      </c>
+      <c r="N31" s="2" t="n">
+        <v>1.988852292756681</v>
+      </c>
+      <c r="O31" s="2" t="n">
+        <v>0.0043796192014877</v>
+      </c>
+      <c r="P31" s="2" t="n">
+        <v>0.0069184656956497</v>
+      </c>
+      <c r="Q31" s="2" t="n">
+        <v>-0.0867486631134482</v>
+      </c>
+      <c r="R31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S31" s="2" t="n">
+        <v>3.979307743674213</v>
+      </c>
+      <c r="T31" s="2" t="n">
+        <v>-0.0127376692527039</v>
+      </c>
+      <c r="U31" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC31" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AD31" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE31" s="2" t="n">
+        <v>53.37</v>
+      </c>
+      <c r="AF31" s="2" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="AG31" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AH31" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI31" s="2" t="n">
+        <v>53.37</v>
+      </c>
+      <c r="AJ31" s="2" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="AK31" s="2" t="n">
+        <v>0.8817</v>
+      </c>
+      <c r="AL31" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AM31" s="2" t="n">
+        <v>53.37</v>
+      </c>
+      <c r="AN31" s="2" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="AO31" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AP31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ31" s="2" t="n">
+        <v>53.37</v>
+      </c>
+      <c r="AR31" s="2" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="AS31" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AT31" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU31" s="2" t="n">
+        <v>53.37</v>
+      </c>
+      <c r="AV31" s="2" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="AW31" s="2" t="n">
+        <v>0.8817</v>
+      </c>
+      <c r="AX31" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AY31" s="2" t="n">
+        <v>53.37</v>
+      </c>
+      <c r="AZ31" s="2" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="BA31" s="2" t="n">
+        <v>0.00299</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>14:57</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>BSP</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="n">
+        <v>52.74</v>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 14:56:00-04:00</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="n"/>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="n">
+        <v>-1.136</v>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>ema_bounce</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="n">
+        <v>327</v>
+      </c>
+      <c r="L32" s="2" t="n">
+        <v>0.4094030573196039</v>
+      </c>
+      <c r="M32" s="2" t="n">
+        <v>0.3280506595012964</v>
+      </c>
+      <c r="N32" s="2" t="n">
+        <v>1.946982379034813</v>
+      </c>
+      <c r="O32" s="2" t="n">
+        <v>0.0023349322002463</v>
+      </c>
+      <c r="P32" s="2" t="n">
+        <v>0.0116192017102654</v>
+      </c>
+      <c r="Q32" s="2" t="n">
+        <v>-0.0887978251535894</v>
+      </c>
+      <c r="R32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S32" s="2" t="n">
+        <v>3.977061413045741</v>
+      </c>
+      <c r="T32" s="2" t="n">
+        <v>-0.0128597379946647</v>
+      </c>
+      <c r="U32" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC32" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AD32" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE32" s="2" t="n">
+        <v>53.25</v>
+      </c>
+      <c r="AF32" s="2" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="AG32" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AH32" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI32" s="2" t="n">
+        <v>53.25</v>
+      </c>
+      <c r="AJ32" s="2" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="AK32" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AL32" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM32" s="2" t="n">
+        <v>53.25</v>
+      </c>
+      <c r="AN32" s="2" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="AO32" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AP32" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ32" s="2" t="n">
+        <v>53.25</v>
+      </c>
+      <c r="AR32" s="2" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="AS32" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AT32" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU32" s="2" t="n">
+        <v>53.25</v>
+      </c>
+      <c r="AV32" s="2" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="AW32" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AX32" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY32" s="2" t="n">
+        <v>53.25</v>
+      </c>
+      <c r="AZ32" s="2" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="BA32" s="2" t="n">
+        <v>0.00281</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>15:42</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>CANG</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 15:41:00-04:00</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="n"/>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="n"/>
+      <c r="I33" s="2" t="n"/>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>eod_squeeze</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="n">
+        <v>372</v>
+      </c>
+      <c r="L33" s="2" t="n">
+        <v>0.0954571451459611</v>
+      </c>
+      <c r="M33" s="2" t="n">
+        <v>0.0171428407941545</v>
+      </c>
+      <c r="N33" s="2" t="n">
+        <v>3.058768267329295</v>
+      </c>
+      <c r="O33" s="2" t="n">
+        <v>0.0249810786014439</v>
+      </c>
+      <c r="P33" s="2" t="n">
+        <v>0.0219347455296283</v>
+      </c>
+      <c r="Q33" s="2" t="n">
+        <v>-0.006709815489339</v>
+      </c>
+      <c r="R33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S33" s="2" t="n">
+        <v>1.343934728793134</v>
+      </c>
+      <c r="T33" s="2" t="n">
+        <v>-0.0117864587795196</v>
+      </c>
+      <c r="U33" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA33" s="2" t="n"/>
+      <c r="AB33" s="2" t="n"/>
+      <c r="AC33" s="2" t="n"/>
+      <c r="AD33" s="2" t="n"/>
+      <c r="AE33" s="2" t="n"/>
+      <c r="AF33" s="2" t="n"/>
+      <c r="AG33" s="2" t="n"/>
+      <c r="AH33" s="2" t="n"/>
+      <c r="AI33" s="2" t="n"/>
+      <c r="AJ33" s="2" t="n"/>
+      <c r="AK33" s="2" t="n"/>
+      <c r="AL33" s="2" t="n"/>
+      <c r="AM33" s="2" t="n"/>
+      <c r="AN33" s="2" t="n"/>
+      <c r="AO33" s="2" t="n"/>
+      <c r="AP33" s="2" t="n"/>
+      <c r="AQ33" s="2" t="n"/>
+      <c r="AR33" s="2" t="n"/>
+      <c r="AS33" s="2" t="n"/>
+      <c r="AT33" s="2" t="n"/>
+      <c r="AU33" s="2" t="n"/>
+      <c r="AV33" s="2" t="n"/>
+      <c r="AW33" s="2" t="n"/>
+      <c r="AX33" s="2" t="n"/>
+      <c r="AY33" s="2" t="n"/>
+      <c r="AZ33" s="2" t="n"/>
+      <c r="BA33" s="2" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>15:45</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>GFS</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 15:44:00-04:00</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="n"/>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="n"/>
+      <c r="I34" s="2" t="n"/>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>eod_squeeze</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="n">
+        <v>375</v>
+      </c>
+      <c r="L34" s="2" t="n">
+        <v>0.0558864576207154</v>
+      </c>
+      <c r="M34" s="2" t="n">
+        <v>0.0246252182525501</v>
+      </c>
+      <c r="N34" s="2" t="n">
+        <v>1.275905382580093</v>
+      </c>
+      <c r="O34" s="2" t="n">
+        <v>0.0110446447468701</v>
+      </c>
+      <c r="P34" s="2" t="n">
+        <v>0.0164246612370103</v>
+      </c>
+      <c r="Q34" s="2" t="n">
+        <v>-0.009841382893656299</v>
+      </c>
+      <c r="R34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S34" s="2" t="n">
+        <v>3.898124839322632</v>
+      </c>
+      <c r="T34" s="2" t="n">
+        <v>-0.0116450912518761</v>
+      </c>
+      <c r="U34" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA34" s="2" t="n"/>
+      <c r="AB34" s="2" t="n"/>
+      <c r="AC34" s="2" t="n"/>
+      <c r="AD34" s="2" t="n"/>
+      <c r="AE34" s="2" t="n"/>
+      <c r="AF34" s="2" t="n"/>
+      <c r="AG34" s="2" t="n"/>
+      <c r="AH34" s="2" t="n"/>
+      <c r="AI34" s="2" t="n"/>
+      <c r="AJ34" s="2" t="n"/>
+      <c r="AK34" s="2" t="n"/>
+      <c r="AL34" s="2" t="n"/>
+      <c r="AM34" s="2" t="n"/>
+      <c r="AN34" s="2" t="n"/>
+      <c r="AO34" s="2" t="n"/>
+      <c r="AP34" s="2" t="n"/>
+      <c r="AQ34" s="2" t="n"/>
+      <c r="AR34" s="2" t="n"/>
+      <c r="AS34" s="2" t="n"/>
+      <c r="AT34" s="2" t="n"/>
+      <c r="AU34" s="2" t="n"/>
+      <c r="AV34" s="2" t="n"/>
+      <c r="AW34" s="2" t="n"/>
+      <c r="AX34" s="2" t="n"/>
+      <c r="AY34" s="2" t="n"/>
+      <c r="AZ34" s="2" t="n"/>
+      <c r="BA34" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5153,7 +7277,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5403,6 +7527,204 @@
         <v>-3.24</v>
       </c>
       <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>eod_squeeze</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>GFR</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>6.76</v>
+      </c>
+      <c r="I7" s="2" t="n">
+        <v>-3.77</v>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>350</v>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>eod_squeeze</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>GFR</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>51</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>51</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>6.76</v>
+      </c>
+      <c r="I8" s="2" t="n">
+        <v>-6.63</v>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>250</v>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>ema_bounce</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>IBRX</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>10.33</v>
+      </c>
+      <c r="I9" s="2" t="n"/>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>partially open</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>550</v>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>bull_flag</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>IBRX</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>-5.88</v>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>10.38</v>
+      </c>
+      <c r="I10" s="2" t="n">
+        <v>-4.44</v>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>vwap_pullback</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>MXCT</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>-5.53</v>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>66</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>66</v>
+      </c>
+      <c r="H11" s="2" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="I11" s="2" t="n">
+        <v>-3.3</v>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>closed</t>
         </is>

</xml_diff>

<commit_message>
bot session end 2026-10-15 16:02
</commit_message>
<xml_diff>
--- a/reports/Paper Bot Live.xlsx
+++ b/reports/Paper Bot Live.xlsx
@@ -864,7 +864,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q11"/>
+  <dimension ref="A1:Q16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1561,6 +1561,311 @@
       <c r="Q11" s="2" t="inlineStr">
         <is>
           <t>VWAP pullback: +31.7%, dipped to VWAP 1.26, reclaimed with green bar | news: [Benzinga] MaxCyte Reports Preliminary Q3 Core Revenue Of ~$</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>250</v>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>ema_bounce</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>RGC</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>10.77</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>10.61</v>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>10.93</v>
+      </c>
+      <c r="I12" s="2" t="n">
+        <v>11.09</v>
+      </c>
+      <c r="J12" s="2" t="n">
+        <v>10.59</v>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="n">
+        <v>-2.7</v>
+      </c>
+      <c r="M12" s="2" t="n">
+        <v>-1.08</v>
+      </c>
+      <c r="N12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O12" s="2" t="n"/>
+      <c r="P12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q12" s="2" t="inlineStr">
+        <is>
+          <t>9/21 EMA bounce: tagged 21 EMA 10.68, closed back over 9 EMA | news: [Newswire] Fengate Private Equity Acquires Majority Stake in</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>ema_bounce</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>RGC</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>10.77</v>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>10.61</v>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>10.93</v>
+      </c>
+      <c r="I13" s="2" t="n">
+        <v>11.09</v>
+      </c>
+      <c r="J13" s="2" t="n">
+        <v>10.59</v>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="n">
+        <v>-4.32</v>
+      </c>
+      <c r="M13" s="2" t="n">
+        <v>-1.08</v>
+      </c>
+      <c r="N13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O13" s="2" t="n"/>
+      <c r="P13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q13" s="2" t="inlineStr">
+        <is>
+          <t>9/21 EMA bounce: tagged 21 EMA 10.68, closed back over 9 EMA | news: [Newswire] Fengate Private Equity Acquires Majority Stake in</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>350</v>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>bull_flag</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>RGC</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>10.6</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>10.39</v>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>10.81</v>
+      </c>
+      <c r="I14" s="2" t="n">
+        <v>11.02</v>
+      </c>
+      <c r="J14" s="2" t="n">
+        <v>10.33</v>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="n">
+        <v>-4.32</v>
+      </c>
+      <c r="M14" s="2" t="n">
+        <v>-1.23</v>
+      </c>
+      <c r="N14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O14" s="2" t="n"/>
+      <c r="P14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q14" s="2" t="inlineStr">
+        <is>
+          <t>Bull flag: 4.5% pole, 1.3% flag on light vol, broke 10.53 | news: [Newswire] Fengate Private Equity Acquires Majority Stake in</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>550</v>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>bull_flag</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>RGC</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="F15" s="2" t="n">
+        <v>10.6</v>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>10.39</v>
+      </c>
+      <c r="H15" s="2" t="n">
+        <v>10.81</v>
+      </c>
+      <c r="I15" s="2" t="n">
+        <v>11.02</v>
+      </c>
+      <c r="J15" s="2" t="n">
+        <v>10.33</v>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="n">
+        <v>-7.02</v>
+      </c>
+      <c r="M15" s="2" t="n">
+        <v>-1.28</v>
+      </c>
+      <c r="N15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O15" s="2" t="n"/>
+      <c r="P15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q15" s="2" t="inlineStr">
+        <is>
+          <t>Bull flag: 4.5% pole, 1.3% flag on light vol, broke 10.53 | news: [Newswire] Fengate Private Equity Acquires Majority Stake in</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>vwap_pullback</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>RGC</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="F16" s="2" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>9.960000000000001</v>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>10.44</v>
+      </c>
+      <c r="I16" s="2" t="n">
+        <v>10.68</v>
+      </c>
+      <c r="J16" s="2" t="n">
+        <v>10.68</v>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>target</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="M16" s="2" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="N16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O16" s="2" t="n"/>
+      <c r="P16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q16" s="2" t="inlineStr">
+        <is>
+          <t>VWAP pullback: +24.3%, dipped to VWAP 10.06, reclaimed with green bar | news: [Newswire] Fengate Private Equity Acquires Majority Stake in</t>
         </is>
       </c>
     </row>
@@ -1575,7 +1880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BA34"/>
+  <dimension ref="A1:BA45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7070,8 +7375,14 @@
           <t>off</t>
         </is>
       </c>
-      <c r="H33" s="2" t="n"/>
-      <c r="I33" s="2" t="n"/>
+      <c r="H33" s="2" t="n">
+        <v>-1.333</v>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
           <t>eod_squeeze</t>
@@ -7125,33 +7436,87 @@
       <c r="Z33" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA33" s="2" t="n"/>
-      <c r="AB33" s="2" t="n"/>
-      <c r="AC33" s="2" t="n"/>
-      <c r="AD33" s="2" t="n"/>
-      <c r="AE33" s="2" t="n"/>
-      <c r="AF33" s="2" t="n"/>
-      <c r="AG33" s="2" t="n"/>
-      <c r="AH33" s="2" t="n"/>
-      <c r="AI33" s="2" t="n"/>
-      <c r="AJ33" s="2" t="n"/>
-      <c r="AK33" s="2" t="n"/>
-      <c r="AL33" s="2" t="n"/>
-      <c r="AM33" s="2" t="n"/>
-      <c r="AN33" s="2" t="n"/>
-      <c r="AO33" s="2" t="n"/>
-      <c r="AP33" s="2" t="n"/>
-      <c r="AQ33" s="2" t="n"/>
-      <c r="AR33" s="2" t="n"/>
-      <c r="AS33" s="2" t="n"/>
-      <c r="AT33" s="2" t="n"/>
-      <c r="AU33" s="2" t="n"/>
-      <c r="AV33" s="2" t="n"/>
-      <c r="AW33" s="2" t="n"/>
-      <c r="AX33" s="2" t="n"/>
-      <c r="AY33" s="2" t="n"/>
-      <c r="AZ33" s="2" t="n"/>
-      <c r="BA33" s="2" t="n"/>
+      <c r="AA33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC33" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AD33" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE33" s="2" t="n">
+        <v>3.79</v>
+      </c>
+      <c r="AF33" s="2" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="AG33" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AH33" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI33" s="2" t="n">
+        <v>3.79</v>
+      </c>
+      <c r="AJ33" s="2" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="AK33" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AL33" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM33" s="2" t="n">
+        <v>3.79</v>
+      </c>
+      <c r="AN33" s="2" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="AO33" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AP33" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ33" s="2" t="n">
+        <v>3.79</v>
+      </c>
+      <c r="AR33" s="2" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="AS33" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AT33" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU33" s="2" t="n">
+        <v>3.79</v>
+      </c>
+      <c r="AV33" s="2" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="AW33" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AX33" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY33" s="2" t="n">
+        <v>3.79</v>
+      </c>
+      <c r="AZ33" s="2" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="BA33" s="2" t="n">
+        <v>0.0105</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -7183,8 +7548,14 @@
           <t>off</t>
         </is>
       </c>
-      <c r="H34" s="2" t="n"/>
-      <c r="I34" s="2" t="n"/>
+      <c r="H34" s="2" t="n">
+        <v>-3.076</v>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>next open</t>
+        </is>
+      </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
           <t>eod_squeeze</t>
@@ -7238,33 +7609,1796 @@
       <c r="Z34" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA34" s="2" t="n"/>
-      <c r="AB34" s="2" t="n"/>
-      <c r="AC34" s="2" t="n"/>
-      <c r="AD34" s="2" t="n"/>
-      <c r="AE34" s="2" t="n"/>
-      <c r="AF34" s="2" t="n"/>
-      <c r="AG34" s="2" t="n"/>
-      <c r="AH34" s="2" t="n"/>
-      <c r="AI34" s="2" t="n"/>
-      <c r="AJ34" s="2" t="n"/>
-      <c r="AK34" s="2" t="n"/>
-      <c r="AL34" s="2" t="n"/>
-      <c r="AM34" s="2" t="n"/>
-      <c r="AN34" s="2" t="n"/>
-      <c r="AO34" s="2" t="n"/>
-      <c r="AP34" s="2" t="n"/>
-      <c r="AQ34" s="2" t="n"/>
-      <c r="AR34" s="2" t="n"/>
-      <c r="AS34" s="2" t="n"/>
-      <c r="AT34" s="2" t="n"/>
-      <c r="AU34" s="2" t="n"/>
-      <c r="AV34" s="2" t="n"/>
-      <c r="AW34" s="2" t="n"/>
-      <c r="AX34" s="2" t="n"/>
-      <c r="AY34" s="2" t="n"/>
-      <c r="AZ34" s="2" t="n"/>
-      <c r="BA34" s="2" t="n"/>
+      <c r="AA34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC34" s="2" t="n">
+        <v>-3.1683</v>
+      </c>
+      <c r="AD34" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE34" s="2" t="n">
+        <v>49.32</v>
+      </c>
+      <c r="AF34" s="2" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="AG34" s="2" t="n">
+        <v>-3.1683</v>
+      </c>
+      <c r="AH34" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI34" s="2" t="n">
+        <v>49.32</v>
+      </c>
+      <c r="AJ34" s="2" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="AK34" s="2" t="n">
+        <v>-3.1683</v>
+      </c>
+      <c r="AL34" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM34" s="2" t="n">
+        <v>49.32</v>
+      </c>
+      <c r="AN34" s="2" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="AO34" s="2" t="n">
+        <v>-3.1953</v>
+      </c>
+      <c r="AP34" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ34" s="2" t="n">
+        <v>49.3099</v>
+      </c>
+      <c r="AR34" s="2" t="n">
+        <v>0.8099</v>
+      </c>
+      <c r="AS34" s="2" t="n">
+        <v>-3.1953</v>
+      </c>
+      <c r="AT34" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU34" s="2" t="n">
+        <v>49.3099</v>
+      </c>
+      <c r="AV34" s="2" t="n">
+        <v>0.8099</v>
+      </c>
+      <c r="AW34" s="2" t="n">
+        <v>-3.1953</v>
+      </c>
+      <c r="AX34" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY34" s="2" t="n">
+        <v>49.3099</v>
+      </c>
+      <c r="AZ34" s="2" t="n">
+        <v>0.8099</v>
+      </c>
+      <c r="BA34" s="2" t="n">
+        <v>0.00061</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>13:18</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>PATK</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="n">
+        <v>66.91</v>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15 13:15:00-04:00</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="n"/>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="n">
+        <v>1.115</v>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>time</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>ema_bounce</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="n">
+        <v>228</v>
+      </c>
+      <c r="L35" s="2" t="n">
+        <v>0.0639709232223955</v>
+      </c>
+      <c r="M35" s="2" t="n">
+        <v>0.0153213929073625</v>
+      </c>
+      <c r="N35" s="2" t="n">
+        <v>1.059106073477457</v>
+      </c>
+      <c r="O35" s="2" t="n">
+        <v>0.004841410123316</v>
+      </c>
+      <c r="P35" s="2" t="n">
+        <v>0.0066805315658267</v>
+      </c>
+      <c r="Q35" s="2" t="n">
+        <v>-0.0083909861955467</v>
+      </c>
+      <c r="R35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S35" s="2" t="n">
+        <v>4.21005137899511</v>
+      </c>
+      <c r="T35" s="2" t="n">
+        <v>0.0012344233850942</v>
+      </c>
+      <c r="U35" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC35" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AD35" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE35" s="2" t="n">
+        <v>67.375</v>
+      </c>
+      <c r="AF35" s="2" t="n">
+        <v>0.465</v>
+      </c>
+      <c r="AG35" s="2" t="n">
+        <v>1.9247</v>
+      </c>
+      <c r="AH35" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI35" s="2" t="n">
+        <v>67.375</v>
+      </c>
+      <c r="AJ35" s="2" t="n">
+        <v>0.465</v>
+      </c>
+      <c r="AK35" s="2" t="n">
+        <v>1.4624</v>
+      </c>
+      <c r="AL35" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AM35" s="2" t="n">
+        <v>67.375</v>
+      </c>
+      <c r="AN35" s="2" t="n">
+        <v>0.465</v>
+      </c>
+      <c r="AO35" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AP35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ35" s="2" t="n">
+        <v>67.36</v>
+      </c>
+      <c r="AR35" s="2" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="AS35" s="2" t="n">
+        <v>2.0222</v>
+      </c>
+      <c r="AT35" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU35" s="2" t="n">
+        <v>67.36</v>
+      </c>
+      <c r="AV35" s="2" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="AW35" s="2" t="n">
+        <v>1.5111</v>
+      </c>
+      <c r="AX35" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AY35" s="2" t="n">
+        <v>67.36</v>
+      </c>
+      <c r="AZ35" s="2" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="BA35" s="2" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>13:21</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>RGC</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="n">
+        <v>10.61</v>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15 13:20:00-04:00</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="n"/>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="n">
+        <v>-1.074</v>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>ema_bounce</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="n">
+        <v>231</v>
+      </c>
+      <c r="L36" s="2" t="n">
+        <v>0.3390875605938934</v>
+      </c>
+      <c r="M36" s="2" t="n">
+        <v>-0.0160295490884178</v>
+      </c>
+      <c r="N36" s="2" t="n">
+        <v>2.323216193178613</v>
+      </c>
+      <c r="O36" s="2" t="n">
+        <v>0.08541890490022939</v>
+      </c>
+      <c r="P36" s="2" t="n">
+        <v>0.0230202269411247</v>
+      </c>
+      <c r="Q36" s="2" t="n">
+        <v>-0.0233725212391703</v>
+      </c>
+      <c r="R36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S36" s="2" t="n">
+        <v>2.385086282892276</v>
+      </c>
+      <c r="T36" s="2" t="n">
+        <v>0.0010524916635776</v>
+      </c>
+      <c r="U36" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z36" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC36" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AD36" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE36" s="2" t="n">
+        <v>10.86</v>
+      </c>
+      <c r="AF36" s="2" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="AG36" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AH36" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI36" s="2" t="n">
+        <v>10.86</v>
+      </c>
+      <c r="AJ36" s="2" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="AK36" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AL36" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM36" s="2" t="n">
+        <v>10.86</v>
+      </c>
+      <c r="AN36" s="2" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="AO36" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AP36" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ36" s="2" t="n">
+        <v>10.86</v>
+      </c>
+      <c r="AR36" s="2" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="AS36" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AT36" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU36" s="2" t="n">
+        <v>10.86</v>
+      </c>
+      <c r="AV36" s="2" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="AW36" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AX36" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY36" s="2" t="n">
+        <v>10.86</v>
+      </c>
+      <c r="AZ36" s="2" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="BA36" s="2" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>13:27</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>LAC</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="n">
+        <v>2.21</v>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15 13:26:00-04:00</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="n"/>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="n">
+        <v>-0.459</v>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>time</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>ema_bounce</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="n">
+        <v>237</v>
+      </c>
+      <c r="L37" s="2" t="n">
+        <v>0.0797101290696873</v>
+      </c>
+      <c r="M37" s="2" t="n">
+        <v>-0.00483091342307</v>
+      </c>
+      <c r="N37" s="2" t="n">
+        <v>1.159949356078415</v>
+      </c>
+      <c r="O37" s="2" t="n">
+        <v>0.0299164875593827</v>
+      </c>
+      <c r="P37" s="2" t="n">
+        <v>0.011185635914651</v>
+      </c>
+      <c r="Q37" s="2" t="n">
+        <v>-0.019736875815185</v>
+      </c>
+      <c r="R37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S37" s="2" t="n">
+        <v>0.80424118112854</v>
+      </c>
+      <c r="T37" s="2" t="n">
+        <v>0.0010135516133313</v>
+      </c>
+      <c r="U37" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X37" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC37" s="2" t="n">
+        <v>0.7176</v>
+      </c>
+      <c r="AD37" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE37" s="2" t="n">
+        <v>2.2362</v>
+      </c>
+      <c r="AF37" s="2" t="n">
+        <v>0.0262</v>
+      </c>
+      <c r="AG37" s="2" t="n">
+        <v>0.7176</v>
+      </c>
+      <c r="AH37" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI37" s="2" t="n">
+        <v>2.2362</v>
+      </c>
+      <c r="AJ37" s="2" t="n">
+        <v>0.0262</v>
+      </c>
+      <c r="AK37" s="2" t="n">
+        <v>0.7176</v>
+      </c>
+      <c r="AL37" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM37" s="2" t="n">
+        <v>2.2362</v>
+      </c>
+      <c r="AN37" s="2" t="n">
+        <v>0.0262</v>
+      </c>
+      <c r="AO37" s="2" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AP37" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AQ37" s="2" t="n">
+        <v>2.235</v>
+      </c>
+      <c r="AR37" s="2" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="AS37" s="2" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AT37" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU37" s="2" t="n">
+        <v>2.235</v>
+      </c>
+      <c r="AV37" s="2" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="AW37" s="2" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AX37" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AY37" s="2" t="n">
+        <v>2.235</v>
+      </c>
+      <c r="AZ37" s="2" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="BA37" s="2" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>13:32</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>RGC</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="n">
+        <v>9.960000000000001</v>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15 13:31:00-04:00</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="n"/>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>target</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>vwap_pullback</t>
+        </is>
+      </c>
+      <c r="K38" s="2" t="n">
+        <v>242</v>
+      </c>
+      <c r="L38" s="2" t="n">
+        <v>0.2428853364747751</v>
+      </c>
+      <c r="M38" s="2" t="n">
+        <v>-0.0160295490884178</v>
+      </c>
+      <c r="N38" s="2" t="n">
+        <v>2.424290474393779</v>
+      </c>
+      <c r="O38" s="2" t="n">
+        <v>0.0022685678470941</v>
+      </c>
+      <c r="P38" s="2" t="n">
+        <v>0.0118851223471147</v>
+      </c>
+      <c r="Q38" s="2" t="n">
+        <v>-0.093535024691125</v>
+      </c>
+      <c r="R38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S38" s="2" t="n">
+        <v>2.310533386661928</v>
+      </c>
+      <c r="T38" s="2" t="n">
+        <v>0.0010135516133313</v>
+      </c>
+      <c r="U38" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z38" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC38" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AD38" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE38" s="2" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="AF38" s="2" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="AG38" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="AH38" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI38" s="2" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="AJ38" s="2" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="AK38" s="2" t="n">
+        <v>0.9286</v>
+      </c>
+      <c r="AL38" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AM38" s="2" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="AN38" s="2" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="AO38" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AP38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ38" s="2" t="n">
+        <v>10.0798</v>
+      </c>
+      <c r="AR38" s="2" t="n">
+        <v>0.1198</v>
+      </c>
+      <c r="AS38" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="AT38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU38" s="2" t="n">
+        <v>10.0798</v>
+      </c>
+      <c r="AV38" s="2" t="n">
+        <v>0.1198</v>
+      </c>
+      <c r="AW38" s="2" t="n">
+        <v>1.0851</v>
+      </c>
+      <c r="AX38" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AY38" s="2" t="n">
+        <v>10.0798</v>
+      </c>
+      <c r="AZ38" s="2" t="n">
+        <v>0.1198</v>
+      </c>
+      <c r="BA38" s="2" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>13:39</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>DNN</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="n">
+        <v>2.29</v>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15 13:38:00-04:00</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="n"/>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="n">
+        <v>0.331</v>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>time</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>ema_bounce</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="n">
+        <v>249</v>
+      </c>
+      <c r="L39" s="2" t="n">
+        <v>0.0717592431623264</v>
+      </c>
+      <c r="M39" s="2" t="n">
+        <v>-0.0138888750915179</v>
+      </c>
+      <c r="N39" s="2" t="n">
+        <v>1.351792630266435</v>
+      </c>
+      <c r="O39" s="2" t="n">
+        <v>0.0062284305762303</v>
+      </c>
+      <c r="P39" s="2" t="n">
+        <v>0.0107991605194496</v>
+      </c>
+      <c r="Q39" s="2" t="n">
+        <v>-0.0190677287608689</v>
+      </c>
+      <c r="R39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S39" s="2" t="n">
+        <v>0.839409712255458</v>
+      </c>
+      <c r="T39" s="2" t="n">
+        <v>0.0019623881940746</v>
+      </c>
+      <c r="U39" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X39" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC39" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AD39" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE39" s="2" t="n">
+        <v>2.315</v>
+      </c>
+      <c r="AF39" s="2" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="AG39" s="2" t="n">
+        <v>2.196</v>
+      </c>
+      <c r="AH39" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI39" s="2" t="n">
+        <v>2.315</v>
+      </c>
+      <c r="AJ39" s="2" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="AK39" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL39" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AM39" s="2" t="n">
+        <v>2.315</v>
+      </c>
+      <c r="AN39" s="2" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="AO39" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AP39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ39" s="2" t="n">
+        <v>2.315</v>
+      </c>
+      <c r="AR39" s="2" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="AS39" s="2" t="n">
+        <v>2.196</v>
+      </c>
+      <c r="AT39" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU39" s="2" t="n">
+        <v>2.315</v>
+      </c>
+      <c r="AV39" s="2" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="AW39" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX39" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AY39" s="2" t="n">
+        <v>2.315</v>
+      </c>
+      <c r="AZ39" s="2" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="BA39" s="2" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>13:42</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>ERIC</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="n">
+        <v>10.43</v>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15 13:41:00-04:00</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="n"/>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="n">
+        <v>1.036</v>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>time</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>ema_bounce</t>
+        </is>
+      </c>
+      <c r="K40" s="2" t="n">
+        <v>252</v>
+      </c>
+      <c r="L40" s="2" t="n">
+        <v>0.0981211421235559</v>
+      </c>
+      <c r="M40" s="2" t="n">
+        <v>0.1115657600256756</v>
+      </c>
+      <c r="N40" s="2" t="n">
+        <v>1.814459349094037</v>
+      </c>
+      <c r="O40" s="2" t="n">
+        <v>0.0090128034427037</v>
+      </c>
+      <c r="P40" s="2" t="n">
+        <v>0.008555176221237901</v>
+      </c>
+      <c r="Q40" s="2" t="n">
+        <v>-0.013133151186904</v>
+      </c>
+      <c r="R40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S40" s="2" t="n">
+        <v>2.35327825082322</v>
+      </c>
+      <c r="T40" s="2" t="n">
+        <v>0.002637613423801</v>
+      </c>
+      <c r="U40" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC40" s="2" t="n">
+        <v>1.3778</v>
+      </c>
+      <c r="AD40" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AE40" s="2" t="n">
+        <v>10.52</v>
+      </c>
+      <c r="AF40" s="2" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="AG40" s="2" t="n">
+        <v>1.7555</v>
+      </c>
+      <c r="AH40" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI40" s="2" t="n">
+        <v>10.52</v>
+      </c>
+      <c r="AJ40" s="2" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="AK40" s="2" t="n">
+        <v>0.9722</v>
+      </c>
+      <c r="AL40" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AM40" s="2" t="n">
+        <v>10.52</v>
+      </c>
+      <c r="AN40" s="2" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="AO40" s="2" t="n">
+        <v>1.3778</v>
+      </c>
+      <c r="AP40" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AQ40" s="2" t="n">
+        <v>10.52</v>
+      </c>
+      <c r="AR40" s="2" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="AS40" s="2" t="n">
+        <v>1.7555</v>
+      </c>
+      <c r="AT40" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU40" s="2" t="n">
+        <v>10.52</v>
+      </c>
+      <c r="AV40" s="2" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="AW40" s="2" t="n">
+        <v>0.9722</v>
+      </c>
+      <c r="AX40" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AY40" s="2" t="n">
+        <v>10.52</v>
+      </c>
+      <c r="AZ40" s="2" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="BA40" s="2" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>13:57</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>RGC</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="n">
+        <v>10.39</v>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15 13:56:00-04:00</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="n"/>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="n">
+        <v>-1.106</v>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>bull_flag</t>
+        </is>
+      </c>
+      <c r="K41" s="2" t="n">
+        <v>267</v>
+      </c>
+      <c r="L41" s="2" t="n">
+        <v>0.3002466735756122</v>
+      </c>
+      <c r="M41" s="2" t="n">
+        <v>-0.0160295490884178</v>
+      </c>
+      <c r="N41" s="2" t="n">
+        <v>2.456114605523753</v>
+      </c>
+      <c r="O41" s="2" t="n">
+        <v>0.0441213982963213</v>
+      </c>
+      <c r="P41" s="2" t="n">
+        <v>0.0146989165644861</v>
+      </c>
+      <c r="Q41" s="2" t="n">
+        <v>-0.051700077015041</v>
+      </c>
+      <c r="R41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S41" s="2" t="n">
+        <v>2.355651821165821</v>
+      </c>
+      <c r="T41" s="2" t="n">
+        <v>0.0023648744568021</v>
+      </c>
+      <c r="U41" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z41" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC41" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AD41" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE41" s="2" t="n">
+        <v>10.559</v>
+      </c>
+      <c r="AF41" s="2" t="n">
+        <v>0.169</v>
+      </c>
+      <c r="AG41" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AH41" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI41" s="2" t="n">
+        <v>10.559</v>
+      </c>
+      <c r="AJ41" s="2" t="n">
+        <v>0.169</v>
+      </c>
+      <c r="AK41" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AL41" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM41" s="2" t="n">
+        <v>10.559</v>
+      </c>
+      <c r="AN41" s="2" t="n">
+        <v>0.169</v>
+      </c>
+      <c r="AO41" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AP41" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ41" s="2" t="n">
+        <v>10.545</v>
+      </c>
+      <c r="AR41" s="2" t="n">
+        <v>0.155</v>
+      </c>
+      <c r="AS41" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AT41" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU41" s="2" t="n">
+        <v>10.545</v>
+      </c>
+      <c r="AV41" s="2" t="n">
+        <v>0.155</v>
+      </c>
+      <c r="AW41" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AX41" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY41" s="2" t="n">
+        <v>10.545</v>
+      </c>
+      <c r="AZ41" s="2" t="n">
+        <v>0.155</v>
+      </c>
+      <c r="BA41" s="2" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>14:47</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>DNN</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="n">
+        <v>2.29</v>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15 14:46:00-04:00</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="n"/>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="n">
+        <v>0.198</v>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>time</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>vwap_pullback</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="n">
+        <v>317</v>
+      </c>
+      <c r="L42" s="2" t="n">
+        <v>0.0717592431623264</v>
+      </c>
+      <c r="M42" s="2" t="n">
+        <v>-0.0138888750915179</v>
+      </c>
+      <c r="N42" s="2" t="n">
+        <v>1.558963719731424</v>
+      </c>
+      <c r="O42" s="2" t="n">
+        <v>0.0040181443508628</v>
+      </c>
+      <c r="P42" s="2" t="n">
+        <v>0.0107991605194496</v>
+      </c>
+      <c r="Q42" s="2" t="n">
+        <v>-0.0190677287608689</v>
+      </c>
+      <c r="R42" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S42" s="2" t="n">
+        <v>0.839409712255458</v>
+      </c>
+      <c r="T42" s="2" t="n">
+        <v>0.0005912384411099</v>
+      </c>
+      <c r="U42" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V42" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W42" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X42" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y42" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z42" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA42" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB42" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC42" s="2" t="n">
+        <v>1.3317</v>
+      </c>
+      <c r="AD42" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AE42" s="2" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="AF42" s="2" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="AG42" s="2" t="n">
+        <v>1.6633</v>
+      </c>
+      <c r="AH42" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI42" s="2" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="AJ42" s="2" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="AK42" s="2" t="n">
+        <v>0.8333</v>
+      </c>
+      <c r="AL42" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AM42" s="2" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="AN42" s="2" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="AO42" s="2" t="n">
+        <v>1.3317</v>
+      </c>
+      <c r="AP42" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AQ42" s="2" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="AR42" s="2" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="AS42" s="2" t="n">
+        <v>1.6633</v>
+      </c>
+      <c r="AT42" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU42" s="2" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="AV42" s="2" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="AW42" s="2" t="n">
+        <v>0.8333</v>
+      </c>
+      <c r="AX42" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AY42" s="2" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="AZ42" s="2" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="BA42" s="2" t="n">
+        <v>0.00432</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>ERIC</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="n">
+        <v>10.54</v>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15 15:29:00-04:00</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="n"/>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="n"/>
+      <c r="I43" s="2" t="n"/>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>eod_squeeze</t>
+        </is>
+      </c>
+      <c r="K43" s="2" t="n">
+        <v>360</v>
+      </c>
+      <c r="L43" s="2" t="n">
+        <v>0.1059499322970869</v>
+      </c>
+      <c r="M43" s="2" t="n">
+        <v>0.1115657600256756</v>
+      </c>
+      <c r="N43" s="2" t="n">
+        <v>1.682021798397494</v>
+      </c>
+      <c r="O43" s="2" t="n">
+        <v>0.0139724806565413</v>
+      </c>
+      <c r="P43" s="2" t="n">
+        <v>0.0051911529629657</v>
+      </c>
+      <c r="Q43" s="2" t="n">
+        <v>-0.0060975216992221</v>
+      </c>
+      <c r="R43" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S43" s="2" t="n">
+        <v>2.360382216923548</v>
+      </c>
+      <c r="T43" s="2" t="n">
+        <v>0.0032225072538731</v>
+      </c>
+      <c r="U43" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V43" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W43" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X43" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y43" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z43" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA43" s="2" t="n"/>
+      <c r="AB43" s="2" t="n"/>
+      <c r="AC43" s="2" t="n"/>
+      <c r="AD43" s="2" t="n"/>
+      <c r="AE43" s="2" t="n"/>
+      <c r="AF43" s="2" t="n"/>
+      <c r="AG43" s="2" t="n"/>
+      <c r="AH43" s="2" t="n"/>
+      <c r="AI43" s="2" t="n"/>
+      <c r="AJ43" s="2" t="n"/>
+      <c r="AK43" s="2" t="n"/>
+      <c r="AL43" s="2" t="n"/>
+      <c r="AM43" s="2" t="n"/>
+      <c r="AN43" s="2" t="n"/>
+      <c r="AO43" s="2" t="n"/>
+      <c r="AP43" s="2" t="n"/>
+      <c r="AQ43" s="2" t="n"/>
+      <c r="AR43" s="2" t="n"/>
+      <c r="AS43" s="2" t="n"/>
+      <c r="AT43" s="2" t="n"/>
+      <c r="AU43" s="2" t="n"/>
+      <c r="AV43" s="2" t="n"/>
+      <c r="AW43" s="2" t="n"/>
+      <c r="AX43" s="2" t="n"/>
+      <c r="AY43" s="2" t="n"/>
+      <c r="AZ43" s="2" t="n"/>
+      <c r="BA43" s="2" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>DNN</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15 15:29:00-04:00</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="n"/>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="n"/>
+      <c r="I44" s="2" t="n"/>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>eod_squeeze</t>
+        </is>
+      </c>
+      <c r="K44" s="2" t="n">
+        <v>360</v>
+      </c>
+      <c r="L44" s="2" t="n">
+        <v>0.0851851888644841</v>
+      </c>
+      <c r="M44" s="2" t="n">
+        <v>-0.0138888750915179</v>
+      </c>
+      <c r="N44" s="2" t="n">
+        <v>1.479226032483189</v>
+      </c>
+      <c r="O44" s="2" t="n">
+        <v>0.0162908093659825</v>
+      </c>
+      <c r="P44" s="2" t="n">
+        <v>0.0187713733753794</v>
+      </c>
+      <c r="Q44" s="2" t="n">
+        <v>-0.0067795740328615</v>
+      </c>
+      <c r="R44" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S44" s="2" t="n">
+        <v>0.8518589148416754</v>
+      </c>
+      <c r="T44" s="2" t="n">
+        <v>0.0032225072538731</v>
+      </c>
+      <c r="U44" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V44" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W44" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X44" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y44" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z44" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA44" s="2" t="n"/>
+      <c r="AB44" s="2" t="n"/>
+      <c r="AC44" s="2" t="n"/>
+      <c r="AD44" s="2" t="n"/>
+      <c r="AE44" s="2" t="n"/>
+      <c r="AF44" s="2" t="n"/>
+      <c r="AG44" s="2" t="n"/>
+      <c r="AH44" s="2" t="n"/>
+      <c r="AI44" s="2" t="n"/>
+      <c r="AJ44" s="2" t="n"/>
+      <c r="AK44" s="2" t="n"/>
+      <c r="AL44" s="2" t="n"/>
+      <c r="AM44" s="2" t="n"/>
+      <c r="AN44" s="2" t="n"/>
+      <c r="AO44" s="2" t="n"/>
+      <c r="AP44" s="2" t="n"/>
+      <c r="AQ44" s="2" t="n"/>
+      <c r="AR44" s="2" t="n"/>
+      <c r="AS44" s="2" t="n"/>
+      <c r="AT44" s="2" t="n"/>
+      <c r="AU44" s="2" t="n"/>
+      <c r="AV44" s="2" t="n"/>
+      <c r="AW44" s="2" t="n"/>
+      <c r="AX44" s="2" t="n"/>
+      <c r="AY44" s="2" t="n"/>
+      <c r="AZ44" s="2" t="n"/>
+      <c r="BA44" s="2" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>15:43</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>LAC</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="n">
+        <v>2.23</v>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15 15:42:00-04:00</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="n"/>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="n"/>
+      <c r="I45" s="2" t="n"/>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>eod_squeeze</t>
+        </is>
+      </c>
+      <c r="K45" s="2" t="n">
+        <v>373</v>
+      </c>
+      <c r="L45" s="2" t="n">
+        <v>0.091787470216393</v>
+      </c>
+      <c r="M45" s="2" t="n">
+        <v>-0.00483091342307</v>
+      </c>
+      <c r="N45" s="2" t="n">
+        <v>1.000391329512645</v>
+      </c>
+      <c r="O45" s="2" t="n">
+        <v>0.0352824473891444</v>
+      </c>
+      <c r="P45" s="2" t="n">
+        <v>0.0132743321194029</v>
+      </c>
+      <c r="Q45" s="2" t="n">
+        <v>-0.0087719215690703</v>
+      </c>
+      <c r="R45" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S45" s="2" t="n">
+        <v>0.8153648090643967</v>
+      </c>
+      <c r="T45" s="2" t="n">
+        <v>0.0034823983835199</v>
+      </c>
+      <c r="U45" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V45" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W45" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X45" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y45" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z45" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA45" s="2" t="n"/>
+      <c r="AB45" s="2" t="n"/>
+      <c r="AC45" s="2" t="n"/>
+      <c r="AD45" s="2" t="n"/>
+      <c r="AE45" s="2" t="n"/>
+      <c r="AF45" s="2" t="n"/>
+      <c r="AG45" s="2" t="n"/>
+      <c r="AH45" s="2" t="n"/>
+      <c r="AI45" s="2" t="n"/>
+      <c r="AJ45" s="2" t="n"/>
+      <c r="AK45" s="2" t="n"/>
+      <c r="AL45" s="2" t="n"/>
+      <c r="AM45" s="2" t="n"/>
+      <c r="AN45" s="2" t="n"/>
+      <c r="AO45" s="2" t="n"/>
+      <c r="AP45" s="2" t="n"/>
+      <c r="AQ45" s="2" t="n"/>
+      <c r="AR45" s="2" t="n"/>
+      <c r="AS45" s="2" t="n"/>
+      <c r="AT45" s="2" t="n"/>
+      <c r="AU45" s="2" t="n"/>
+      <c r="AV45" s="2" t="n"/>
+      <c r="AW45" s="2" t="n"/>
+      <c r="AX45" s="2" t="n"/>
+      <c r="AY45" s="2" t="n"/>
+      <c r="AZ45" s="2" t="n"/>
+      <c r="BA45" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7277,7 +9411,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7727,6 +9861,186 @@
       <c r="J11" s="2" t="inlineStr">
         <is>
           <t>closed</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>250</v>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>ema_bounce</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>RGC</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>-2.7</v>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="2" t="n"/>
+      <c r="I12" s="2" t="n"/>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>no fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>ema_bounce</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>RGC</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>-4.32</v>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="2" t="n"/>
+      <c r="I13" s="2" t="n"/>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>no fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>350</v>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>bull_flag</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>RGC</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>-4.32</v>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="2" t="n"/>
+      <c r="I14" s="2" t="n"/>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>no fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>550</v>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>bull_flag</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>RGC</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>-7.02</v>
+      </c>
+      <c r="F15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="2" t="n"/>
+      <c r="I15" s="2" t="n"/>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>no fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>vwap_pullback</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>RGC</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="F16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="2" t="n"/>
+      <c r="I16" s="2" t="n"/>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>no fill</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
bot session end 2026-10-16 16:02
</commit_message>
<xml_diff>
--- a/reports/Paper Bot Live.xlsx
+++ b/reports/Paper Bot Live.xlsx
@@ -1880,7 +1880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BA45"/>
+  <dimension ref="A1:BA46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9091,8 +9091,14 @@
           <t>off</t>
         </is>
       </c>
-      <c r="H43" s="2" t="n"/>
-      <c r="I43" s="2" t="n"/>
+      <c r="H43" s="2" t="n">
+        <v>0.063</v>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>next open</t>
+        </is>
+      </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
           <t>eod_squeeze</t>
@@ -9146,33 +9152,87 @@
       <c r="Z43" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA43" s="2" t="n"/>
-      <c r="AB43" s="2" t="n"/>
-      <c r="AC43" s="2" t="n"/>
-      <c r="AD43" s="2" t="n"/>
-      <c r="AE43" s="2" t="n"/>
-      <c r="AF43" s="2" t="n"/>
-      <c r="AG43" s="2" t="n"/>
-      <c r="AH43" s="2" t="n"/>
-      <c r="AI43" s="2" t="n"/>
-      <c r="AJ43" s="2" t="n"/>
-      <c r="AK43" s="2" t="n"/>
-      <c r="AL43" s="2" t="n"/>
-      <c r="AM43" s="2" t="n"/>
-      <c r="AN43" s="2" t="n"/>
-      <c r="AO43" s="2" t="n"/>
-      <c r="AP43" s="2" t="n"/>
-      <c r="AQ43" s="2" t="n"/>
-      <c r="AR43" s="2" t="n"/>
-      <c r="AS43" s="2" t="n"/>
-      <c r="AT43" s="2" t="n"/>
-      <c r="AU43" s="2" t="n"/>
-      <c r="AV43" s="2" t="n"/>
-      <c r="AW43" s="2" t="n"/>
-      <c r="AX43" s="2" t="n"/>
-      <c r="AY43" s="2" t="n"/>
-      <c r="AZ43" s="2" t="n"/>
-      <c r="BA43" s="2" t="n"/>
+      <c r="AA43" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB43" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC43" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AD43" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE43" s="2" t="n">
+        <v>10.5988</v>
+      </c>
+      <c r="AF43" s="2" t="n">
+        <v>0.0588</v>
+      </c>
+      <c r="AG43" s="2" t="n">
+        <v>-0.4898</v>
+      </c>
+      <c r="AH43" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI43" s="2" t="n">
+        <v>10.5988</v>
+      </c>
+      <c r="AJ43" s="2" t="n">
+        <v>0.0588</v>
+      </c>
+      <c r="AK43" s="2" t="n">
+        <v>0.8512</v>
+      </c>
+      <c r="AL43" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AM43" s="2" t="n">
+        <v>10.5988</v>
+      </c>
+      <c r="AN43" s="2" t="n">
+        <v>0.0588</v>
+      </c>
+      <c r="AO43" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AP43" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ43" s="2" t="n">
+        <v>10.595</v>
+      </c>
+      <c r="AR43" s="2" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="AS43" s="2" t="n">
+        <v>-0.4546</v>
+      </c>
+      <c r="AT43" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU43" s="2" t="n">
+        <v>10.595</v>
+      </c>
+      <c r="AV43" s="2" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="AW43" s="2" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="AX43" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AY43" s="2" t="n">
+        <v>10.595</v>
+      </c>
+      <c r="AZ43" s="2" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="BA43" s="2" t="n">
+        <v>0.00094</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -9204,8 +9264,14 @@
           <t>off</t>
         </is>
       </c>
-      <c r="H44" s="2" t="n"/>
-      <c r="I44" s="2" t="n"/>
+      <c r="H44" s="2" t="n">
+        <v>-0.538</v>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>next open</t>
+        </is>
+      </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
           <t>eod_squeeze</t>
@@ -9259,33 +9325,87 @@
       <c r="Z44" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA44" s="2" t="n"/>
-      <c r="AB44" s="2" t="n"/>
-      <c r="AC44" s="2" t="n"/>
-      <c r="AD44" s="2" t="n"/>
-      <c r="AE44" s="2" t="n"/>
-      <c r="AF44" s="2" t="n"/>
-      <c r="AG44" s="2" t="n"/>
-      <c r="AH44" s="2" t="n"/>
-      <c r="AI44" s="2" t="n"/>
-      <c r="AJ44" s="2" t="n"/>
-      <c r="AK44" s="2" t="n"/>
-      <c r="AL44" s="2" t="n"/>
-      <c r="AM44" s="2" t="n"/>
-      <c r="AN44" s="2" t="n"/>
-      <c r="AO44" s="2" t="n"/>
-      <c r="AP44" s="2" t="n"/>
-      <c r="AQ44" s="2" t="n"/>
-      <c r="AR44" s="2" t="n"/>
-      <c r="AS44" s="2" t="n"/>
-      <c r="AT44" s="2" t="n"/>
-      <c r="AU44" s="2" t="n"/>
-      <c r="AV44" s="2" t="n"/>
-      <c r="AW44" s="2" t="n"/>
-      <c r="AX44" s="2" t="n"/>
-      <c r="AY44" s="2" t="n"/>
-      <c r="AZ44" s="2" t="n"/>
-      <c r="BA44" s="2" t="n"/>
+      <c r="AA44" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB44" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC44" s="2" t="n">
+        <v>0.1111</v>
+      </c>
+      <c r="AD44" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE44" s="2" t="n">
+        <v>2.345</v>
+      </c>
+      <c r="AF44" s="2" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="AG44" s="2" t="n">
+        <v>0.1111</v>
+      </c>
+      <c r="AH44" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI44" s="2" t="n">
+        <v>2.345</v>
+      </c>
+      <c r="AJ44" s="2" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="AK44" s="2" t="n">
+        <v>0.1111</v>
+      </c>
+      <c r="AL44" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM44" s="2" t="n">
+        <v>2.345</v>
+      </c>
+      <c r="AN44" s="2" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="AO44" s="2" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="AP44" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ44" s="2" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="AR44" s="2" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="AS44" s="2" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="AT44" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU44" s="2" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="AV44" s="2" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="AW44" s="2" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="AX44" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY44" s="2" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="AZ44" s="2" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="BA44" s="2" t="n">
+        <v>0.00426</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -9317,8 +9437,14 @@
           <t>off</t>
         </is>
       </c>
-      <c r="H45" s="2" t="n"/>
-      <c r="I45" s="2" t="n"/>
+      <c r="H45" s="2" t="n">
+        <v>-1.667</v>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>next open</t>
+        </is>
+      </c>
       <c r="J45" s="2" t="inlineStr">
         <is>
           <t>eod_squeeze</t>
@@ -9372,33 +9498,260 @@
       <c r="Z45" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA45" s="2" t="n"/>
-      <c r="AB45" s="2" t="n"/>
-      <c r="AC45" s="2" t="n"/>
-      <c r="AD45" s="2" t="n"/>
-      <c r="AE45" s="2" t="n"/>
-      <c r="AF45" s="2" t="n"/>
-      <c r="AG45" s="2" t="n"/>
-      <c r="AH45" s="2" t="n"/>
-      <c r="AI45" s="2" t="n"/>
-      <c r="AJ45" s="2" t="n"/>
-      <c r="AK45" s="2" t="n"/>
-      <c r="AL45" s="2" t="n"/>
-      <c r="AM45" s="2" t="n"/>
-      <c r="AN45" s="2" t="n"/>
-      <c r="AO45" s="2" t="n"/>
-      <c r="AP45" s="2" t="n"/>
-      <c r="AQ45" s="2" t="n"/>
-      <c r="AR45" s="2" t="n"/>
-      <c r="AS45" s="2" t="n"/>
-      <c r="AT45" s="2" t="n"/>
-      <c r="AU45" s="2" t="n"/>
-      <c r="AV45" s="2" t="n"/>
-      <c r="AW45" s="2" t="n"/>
-      <c r="AX45" s="2" t="n"/>
-      <c r="AY45" s="2" t="n"/>
-      <c r="AZ45" s="2" t="n"/>
-      <c r="BA45" s="2" t="n"/>
+      <c r="AA45" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB45" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC45" s="2" t="n">
+        <v>-1.4</v>
+      </c>
+      <c r="AD45" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE45" s="2" t="n">
+        <v>2.255</v>
+      </c>
+      <c r="AF45" s="2" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="AG45" s="2" t="n">
+        <v>-1.4</v>
+      </c>
+      <c r="AH45" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI45" s="2" t="n">
+        <v>2.255</v>
+      </c>
+      <c r="AJ45" s="2" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="AK45" s="2" t="n">
+        <v>-1.4</v>
+      </c>
+      <c r="AL45" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM45" s="2" t="n">
+        <v>2.255</v>
+      </c>
+      <c r="AN45" s="2" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="AO45" s="2" t="n">
+        <v>-1.4</v>
+      </c>
+      <c r="AP45" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ45" s="2" t="n">
+        <v>2.255</v>
+      </c>
+      <c r="AR45" s="2" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="AS45" s="2" t="n">
+        <v>-1.4</v>
+      </c>
+      <c r="AT45" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU45" s="2" t="n">
+        <v>2.255</v>
+      </c>
+      <c r="AV45" s="2" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="AW45" s="2" t="n">
+        <v>-1.4</v>
+      </c>
+      <c r="AX45" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY45" s="2" t="n">
+        <v>2.255</v>
+      </c>
+      <c r="AZ45" s="2" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="BA45" s="2" t="n">
+        <v>0.00443</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>14:55</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>FMC</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="n">
+        <v>5.72</v>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16 14:54:00-04:00</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="n"/>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="n">
+        <v>-1.235</v>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>ema_bounce</t>
+        </is>
+      </c>
+      <c r="K46" s="2" t="n">
+        <v>325</v>
+      </c>
+      <c r="L46" s="2" t="n">
+        <v>0.0302313067527439</v>
+      </c>
+      <c r="M46" s="2" t="n">
+        <v>-0.029359424415115</v>
+      </c>
+      <c r="N46" s="2" t="n">
+        <v>1.999813653745339</v>
+      </c>
+      <c r="O46" s="2" t="n">
+        <v>0.0047240496639835</v>
+      </c>
+      <c r="P46" s="2" t="n">
+        <v>0.0120727176893999</v>
+      </c>
+      <c r="Q46" s="2" t="n">
+        <v>-0.0366223618052974</v>
+      </c>
+      <c r="R46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S46" s="2" t="n">
+        <v>1.756114990234857</v>
+      </c>
+      <c r="T46" s="2" t="n">
+        <v>-0.0133585533009195</v>
+      </c>
+      <c r="U46" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC46" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AD46" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE46" s="2" t="n">
+        <v>5.785</v>
+      </c>
+      <c r="AF46" s="2" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="AG46" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AH46" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI46" s="2" t="n">
+        <v>5.785</v>
+      </c>
+      <c r="AJ46" s="2" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="AK46" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AL46" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM46" s="2" t="n">
+        <v>5.785</v>
+      </c>
+      <c r="AN46" s="2" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="AO46" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AP46" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ46" s="2" t="n">
+        <v>5.785</v>
+      </c>
+      <c r="AR46" s="2" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="AS46" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AT46" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU46" s="2" t="n">
+        <v>5.785</v>
+      </c>
+      <c r="AV46" s="2" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="AW46" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AX46" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY46" s="2" t="n">
+        <v>5.785</v>
+      </c>
+      <c r="AZ46" s="2" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="BA46" s="2" t="n">
+        <v>0.00173</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
bot session end 2026-10-19 16:02
</commit_message>
<xml_diff>
--- a/reports/Paper Bot Live.xlsx
+++ b/reports/Paper Bot Live.xlsx
@@ -864,7 +864,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q16"/>
+  <dimension ref="A1:Q19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1866,6 +1866,189 @@
       <c r="Q16" s="2" t="inlineStr">
         <is>
           <t>VWAP pullback: +24.3%, dipped to VWAP 10.06, reclaimed with green bar | news: [Newswire] Fengate Private Equity Acquires Majority Stake in</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>vwap_pullback</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>PBLS</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="F17" s="2" t="n">
+        <v>25.4</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>25.33</v>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>25.47</v>
+      </c>
+      <c r="I17" s="2" t="n">
+        <v>25.54</v>
+      </c>
+      <c r="J17" s="2" t="n">
+        <v>25.25</v>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="n">
+        <v>-2.25</v>
+      </c>
+      <c r="M17" s="2" t="n">
+        <v>-0.5600000000000001</v>
+      </c>
+      <c r="N17" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O17" s="2" t="n"/>
+      <c r="P17" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q17" s="2" t="inlineStr">
+        <is>
+          <t>VWAP pullback: +11.5%, dipped to VWAP 25.32, reclaimed with green bar | news: [Benzinga] Parabilis Medicines To Present Updated Clinical D</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>eod_squeeze</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>CLF</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="F18" s="2" t="n">
+        <v>14.46</v>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>14.19</v>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>14.73</v>
+      </c>
+      <c r="I18" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J18" s="2" t="n">
+        <v>14.17</v>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="n">
+        <v>-2.03</v>
+      </c>
+      <c r="M18" s="2" t="n">
+        <v>-1.01</v>
+      </c>
+      <c r="N18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O18" s="2" t="n"/>
+      <c r="P18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q18" s="2" t="inlineStr">
+        <is>
+          <t>EOD squeeze: +19.1%, within 1% of HOD 14.58, hold to next open | news: [Benzinga] Stock Market Today: Nasdaq 100 Rises as AI Chip R</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>350</v>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>eod_squeeze</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>CLF</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="F19" s="2" t="n">
+        <v>14.46</v>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>14.19</v>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>14.73</v>
+      </c>
+      <c r="I19" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J19" s="2" t="n">
+        <v>14.17</v>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="n">
+        <v>-3.48</v>
+      </c>
+      <c r="M19" s="2" t="n">
+        <v>-0.99</v>
+      </c>
+      <c r="N19" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O19" s="2" t="n"/>
+      <c r="P19" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q19" s="2" t="inlineStr">
+        <is>
+          <t>EOD squeeze: +19.1%, within 1% of HOD 14.58, hold to next open | news: [Benzinga] Stock Market Today: Nasdaq 100 Rises as AI Chip R</t>
         </is>
       </c>
     </row>
@@ -1880,7 +2063,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BA46"/>
+  <dimension ref="A1:BA48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9753,6 +9936,242 @@
         <v>0.00173</v>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>14:51</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>PBLS</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="n">
+        <v>25.33</v>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19 14:50:00-04:00</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="n"/>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="n">
+        <v>-1.571</v>
+      </c>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t>vwap_pullback</t>
+        </is>
+      </c>
+      <c r="K47" s="2" t="n">
+        <v>321</v>
+      </c>
+      <c r="L47" s="2" t="n">
+        <v>0.114945044884315</v>
+      </c>
+      <c r="M47" s="2" t="n">
+        <v>0.0101098699884101</v>
+      </c>
+      <c r="N47" s="2" t="n">
+        <v>0.9477842202978118</v>
+      </c>
+      <c r="O47" s="2" t="n">
+        <v>0.0018451131897441</v>
+      </c>
+      <c r="P47" s="2" t="n">
+        <v>0.0013798451186275</v>
+      </c>
+      <c r="Q47" s="2" t="n">
+        <v>-0.033346036876231</v>
+      </c>
+      <c r="R47" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S47" s="2" t="n">
+        <v>3.233370261995123</v>
+      </c>
+      <c r="T47" s="2" t="n">
+        <v>0.0057743696005978</v>
+      </c>
+      <c r="U47" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V47" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W47" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X47" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y47" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z47" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA47" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB47" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC47" s="2" t="n"/>
+      <c r="AD47" s="2" t="n"/>
+      <c r="AE47" s="2" t="n"/>
+      <c r="AF47" s="2" t="n"/>
+      <c r="AG47" s="2" t="n"/>
+      <c r="AH47" s="2" t="n"/>
+      <c r="AI47" s="2" t="n"/>
+      <c r="AJ47" s="2" t="n"/>
+      <c r="AK47" s="2" t="n"/>
+      <c r="AL47" s="2" t="n"/>
+      <c r="AM47" s="2" t="n"/>
+      <c r="AN47" s="2" t="n"/>
+      <c r="AO47" s="2" t="n"/>
+      <c r="AP47" s="2" t="n"/>
+      <c r="AQ47" s="2" t="n"/>
+      <c r="AR47" s="2" t="n"/>
+      <c r="AS47" s="2" t="n"/>
+      <c r="AT47" s="2" t="n"/>
+      <c r="AU47" s="2" t="n"/>
+      <c r="AV47" s="2" t="n"/>
+      <c r="AW47" s="2" t="n"/>
+      <c r="AX47" s="2" t="n"/>
+      <c r="AY47" s="2" t="n"/>
+      <c r="AZ47" s="2" t="n"/>
+      <c r="BA47" s="2" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>15:41</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>CLF</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="n">
+        <v>14.19</v>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19 15:40:00-04:00</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="n"/>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="n"/>
+      <c r="I48" s="2" t="n"/>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>eod_squeeze</t>
+        </is>
+      </c>
+      <c r="K48" s="2" t="n">
+        <v>371</v>
+      </c>
+      <c r="L48" s="2" t="n">
+        <v>0.1910066465277717</v>
+      </c>
+      <c r="M48" s="2" t="n">
+        <v>0.1716171570417557</v>
+      </c>
+      <c r="N48" s="2" t="n">
+        <v>1.662554928578008</v>
+      </c>
+      <c r="O48" s="2" t="n">
+        <v>0.0373658757717905</v>
+      </c>
+      <c r="P48" s="2" t="n">
+        <v>0.0169726645302865</v>
+      </c>
+      <c r="Q48" s="2" t="n">
+        <v>-0.0099450963544653</v>
+      </c>
+      <c r="R48" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S48" s="2" t="n">
+        <v>2.669655842184292</v>
+      </c>
+      <c r="T48" s="2" t="n">
+        <v>0.0064723255046266</v>
+      </c>
+      <c r="U48" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V48" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W48" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X48" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y48" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z48" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA48" s="2" t="n"/>
+      <c r="AB48" s="2" t="n"/>
+      <c r="AC48" s="2" t="n"/>
+      <c r="AD48" s="2" t="n"/>
+      <c r="AE48" s="2" t="n"/>
+      <c r="AF48" s="2" t="n"/>
+      <c r="AG48" s="2" t="n"/>
+      <c r="AH48" s="2" t="n"/>
+      <c r="AI48" s="2" t="n"/>
+      <c r="AJ48" s="2" t="n"/>
+      <c r="AK48" s="2" t="n"/>
+      <c r="AL48" s="2" t="n"/>
+      <c r="AM48" s="2" t="n"/>
+      <c r="AN48" s="2" t="n"/>
+      <c r="AO48" s="2" t="n"/>
+      <c r="AP48" s="2" t="n"/>
+      <c r="AQ48" s="2" t="n"/>
+      <c r="AR48" s="2" t="n"/>
+      <c r="AS48" s="2" t="n"/>
+      <c r="AT48" s="2" t="n"/>
+      <c r="AU48" s="2" t="n"/>
+      <c r="AV48" s="2" t="n"/>
+      <c r="AW48" s="2" t="n"/>
+      <c r="AX48" s="2" t="n"/>
+      <c r="AY48" s="2" t="n"/>
+      <c r="AZ48" s="2" t="n"/>
+      <c r="BA48" s="2" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9764,7 +10183,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10394,6 +10813,122 @@
       <c r="J16" s="2" t="inlineStr">
         <is>
           <t>no fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>vwap_pullback</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>PBLS</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>-2.25</v>
+      </c>
+      <c r="F17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="2" t="n"/>
+      <c r="I17" s="2" t="n"/>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>no fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>eod_squeeze</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>CLF</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="n">
+        <v>-2.03</v>
+      </c>
+      <c r="F18" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>14.44</v>
+      </c>
+      <c r="I18" s="2" t="n">
+        <v>-1.82</v>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>350</v>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>eod_squeeze</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>CLF</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>-3.48</v>
+      </c>
+      <c r="F19" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>14.44</v>
+      </c>
+      <c r="I19" s="2" t="n">
+        <v>-3.12</v>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>closed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
bot session end 2026-10-20 16:02
</commit_message>
<xml_diff>
--- a/reports/Paper Bot Live.xlsx
+++ b/reports/Paper Bot Live.xlsx
@@ -864,7 +864,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q19"/>
+  <dimension ref="A1:Q22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2049,6 +2049,189 @@
       <c r="Q19" s="2" t="inlineStr">
         <is>
           <t>EOD squeeze: +19.1%, within 1% of HOD 14.58, hold to next open | news: [Benzinga] Stock Market Today: Nasdaq 100 Rises as AI Chip R</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>vwap_pullback</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>CANG</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>66</v>
+      </c>
+      <c r="F20" s="2" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>2.29</v>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="I20" s="2" t="n">
+        <v>2.38</v>
+      </c>
+      <c r="J20" s="2" t="n">
+        <v>2.23</v>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="n">
+        <v>-5.94</v>
+      </c>
+      <c r="M20" s="2" t="n">
+        <v>-2.97</v>
+      </c>
+      <c r="N20" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O20" s="2" t="n"/>
+      <c r="P20" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VWAP pullback: +8.1%, dipped to VWAP 2.32, reclaimed with green bar | news: [Newswire] TheEnergyMag | Energy, Compute, Markets, Stocks, </t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>250</v>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>ema_bounce</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>HSAI</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="F21" s="2" t="n">
+        <v>14.1</v>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>13.96</v>
+      </c>
+      <c r="H21" s="2" t="n">
+        <v>14.24</v>
+      </c>
+      <c r="I21" s="2" t="n">
+        <v>14.38</v>
+      </c>
+      <c r="J21" s="2" t="n">
+        <v>13.94</v>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="n">
+        <v>-2.72</v>
+      </c>
+      <c r="M21" s="2" t="n">
+        <v>-1.09</v>
+      </c>
+      <c r="N21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O21" s="2" t="n"/>
+      <c r="P21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q21" s="2" t="inlineStr">
+        <is>
+          <t>9/21 EMA bounce: tagged 21 EMA 14.04, closed back over 9 EMA | news: [Newswire] Hesai Group to Report Third Quarter 2026 Financia</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>ema_bounce</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>HSAI</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="F22" s="2" t="n">
+        <v>14.1</v>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>13.96</v>
+      </c>
+      <c r="H22" s="2" t="n">
+        <v>14.24</v>
+      </c>
+      <c r="I22" s="2" t="n">
+        <v>14.38</v>
+      </c>
+      <c r="J22" s="2" t="n">
+        <v>13.94</v>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="n">
+        <v>-4.48</v>
+      </c>
+      <c r="M22" s="2" t="n">
+        <v>-1.12</v>
+      </c>
+      <c r="N22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O22" s="2" t="n"/>
+      <c r="P22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q22" s="2" t="inlineStr">
+        <is>
+          <t>9/21 EMA bounce: tagged 21 EMA 14.04, closed back over 9 EMA | news: [Newswire] Hesai Group to Report Third Quarter 2026 Financia</t>
         </is>
       </c>
     </row>
@@ -2063,7 +2246,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BA48"/>
+  <dimension ref="A1:BA58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10089,8 +10272,14 @@
           <t>off</t>
         </is>
       </c>
-      <c r="H48" s="2" t="n"/>
-      <c r="I48" s="2" t="n"/>
+      <c r="H48" s="2" t="n">
+        <v>-1.075</v>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
       <c r="J48" s="2" t="inlineStr">
         <is>
           <t>eod_squeeze</t>
@@ -10144,33 +10333,1583 @@
       <c r="Z48" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA48" s="2" t="n"/>
-      <c r="AB48" s="2" t="n"/>
-      <c r="AC48" s="2" t="n"/>
-      <c r="AD48" s="2" t="n"/>
-      <c r="AE48" s="2" t="n"/>
-      <c r="AF48" s="2" t="n"/>
-      <c r="AG48" s="2" t="n"/>
-      <c r="AH48" s="2" t="n"/>
-      <c r="AI48" s="2" t="n"/>
-      <c r="AJ48" s="2" t="n"/>
-      <c r="AK48" s="2" t="n"/>
-      <c r="AL48" s="2" t="n"/>
-      <c r="AM48" s="2" t="n"/>
-      <c r="AN48" s="2" t="n"/>
-      <c r="AO48" s="2" t="n"/>
-      <c r="AP48" s="2" t="n"/>
-      <c r="AQ48" s="2" t="n"/>
-      <c r="AR48" s="2" t="n"/>
-      <c r="AS48" s="2" t="n"/>
-      <c r="AT48" s="2" t="n"/>
-      <c r="AU48" s="2" t="n"/>
-      <c r="AV48" s="2" t="n"/>
-      <c r="AW48" s="2" t="n"/>
-      <c r="AX48" s="2" t="n"/>
-      <c r="AY48" s="2" t="n"/>
-      <c r="AZ48" s="2" t="n"/>
-      <c r="BA48" s="2" t="n"/>
+      <c r="AA48" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB48" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC48" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AD48" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE48" s="2" t="n">
+        <v>14.4377</v>
+      </c>
+      <c r="AF48" s="2" t="n">
+        <v>0.2477</v>
+      </c>
+      <c r="AG48" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AH48" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI48" s="2" t="n">
+        <v>14.4377</v>
+      </c>
+      <c r="AJ48" s="2" t="n">
+        <v>0.2477</v>
+      </c>
+      <c r="AK48" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AL48" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM48" s="2" t="n">
+        <v>14.4377</v>
+      </c>
+      <c r="AN48" s="2" t="n">
+        <v>0.2477</v>
+      </c>
+      <c r="AO48" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AP48" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ48" s="2" t="n">
+        <v>14.435</v>
+      </c>
+      <c r="AR48" s="2" t="n">
+        <v>0.245</v>
+      </c>
+      <c r="AS48" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AT48" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU48" s="2" t="n">
+        <v>14.435</v>
+      </c>
+      <c r="AV48" s="2" t="n">
+        <v>0.245</v>
+      </c>
+      <c r="AW48" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AX48" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY48" s="2" t="n">
+        <v>14.435</v>
+      </c>
+      <c r="AZ48" s="2" t="n">
+        <v>0.245</v>
+      </c>
+      <c r="BA48" s="2" t="n">
+        <v>0.00069</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>13:28</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>HSAI</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="n">
+        <v>13.96</v>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 13:27:00-04:00</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="n"/>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="n">
+        <v>-1.143</v>
+      </c>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="J49" s="2" t="inlineStr">
+        <is>
+          <t>ema_bounce</t>
+        </is>
+      </c>
+      <c r="K49" s="2" t="n">
+        <v>238</v>
+      </c>
+      <c r="L49" s="2" t="n">
+        <v>0.0905572809121495</v>
+      </c>
+      <c r="M49" s="2" t="n">
+        <v>0.0804953526092662</v>
+      </c>
+      <c r="N49" s="2" t="n">
+        <v>1.283513426620093</v>
+      </c>
+      <c r="O49" s="2" t="n">
+        <v>0.0121395430531656</v>
+      </c>
+      <c r="P49" s="2" t="n">
+        <v>0.0092264124329347</v>
+      </c>
+      <c r="Q49" s="2" t="n">
+        <v>-0.0126138962439802</v>
+      </c>
+      <c r="R49" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S49" s="2" t="n">
+        <v>2.645465336740105</v>
+      </c>
+      <c r="T49" s="2" t="n">
+        <v>0.0037966212475737</v>
+      </c>
+      <c r="U49" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V49" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="W49" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X49" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y49" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z49" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA49" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB49" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC49" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AD49" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE49" s="2" t="n">
+        <v>14.08</v>
+      </c>
+      <c r="AF49" s="2" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="AG49" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AH49" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI49" s="2" t="n">
+        <v>14.08</v>
+      </c>
+      <c r="AJ49" s="2" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="AK49" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AL49" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM49" s="2" t="n">
+        <v>14.08</v>
+      </c>
+      <c r="AN49" s="2" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="AO49" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AP49" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ49" s="2" t="n">
+        <v>14.08</v>
+      </c>
+      <c r="AR49" s="2" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="AS49" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AT49" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU49" s="2" t="n">
+        <v>14.08</v>
+      </c>
+      <c r="AV49" s="2" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="AW49" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AX49" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY49" s="2" t="n">
+        <v>14.08</v>
+      </c>
+      <c r="AZ49" s="2" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="BA49" s="2" t="n">
+        <v>0.00071</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>13:31</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>BRZE</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="n">
+        <v>45.26</v>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 13:30:00-04:00</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="n"/>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="n">
+        <v>-0.587</v>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>time</t>
+        </is>
+      </c>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>ema_bounce</t>
+        </is>
+      </c>
+      <c r="K50" s="2" t="n">
+        <v>241</v>
+      </c>
+      <c r="L50" s="2" t="n">
+        <v>0.5148135712803592</v>
+      </c>
+      <c r="M50" s="2" t="n">
+        <v>0.5156457187643733</v>
+      </c>
+      <c r="N50" s="2" t="n">
+        <v>3.84389096961956</v>
+      </c>
+      <c r="O50" s="2" t="n">
+        <v>0.003203872757401</v>
+      </c>
+      <c r="P50" s="2" t="n">
+        <v>0.0053840470797594</v>
+      </c>
+      <c r="Q50" s="2" t="n">
+        <v>-0.00186442386901</v>
+      </c>
+      <c r="R50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S50" s="2" t="n">
+        <v>3.817822233501799</v>
+      </c>
+      <c r="T50" s="2" t="n">
+        <v>0.0042924005144764</v>
+      </c>
+      <c r="U50" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC50" s="2" t="n">
+        <v>-0.1837</v>
+      </c>
+      <c r="AD50" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE50" s="2" t="n">
+        <v>45.505</v>
+      </c>
+      <c r="AF50" s="2" t="n">
+        <v>0.245</v>
+      </c>
+      <c r="AG50" s="2" t="n">
+        <v>-0.1837</v>
+      </c>
+      <c r="AH50" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI50" s="2" t="n">
+        <v>45.505</v>
+      </c>
+      <c r="AJ50" s="2" t="n">
+        <v>0.245</v>
+      </c>
+      <c r="AK50" s="2" t="n">
+        <v>-0.1837</v>
+      </c>
+      <c r="AL50" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM50" s="2" t="n">
+        <v>45.505</v>
+      </c>
+      <c r="AN50" s="2" t="n">
+        <v>0.245</v>
+      </c>
+      <c r="AO50" s="2" t="n">
+        <v>-0.1837</v>
+      </c>
+      <c r="AP50" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ50" s="2" t="n">
+        <v>45.505</v>
+      </c>
+      <c r="AR50" s="2" t="n">
+        <v>0.245</v>
+      </c>
+      <c r="AS50" s="2" t="n">
+        <v>-0.1837</v>
+      </c>
+      <c r="AT50" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU50" s="2" t="n">
+        <v>45.505</v>
+      </c>
+      <c r="AV50" s="2" t="n">
+        <v>0.245</v>
+      </c>
+      <c r="AW50" s="2" t="n">
+        <v>-0.1837</v>
+      </c>
+      <c r="AX50" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY50" s="2" t="n">
+        <v>45.505</v>
+      </c>
+      <c r="AZ50" s="2" t="n">
+        <v>0.245</v>
+      </c>
+      <c r="BA50" s="2" t="n">
+        <v>0.00022</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>13:37</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>BRZE</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="n">
+        <v>45.47</v>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 13:36:00-04:00</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="n"/>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="n"/>
+      <c r="I51" s="2" t="n"/>
+      <c r="J51" s="2" t="inlineStr">
+        <is>
+          <t>vwap_pullback</t>
+        </is>
+      </c>
+      <c r="K51" s="2" t="n">
+        <v>247</v>
+      </c>
+      <c r="L51" s="2" t="n">
+        <v>0.5144806106969493</v>
+      </c>
+      <c r="M51" s="2" t="n">
+        <v>0.5156457187643733</v>
+      </c>
+      <c r="N51" s="2" t="n">
+        <v>3.823536846097816</v>
+      </c>
+      <c r="O51" s="2" t="n">
+        <v>0.002971792948248</v>
+      </c>
+      <c r="P51" s="2" t="n">
+        <v>0.0005494874705282</v>
+      </c>
+      <c r="Q51" s="2" t="n">
+        <v>-0.0020838170735941</v>
+      </c>
+      <c r="R51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S51" s="2" t="n">
+        <v>3.817602406331014</v>
+      </c>
+      <c r="T51" s="2" t="n">
+        <v>0.0039771435087476</v>
+      </c>
+      <c r="U51" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC51" s="2" t="n"/>
+      <c r="AD51" s="2" t="n"/>
+      <c r="AE51" s="2" t="n"/>
+      <c r="AF51" s="2" t="n"/>
+      <c r="AG51" s="2" t="n"/>
+      <c r="AH51" s="2" t="n"/>
+      <c r="AI51" s="2" t="n"/>
+      <c r="AJ51" s="2" t="n"/>
+      <c r="AK51" s="2" t="n"/>
+      <c r="AL51" s="2" t="n"/>
+      <c r="AM51" s="2" t="n"/>
+      <c r="AN51" s="2" t="n"/>
+      <c r="AO51" s="2" t="n"/>
+      <c r="AP51" s="2" t="n"/>
+      <c r="AQ51" s="2" t="n"/>
+      <c r="AR51" s="2" t="n"/>
+      <c r="AS51" s="2" t="n"/>
+      <c r="AT51" s="2" t="n"/>
+      <c r="AU51" s="2" t="n"/>
+      <c r="AV51" s="2" t="n"/>
+      <c r="AW51" s="2" t="n"/>
+      <c r="AX51" s="2" t="n"/>
+      <c r="AY51" s="2" t="n"/>
+      <c r="AZ51" s="2" t="n"/>
+      <c r="BA51" s="2" t="n">
+        <v>0.00022</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>14:05</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>RCUS</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="n">
+        <v>24.08</v>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 14:03:00-04:00</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="n"/>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>target</t>
+        </is>
+      </c>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>ema_bounce</t>
+        </is>
+      </c>
+      <c r="K52" s="2" t="n">
+        <v>275</v>
+      </c>
+      <c r="L52" s="2" t="n">
+        <v>0.09372180759452139</v>
+      </c>
+      <c r="M52" s="2" t="n">
+        <v>-0.0397470273272927</v>
+      </c>
+      <c r="N52" s="2" t="n">
+        <v>2.452828025918519</v>
+      </c>
+      <c r="O52" s="2" t="n">
+        <v>0.0176266067619339</v>
+      </c>
+      <c r="P52" s="2" t="n">
+        <v>0.0055750630492341</v>
+      </c>
+      <c r="Q52" s="2" t="n">
+        <v>-0.0196356516344432</v>
+      </c>
+      <c r="R52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S52" s="2" t="n">
+        <v>3.186972282156572</v>
+      </c>
+      <c r="T52" s="2" t="n">
+        <v>0.0036791663136381</v>
+      </c>
+      <c r="U52" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W52" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="X52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC52" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AD52" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE52" s="2" t="n">
+        <v>24.19</v>
+      </c>
+      <c r="AF52" s="2" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="AG52" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="AH52" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI52" s="2" t="n">
+        <v>24.19</v>
+      </c>
+      <c r="AJ52" s="2" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="AK52" s="2" t="n">
+        <v>1.8636</v>
+      </c>
+      <c r="AL52" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AM52" s="2" t="n">
+        <v>24.19</v>
+      </c>
+      <c r="AN52" s="2" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="AO52" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AP52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ52" s="2" t="n">
+        <v>24.19</v>
+      </c>
+      <c r="AR52" s="2" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="AS52" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="AT52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU52" s="2" t="n">
+        <v>24.19</v>
+      </c>
+      <c r="AV52" s="2" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="AW52" s="2" t="n">
+        <v>1.8636</v>
+      </c>
+      <c r="AX52" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AY52" s="2" t="n">
+        <v>24.19</v>
+      </c>
+      <c r="AZ52" s="2" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="BA52" s="2" t="n">
+        <v>0.00165</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>14:11</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>CANG</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="n">
+        <v>2.29</v>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 14:08:00-04:00</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="n"/>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="n">
+        <v>-1.4</v>
+      </c>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="J53" s="2" t="inlineStr">
+        <is>
+          <t>vwap_pullback</t>
+        </is>
+      </c>
+      <c r="K53" s="2" t="n">
+        <v>281</v>
+      </c>
+      <c r="L53" s="2" t="n">
+        <v>0.0813953230482888</v>
+      </c>
+      <c r="M53" s="2" t="n">
+        <v>-0.0418605342305855</v>
+      </c>
+      <c r="N53" s="2" t="n">
+        <v>1.293064629741095</v>
+      </c>
+      <c r="O53" s="2" t="n">
+        <v>0.0038466742674956</v>
+      </c>
+      <c r="P53" s="2" t="n">
+        <v>0.0150537836412453</v>
+      </c>
+      <c r="Q53" s="2" t="n">
+        <v>-0.0699999809265137</v>
+      </c>
+      <c r="R53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S53" s="2" t="n">
+        <v>0.8437200595484445</v>
+      </c>
+      <c r="T53" s="2" t="n">
+        <v>0.0040836094386944</v>
+      </c>
+      <c r="U53" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC53" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AD53" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE53" s="2" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="AF53" s="2" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="AG53" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AH53" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI53" s="2" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="AJ53" s="2" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="AK53" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AL53" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM53" s="2" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="AN53" s="2" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="AO53" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AP53" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ53" s="2" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="AR53" s="2" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="AS53" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AT53" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU53" s="2" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="AV53" s="2" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="AW53" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AX53" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY53" s="2" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="AZ53" s="2" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="BA53" s="2" t="n">
+        <v>0.0043</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>14:48</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>XPEV</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="n">
+        <v>9.82</v>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 14:47:00-04:00</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="n"/>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="n">
+        <v>-0.139</v>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>time</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>ema_bounce</t>
+        </is>
+      </c>
+      <c r="K54" s="2" t="n">
+        <v>318</v>
+      </c>
+      <c r="L54" s="2" t="n">
+        <v>0.0743757238631368</v>
+      </c>
+      <c r="M54" s="2" t="n">
+        <v>0.0369164116373117</v>
+      </c>
+      <c r="N54" s="2" t="n">
+        <v>1.599715087213526</v>
+      </c>
+      <c r="O54" s="2" t="n">
+        <v>0.0043044078162073</v>
+      </c>
+      <c r="P54" s="2" t="n">
+        <v>0.0075796315607874</v>
+      </c>
+      <c r="Q54" s="2" t="n">
+        <v>-0.009509440994097101</v>
+      </c>
+      <c r="R54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S54" s="2" t="n">
+        <v>2.292029625316647</v>
+      </c>
+      <c r="T54" s="2" t="n">
+        <v>0.0031051103009329</v>
+      </c>
+      <c r="U54" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X54" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC54" s="2" t="n">
+        <v>0.3923</v>
+      </c>
+      <c r="AD54" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE54" s="2" t="n">
+        <v>9.8901</v>
+      </c>
+      <c r="AF54" s="2" t="n">
+        <v>0.0701</v>
+      </c>
+      <c r="AG54" s="2" t="n">
+        <v>0.3923</v>
+      </c>
+      <c r="AH54" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI54" s="2" t="n">
+        <v>9.8901</v>
+      </c>
+      <c r="AJ54" s="2" t="n">
+        <v>0.0701</v>
+      </c>
+      <c r="AK54" s="2" t="n">
+        <v>0.3923</v>
+      </c>
+      <c r="AL54" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM54" s="2" t="n">
+        <v>9.8901</v>
+      </c>
+      <c r="AN54" s="2" t="n">
+        <v>0.0701</v>
+      </c>
+      <c r="AO54" s="2" t="n">
+        <v>0.3923</v>
+      </c>
+      <c r="AP54" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ54" s="2" t="n">
+        <v>9.8901</v>
+      </c>
+      <c r="AR54" s="2" t="n">
+        <v>0.0701</v>
+      </c>
+      <c r="AS54" s="2" t="n">
+        <v>0.3923</v>
+      </c>
+      <c r="AT54" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU54" s="2" t="n">
+        <v>9.8901</v>
+      </c>
+      <c r="AV54" s="2" t="n">
+        <v>0.0701</v>
+      </c>
+      <c r="AW54" s="2" t="n">
+        <v>0.3923</v>
+      </c>
+      <c r="AX54" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY54" s="2" t="n">
+        <v>9.8901</v>
+      </c>
+      <c r="AZ54" s="2" t="n">
+        <v>0.0701</v>
+      </c>
+      <c r="BA54" s="2" t="n">
+        <v>0.00101</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>15:26</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>XPEV</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="n">
+        <v>9.84</v>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 15:25:00-04:00</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="n"/>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="n">
+        <v>0.244</v>
+      </c>
+      <c r="I55" s="2" t="inlineStr">
+        <is>
+          <t>time</t>
+        </is>
+      </c>
+      <c r="J55" s="2" t="inlineStr">
+        <is>
+          <t>vwap_pullback</t>
+        </is>
+      </c>
+      <c r="K55" s="2" t="n">
+        <v>356</v>
+      </c>
+      <c r="L55" s="2" t="n">
+        <v>0.0711183203320566</v>
+      </c>
+      <c r="M55" s="2" t="n">
+        <v>0.0369164116373117</v>
+      </c>
+      <c r="N55" s="2" t="n">
+        <v>1.540082950768645</v>
+      </c>
+      <c r="O55" s="2" t="n">
+        <v>0.0011559914637337</v>
+      </c>
+      <c r="P55" s="2" t="n">
+        <v>0.0025341887175057</v>
+      </c>
+      <c r="Q55" s="2" t="n">
+        <v>-0.0125125127991878</v>
+      </c>
+      <c r="R55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S55" s="2" t="n">
+        <v>2.288993116273176</v>
+      </c>
+      <c r="T55" s="2" t="n">
+        <v>0.0022831646547765</v>
+      </c>
+      <c r="U55" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X55" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC55" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AD55" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE55" s="2" t="n">
+        <v>9.866300000000001</v>
+      </c>
+      <c r="AF55" s="2" t="n">
+        <v>0.0263</v>
+      </c>
+      <c r="AG55" s="2" t="n">
+        <v>1.9506</v>
+      </c>
+      <c r="AH55" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI55" s="2" t="n">
+        <v>9.866300000000001</v>
+      </c>
+      <c r="AJ55" s="2" t="n">
+        <v>0.0263</v>
+      </c>
+      <c r="AK55" s="2" t="n">
+        <v>1.0457</v>
+      </c>
+      <c r="AL55" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AM55" s="2" t="n">
+        <v>9.866300000000001</v>
+      </c>
+      <c r="AN55" s="2" t="n">
+        <v>0.0263</v>
+      </c>
+      <c r="AO55" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AP55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ55" s="2" t="n">
+        <v>9.865</v>
+      </c>
+      <c r="AR55" s="2" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="AS55" s="2" t="n">
+        <v>2.104</v>
+      </c>
+      <c r="AT55" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU55" s="2" t="n">
+        <v>9.865</v>
+      </c>
+      <c r="AV55" s="2" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="AW55" s="2" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="AX55" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AY55" s="2" t="n">
+        <v>9.865</v>
+      </c>
+      <c r="AZ55" s="2" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="BA55" s="2" t="n">
+        <v>0.00101</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>TLK</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="n">
+        <v>11.59</v>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 15:29:00-04:00</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="n"/>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="n"/>
+      <c r="I56" s="2" t="n"/>
+      <c r="J56" s="2" t="inlineStr">
+        <is>
+          <t>eod_squeeze</t>
+        </is>
+      </c>
+      <c r="K56" s="2" t="n">
+        <v>360</v>
+      </c>
+      <c r="L56" s="2" t="n">
+        <v>0.1138660688969017</v>
+      </c>
+      <c r="M56" s="2" t="n">
+        <v>0.077512003291956</v>
+      </c>
+      <c r="N56" s="2" t="n">
+        <v>2.401478861785644</v>
+      </c>
+      <c r="O56" s="2" t="n">
+        <v>0.0108972857059026</v>
+      </c>
+      <c r="P56" s="2" t="n">
+        <v>0.0042869961623292</v>
+      </c>
+      <c r="Q56" s="2" t="n">
+        <v>-0.0017238113341003</v>
+      </c>
+      <c r="R56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S56" s="2" t="n">
+        <v>2.454438869029388</v>
+      </c>
+      <c r="T56" s="2" t="n">
+        <v>0.0021527299552603</v>
+      </c>
+      <c r="U56" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA56" s="2" t="n"/>
+      <c r="AB56" s="2" t="n"/>
+      <c r="AC56" s="2" t="n"/>
+      <c r="AD56" s="2" t="n"/>
+      <c r="AE56" s="2" t="n"/>
+      <c r="AF56" s="2" t="n"/>
+      <c r="AG56" s="2" t="n"/>
+      <c r="AH56" s="2" t="n"/>
+      <c r="AI56" s="2" t="n"/>
+      <c r="AJ56" s="2" t="n"/>
+      <c r="AK56" s="2" t="n"/>
+      <c r="AL56" s="2" t="n"/>
+      <c r="AM56" s="2" t="n"/>
+      <c r="AN56" s="2" t="n"/>
+      <c r="AO56" s="2" t="n"/>
+      <c r="AP56" s="2" t="n"/>
+      <c r="AQ56" s="2" t="n"/>
+      <c r="AR56" s="2" t="n"/>
+      <c r="AS56" s="2" t="n"/>
+      <c r="AT56" s="2" t="n"/>
+      <c r="AU56" s="2" t="n"/>
+      <c r="AV56" s="2" t="n"/>
+      <c r="AW56" s="2" t="n"/>
+      <c r="AX56" s="2" t="n"/>
+      <c r="AY56" s="2" t="n"/>
+      <c r="AZ56" s="2" t="n"/>
+      <c r="BA56" s="2" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>BRZE</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="n">
+        <v>45.38</v>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 15:29:00-04:00</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="n"/>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="n"/>
+      <c r="I57" s="2" t="n"/>
+      <c r="J57" s="2" t="inlineStr">
+        <is>
+          <t>eod_squeeze</t>
+        </is>
+      </c>
+      <c r="K57" s="2" t="n">
+        <v>360</v>
+      </c>
+      <c r="L57" s="2" t="n">
+        <v>0.5128161887416656</v>
+      </c>
+      <c r="M57" s="2" t="n">
+        <v>0.5156457187643733</v>
+      </c>
+      <c r="N57" s="2" t="n">
+        <v>3.527450597250498</v>
+      </c>
+      <c r="O57" s="2" t="n">
+        <v>0.00164365963832</v>
+      </c>
+      <c r="P57" s="2" t="n">
+        <v>0.0014302936574036</v>
+      </c>
+      <c r="Q57" s="2" t="n">
+        <v>-0.0036176477377616</v>
+      </c>
+      <c r="R57" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S57" s="2" t="n">
+        <v>3.816502796855456</v>
+      </c>
+      <c r="T57" s="2" t="n">
+        <v>0.0021527299552603</v>
+      </c>
+      <c r="U57" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V57" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W57" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X57" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y57" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z57" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA57" s="2" t="n"/>
+      <c r="AB57" s="2" t="n"/>
+      <c r="AC57" s="2" t="n"/>
+      <c r="AD57" s="2" t="n"/>
+      <c r="AE57" s="2" t="n"/>
+      <c r="AF57" s="2" t="n"/>
+      <c r="AG57" s="2" t="n"/>
+      <c r="AH57" s="2" t="n"/>
+      <c r="AI57" s="2" t="n"/>
+      <c r="AJ57" s="2" t="n"/>
+      <c r="AK57" s="2" t="n"/>
+      <c r="AL57" s="2" t="n"/>
+      <c r="AM57" s="2" t="n"/>
+      <c r="AN57" s="2" t="n"/>
+      <c r="AO57" s="2" t="n"/>
+      <c r="AP57" s="2" t="n"/>
+      <c r="AQ57" s="2" t="n"/>
+      <c r="AR57" s="2" t="n"/>
+      <c r="AS57" s="2" t="n"/>
+      <c r="AT57" s="2" t="n"/>
+      <c r="AU57" s="2" t="n"/>
+      <c r="AV57" s="2" t="n"/>
+      <c r="AW57" s="2" t="n"/>
+      <c r="AX57" s="2" t="n"/>
+      <c r="AY57" s="2" t="n"/>
+      <c r="AZ57" s="2" t="n"/>
+      <c r="BA57" s="2" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>15:35</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>XPEV</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="n">
+        <v>9.84</v>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 15:34:00-04:00</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="n"/>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="n"/>
+      <c r="I58" s="2" t="n"/>
+      <c r="J58" s="2" t="inlineStr">
+        <is>
+          <t>eod_squeeze</t>
+        </is>
+      </c>
+      <c r="K58" s="2" t="n">
+        <v>365</v>
+      </c>
+      <c r="L58" s="2" t="n">
+        <v>0.075461421492464</v>
+      </c>
+      <c r="M58" s="2" t="n">
+        <v>0.0369164116373117</v>
+      </c>
+      <c r="N58" s="2" t="n">
+        <v>1.537655622122121</v>
+      </c>
+      <c r="O58" s="2" t="n">
+        <v>0.0051440260165827</v>
+      </c>
+      <c r="P58" s="2" t="n">
+        <v>0.0065623154693103</v>
+      </c>
+      <c r="Q58" s="2" t="n">
+        <v>-0.0085085125219636</v>
+      </c>
+      <c r="R58" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S58" s="2" t="n">
+        <v>2.293039653191522</v>
+      </c>
+      <c r="T58" s="2" t="n">
+        <v>0.0026485092221633</v>
+      </c>
+      <c r="U58" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V58" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W58" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X58" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y58" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z58" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA58" s="2" t="n"/>
+      <c r="AB58" s="2" t="n"/>
+      <c r="AC58" s="2" t="n"/>
+      <c r="AD58" s="2" t="n"/>
+      <c r="AE58" s="2" t="n"/>
+      <c r="AF58" s="2" t="n"/>
+      <c r="AG58" s="2" t="n"/>
+      <c r="AH58" s="2" t="n"/>
+      <c r="AI58" s="2" t="n"/>
+      <c r="AJ58" s="2" t="n"/>
+      <c r="AK58" s="2" t="n"/>
+      <c r="AL58" s="2" t="n"/>
+      <c r="AM58" s="2" t="n"/>
+      <c r="AN58" s="2" t="n"/>
+      <c r="AO58" s="2" t="n"/>
+      <c r="AP58" s="2" t="n"/>
+      <c r="AQ58" s="2" t="n"/>
+      <c r="AR58" s="2" t="n"/>
+      <c r="AS58" s="2" t="n"/>
+      <c r="AT58" s="2" t="n"/>
+      <c r="AU58" s="2" t="n"/>
+      <c r="AV58" s="2" t="n"/>
+      <c r="AW58" s="2" t="n"/>
+      <c r="AX58" s="2" t="n"/>
+      <c r="AY58" s="2" t="n"/>
+      <c r="AZ58" s="2" t="n"/>
+      <c r="BA58" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -10183,7 +11922,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J19"/>
+  <dimension ref="A1:J22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10927,6 +12666,126 @@
         <v>-3.12</v>
       </c>
       <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>vwap_pullback</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>CANG</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>-5.94</v>
+      </c>
+      <c r="F20" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="I20" s="2" t="n">
+        <v>-2.1</v>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>250</v>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>ema_bounce</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>HSAI</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>-2.72</v>
+      </c>
+      <c r="F21" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H21" s="2" t="n">
+        <v>14.08</v>
+      </c>
+      <c r="I21" s="2" t="n">
+        <v>-1.95</v>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>ema_bounce</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>HSAI</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="n">
+        <v>-4.48</v>
+      </c>
+      <c r="F22" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="H22" s="2" t="n">
+        <v>14.08</v>
+      </c>
+      <c r="I22" s="2" t="n">
+        <v>-3.12</v>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
         <is>
           <t>closed</t>
         </is>

</xml_diff>

<commit_message>
bot session end 2026-10-21 16:02
</commit_message>
<xml_diff>
--- a/reports/Paper Bot Live.xlsx
+++ b/reports/Paper Bot Live.xlsx
@@ -864,7 +864,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q22"/>
+  <dimension ref="A1:Q27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2232,6 +2232,311 @@
       <c r="Q22" s="2" t="inlineStr">
         <is>
           <t>9/21 EMA bounce: tagged 21 EMA 14.04, closed back over 9 EMA | news: [Newswire] Hesai Group to Report Third Quarter 2026 Financia</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="n">
+        <v>350</v>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>eod_squeeze</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>TLK</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="F23" s="2" t="n">
+        <v>11.66</v>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>11.59</v>
+      </c>
+      <c r="H23" s="2" t="n">
+        <v>11.73</v>
+      </c>
+      <c r="I23" s="2" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="J23" s="2" t="n">
+        <v>11.76</v>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>next open</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="M23" s="2" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="N23" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O23" s="2" t="n"/>
+      <c r="P23" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q23" s="2" t="inlineStr">
+        <is>
+          <t>EOD squeeze: +11.4%, within 1% of HOD 11.66, hold to next open | news: [Newswire] ORCL Stock Price | Oracle Corp. Stock Quote (U.S.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>vwap_pullback</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>WULF</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="F24" s="2" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>12.64</v>
+      </c>
+      <c r="H24" s="2" t="n">
+        <v>12.76</v>
+      </c>
+      <c r="I24" s="2" t="n">
+        <v>12.82</v>
+      </c>
+      <c r="J24" s="2" t="n">
+        <v>12.62</v>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="n">
+        <v>-1.2</v>
+      </c>
+      <c r="M24" s="2" t="n">
+        <v>-0.6</v>
+      </c>
+      <c r="N24" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O24" s="2" t="n"/>
+      <c r="P24" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q24" s="2" t="inlineStr">
+        <is>
+          <t>VWAP pullback: +5.5%, dipped to VWAP 12.63, reclaimed with green bar | news: [Benzinga] 10 Information Technology Stocks With Whale Alert</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>250</v>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>ema_bounce</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>AHT</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="F25" s="2" t="n">
+        <v>2.53</v>
+      </c>
+      <c r="G25" s="2" t="n">
+        <v>2.45</v>
+      </c>
+      <c r="H25" s="2" t="n">
+        <v>2.61</v>
+      </c>
+      <c r="I25" s="2" t="n">
+        <v>2.69</v>
+      </c>
+      <c r="J25" s="2" t="n">
+        <v>2.69</v>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>target</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="n">
+        <v>3.76</v>
+      </c>
+      <c r="M25" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="N25" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O25" s="2" t="n"/>
+      <c r="P25" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q25" s="2" t="inlineStr">
+        <is>
+          <t>9/21 EMA bounce: tagged 21 EMA 2.49, closed back over 9 EMA | news: [Benzinga] Ashford Hospitality Trust Announces $17 Million A</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>ema_bounce</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>AHT</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="F26" s="2" t="n">
+        <v>2.53</v>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>2.45</v>
+      </c>
+      <c r="H26" s="2" t="n">
+        <v>2.61</v>
+      </c>
+      <c r="I26" s="2" t="n">
+        <v>2.69</v>
+      </c>
+      <c r="J26" s="2" t="n">
+        <v>2.69</v>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>target</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="M26" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="N26" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O26" s="2" t="n"/>
+      <c r="P26" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q26" s="2" t="inlineStr">
+        <is>
+          <t>9/21 EMA bounce: tagged 21 EMA 2.49, closed back over 9 EMA | news: [Benzinga] Ashford Hospitality Trust Announces $17 Million A</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="n">
+        <v>550</v>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>afternoon_hod</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>APLD</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="F27" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="G27" s="2" t="n">
+        <v>20.73</v>
+      </c>
+      <c r="H27" s="2" t="n">
+        <v>21.27</v>
+      </c>
+      <c r="I27" s="2" t="n">
+        <v>21.54</v>
+      </c>
+      <c r="J27" s="2" t="n">
+        <v>21.54</v>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>target</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="M27" s="2" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="N27" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O27" s="2" t="n"/>
+      <c r="P27" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q27" s="2" t="inlineStr">
+        <is>
+          <t>Afternoon HOD: +8.5%, new high 20.94 after 1pm on 1.5x vol | news: [Benzinga] Soluna Holdings and Applied Digital Form Strategi</t>
         </is>
       </c>
     </row>
@@ -2246,7 +2551,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BA58"/>
+  <dimension ref="A1:BA82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11602,8 +11907,14 @@
           <t>off</t>
         </is>
       </c>
-      <c r="H56" s="2" t="n"/>
-      <c r="I56" s="2" t="n"/>
+      <c r="H56" s="2" t="n">
+        <v>1.429</v>
+      </c>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>next open</t>
+        </is>
+      </c>
       <c r="J56" s="2" t="inlineStr">
         <is>
           <t>eod_squeeze</t>
@@ -11657,33 +11968,87 @@
       <c r="Z56" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA56" s="2" t="n"/>
-      <c r="AB56" s="2" t="n"/>
-      <c r="AC56" s="2" t="n"/>
-      <c r="AD56" s="2" t="n"/>
-      <c r="AE56" s="2" t="n"/>
-      <c r="AF56" s="2" t="n"/>
-      <c r="AG56" s="2" t="n"/>
-      <c r="AH56" s="2" t="n"/>
-      <c r="AI56" s="2" t="n"/>
-      <c r="AJ56" s="2" t="n"/>
-      <c r="AK56" s="2" t="n"/>
-      <c r="AL56" s="2" t="n"/>
-      <c r="AM56" s="2" t="n"/>
-      <c r="AN56" s="2" t="n"/>
-      <c r="AO56" s="2" t="n"/>
-      <c r="AP56" s="2" t="n"/>
-      <c r="AQ56" s="2" t="n"/>
-      <c r="AR56" s="2" t="n"/>
-      <c r="AS56" s="2" t="n"/>
-      <c r="AT56" s="2" t="n"/>
-      <c r="AU56" s="2" t="n"/>
-      <c r="AV56" s="2" t="n"/>
-      <c r="AW56" s="2" t="n"/>
-      <c r="AX56" s="2" t="n"/>
-      <c r="AY56" s="2" t="n"/>
-      <c r="AZ56" s="2" t="n"/>
-      <c r="BA56" s="2" t="n"/>
+      <c r="AA56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC56" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AD56" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AE56" s="2" t="n">
+        <v>11.64</v>
+      </c>
+      <c r="AF56" s="2" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="AG56" s="2" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="AH56" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI56" s="2" t="n">
+        <v>11.64</v>
+      </c>
+      <c r="AJ56" s="2" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="AK56" s="2" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AL56" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AM56" s="2" t="n">
+        <v>11.64</v>
+      </c>
+      <c r="AN56" s="2" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="AO56" s="2" t="n">
+        <v>1.9038</v>
+      </c>
+      <c r="AP56" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AQ56" s="2" t="n">
+        <v>11.6399</v>
+      </c>
+      <c r="AR56" s="2" t="n">
+        <v>0.0499</v>
+      </c>
+      <c r="AS56" s="2" t="n">
+        <v>2.8076</v>
+      </c>
+      <c r="AT56" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU56" s="2" t="n">
+        <v>11.6399</v>
+      </c>
+      <c r="AV56" s="2" t="n">
+        <v>0.0499</v>
+      </c>
+      <c r="AW56" s="2" t="n">
+        <v>0.7014</v>
+      </c>
+      <c r="AX56" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AY56" s="2" t="n">
+        <v>11.6399</v>
+      </c>
+      <c r="AZ56" s="2" t="n">
+        <v>0.0499</v>
+      </c>
+      <c r="BA56" s="2" t="n">
+        <v>0.00086</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -11715,8 +12080,14 @@
           <t>off</t>
         </is>
       </c>
-      <c r="H57" s="2" t="n"/>
-      <c r="I57" s="2" t="n"/>
+      <c r="H57" s="2" t="n">
+        <v>-0.654</v>
+      </c>
+      <c r="I57" s="2" t="inlineStr">
+        <is>
+          <t>next open</t>
+        </is>
+      </c>
       <c r="J57" s="2" t="inlineStr">
         <is>
           <t>eod_squeeze</t>
@@ -11770,8 +12141,12 @@
       <c r="Z57" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA57" s="2" t="n"/>
-      <c r="AB57" s="2" t="n"/>
+      <c r="AA57" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB57" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="AC57" s="2" t="n"/>
       <c r="AD57" s="2" t="n"/>
       <c r="AE57" s="2" t="n"/>
@@ -11796,7 +12171,9 @@
       <c r="AX57" s="2" t="n"/>
       <c r="AY57" s="2" t="n"/>
       <c r="AZ57" s="2" t="n"/>
-      <c r="BA57" s="2" t="n"/>
+      <c r="BA57" s="2" t="n">
+        <v>0.00022</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -11828,8 +12205,14 @@
           <t>off</t>
         </is>
       </c>
-      <c r="H58" s="2" t="n"/>
-      <c r="I58" s="2" t="n"/>
+      <c r="H58" s="2" t="n">
+        <v>-5.25</v>
+      </c>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>next open</t>
+        </is>
+      </c>
       <c r="J58" s="2" t="inlineStr">
         <is>
           <t>eod_squeeze</t>
@@ -11883,33 +12266,3987 @@
       <c r="Z58" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA58" s="2" t="n"/>
-      <c r="AB58" s="2" t="n"/>
-      <c r="AC58" s="2" t="n"/>
-      <c r="AD58" s="2" t="n"/>
-      <c r="AE58" s="2" t="n"/>
-      <c r="AF58" s="2" t="n"/>
-      <c r="AG58" s="2" t="n"/>
-      <c r="AH58" s="2" t="n"/>
-      <c r="AI58" s="2" t="n"/>
-      <c r="AJ58" s="2" t="n"/>
-      <c r="AK58" s="2" t="n"/>
-      <c r="AL58" s="2" t="n"/>
-      <c r="AM58" s="2" t="n"/>
-      <c r="AN58" s="2" t="n"/>
-      <c r="AO58" s="2" t="n"/>
-      <c r="AP58" s="2" t="n"/>
-      <c r="AQ58" s="2" t="n"/>
-      <c r="AR58" s="2" t="n"/>
-      <c r="AS58" s="2" t="n"/>
-      <c r="AT58" s="2" t="n"/>
-      <c r="AU58" s="2" t="n"/>
-      <c r="AV58" s="2" t="n"/>
-      <c r="AW58" s="2" t="n"/>
-      <c r="AX58" s="2" t="n"/>
-      <c r="AY58" s="2" t="n"/>
-      <c r="AZ58" s="2" t="n"/>
-      <c r="BA58" s="2" t="n"/>
+      <c r="AA58" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB58" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC58" s="2" t="n">
+        <v>-6.3334</v>
+      </c>
+      <c r="AD58" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE58" s="2" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="AF58" s="2" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="AG58" s="2" t="n">
+        <v>-6.3334</v>
+      </c>
+      <c r="AH58" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI58" s="2" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="AJ58" s="2" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="AK58" s="2" t="n">
+        <v>-6.3334</v>
+      </c>
+      <c r="AL58" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM58" s="2" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="AN58" s="2" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="AO58" s="2" t="n">
+        <v>-6.3334</v>
+      </c>
+      <c r="AP58" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ58" s="2" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="AR58" s="2" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="AS58" s="2" t="n">
+        <v>-6.3334</v>
+      </c>
+      <c r="AT58" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU58" s="2" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="AV58" s="2" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="AW58" s="2" t="n">
+        <v>-6.3334</v>
+      </c>
+      <c r="AX58" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY58" s="2" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="AZ58" s="2" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="BA58" s="2" t="n">
+        <v>0.00101</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>10:58</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>WFRD</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="n">
+        <v>83.73</v>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21 10:57:00-04:00</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="n"/>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="n">
+        <v>-1.406</v>
+      </c>
+      <c r="I59" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="J59" s="2" t="inlineStr">
+        <is>
+          <t>vwap_pullback</t>
+        </is>
+      </c>
+      <c r="K59" s="2" t="n">
+        <v>88</v>
+      </c>
+      <c r="L59" s="2" t="n">
+        <v>0.0587346089891849</v>
+      </c>
+      <c r="M59" s="2" t="n">
+        <v>0.0470129005432313</v>
+      </c>
+      <c r="N59" s="2" t="n">
+        <v>1.240442109503898</v>
+      </c>
+      <c r="O59" s="2" t="n">
+        <v>0.0002604287086194</v>
+      </c>
+      <c r="P59" s="2" t="n">
+        <v>0.0032142857142856</v>
+      </c>
+      <c r="Q59" s="2" t="n">
+        <v>-0.0172564902071062</v>
+      </c>
+      <c r="R59" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S59" s="2" t="n">
+        <v>4.430816798843313</v>
+      </c>
+      <c r="T59" s="2" t="n">
+        <v>0.0025746590408104</v>
+      </c>
+      <c r="U59" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V59" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="W59" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X59" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y59" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z59" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA59" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB59" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC59" s="2" t="n">
+        <v>0.3684</v>
+      </c>
+      <c r="AD59" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AE59" s="2" t="n">
+        <v>83.92</v>
+      </c>
+      <c r="AF59" s="2" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="AG59" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AH59" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI59" s="2" t="n">
+        <v>83.92</v>
+      </c>
+      <c r="AJ59" s="2" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="AK59" s="2" t="n">
+        <v>0.8552999999999999</v>
+      </c>
+      <c r="AL59" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AM59" s="2" t="n">
+        <v>83.92</v>
+      </c>
+      <c r="AN59" s="2" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="AO59" s="2" t="n">
+        <v>0.3684</v>
+      </c>
+      <c r="AP59" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AQ59" s="2" t="n">
+        <v>83.92</v>
+      </c>
+      <c r="AR59" s="2" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="AS59" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AT59" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU59" s="2" t="n">
+        <v>83.92</v>
+      </c>
+      <c r="AV59" s="2" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="AW59" s="2" t="n">
+        <v>0.8552999999999999</v>
+      </c>
+      <c r="AX59" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AY59" s="2" t="n">
+        <v>83.92</v>
+      </c>
+      <c r="AZ59" s="2" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="BA59" s="2" t="n">
+        <v>0.00524</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>10:58</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>ROIV</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="n">
+        <v>36.94</v>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21 10:57:00-04:00</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="n"/>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="n">
+        <v>-1.261</v>
+      </c>
+      <c r="I60" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="J60" s="2" t="inlineStr">
+        <is>
+          <t>vwap_pullback</t>
+        </is>
+      </c>
+      <c r="K60" s="2" t="n">
+        <v>88</v>
+      </c>
+      <c r="L60" s="2" t="n">
+        <v>0.06257163481853099</v>
+      </c>
+      <c r="M60" s="2" t="n">
+        <v>0.09851095709579601</v>
+      </c>
+      <c r="N60" s="2" t="n">
+        <v>1.776154488737042</v>
+      </c>
+      <c r="O60" s="2" t="n">
+        <v>0.0039891301899144</v>
+      </c>
+      <c r="P60" s="2" t="n">
+        <v>0.0044468277663906</v>
+      </c>
+      <c r="Q60" s="2" t="n">
+        <v>-0.0329684499573245</v>
+      </c>
+      <c r="R60" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S60" s="2" t="n">
+        <v>3.613751719085116</v>
+      </c>
+      <c r="T60" s="2" t="n">
+        <v>0.0025746590408104</v>
+      </c>
+      <c r="U60" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V60" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="W60" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="X60" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y60" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z60" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA60" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB60" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC60" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AD60" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AE60" s="2" t="n">
+        <v>37.11</v>
+      </c>
+      <c r="AF60" s="2" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="AG60" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AH60" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI60" s="2" t="n">
+        <v>37.11</v>
+      </c>
+      <c r="AJ60" s="2" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="AK60" s="2" t="n">
+        <v>0.8088</v>
+      </c>
+      <c r="AL60" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AM60" s="2" t="n">
+        <v>37.11</v>
+      </c>
+      <c r="AN60" s="2" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="AO60" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AP60" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AQ60" s="2" t="n">
+        <v>37.105</v>
+      </c>
+      <c r="AR60" s="2" t="n">
+        <v>0.165</v>
+      </c>
+      <c r="AS60" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AT60" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU60" s="2" t="n">
+        <v>37.105</v>
+      </c>
+      <c r="AV60" s="2" t="n">
+        <v>0.165</v>
+      </c>
+      <c r="AW60" s="2" t="n">
+        <v>0.8333</v>
+      </c>
+      <c r="AX60" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AY60" s="2" t="n">
+        <v>37.105</v>
+      </c>
+      <c r="AZ60" s="2" t="n">
+        <v>0.165</v>
+      </c>
+      <c r="BA60" s="2" t="n">
+        <v>0.00054</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>10:58</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>AHT</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="n">
+        <v>2.45</v>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21 10:57:00-04:00</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="n"/>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I61" s="2" t="inlineStr">
+        <is>
+          <t>target</t>
+        </is>
+      </c>
+      <c r="J61" s="2" t="inlineStr">
+        <is>
+          <t>ema_bounce</t>
+        </is>
+      </c>
+      <c r="K61" s="2" t="n">
+        <v>88</v>
+      </c>
+      <c r="L61" s="2" t="n">
+        <v>0.4022346614269632</v>
+      </c>
+      <c r="M61" s="2" t="n">
+        <v>0.3351956177865058</v>
+      </c>
+      <c r="N61" s="2" t="n">
+        <v>8.195914992210318</v>
+      </c>
+      <c r="O61" s="2" t="n">
+        <v>0.0400584169240663</v>
+      </c>
+      <c r="P61" s="2" t="n">
+        <v>0.0239043787614448</v>
+      </c>
+      <c r="Q61" s="2" t="n">
+        <v>-0.0271317578731731</v>
+      </c>
+      <c r="R61" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S61" s="2" t="n">
+        <v>0.9202827493441932</v>
+      </c>
+      <c r="T61" s="2" t="n">
+        <v>0.0025746590408104</v>
+      </c>
+      <c r="U61" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V61" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W61" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X61" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y61" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z61" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA61" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB61" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC61" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AD61" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE61" s="2" t="n">
+        <v>2.5112</v>
+      </c>
+      <c r="AF61" s="2" t="n">
+        <v>0.0612</v>
+      </c>
+      <c r="AG61" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="AH61" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI61" s="2" t="n">
+        <v>2.5112</v>
+      </c>
+      <c r="AJ61" s="2" t="n">
+        <v>0.0612</v>
+      </c>
+      <c r="AK61" s="2" t="n">
+        <v>0.8178</v>
+      </c>
+      <c r="AL61" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AM61" s="2" t="n">
+        <v>2.5112</v>
+      </c>
+      <c r="AN61" s="2" t="n">
+        <v>0.0612</v>
+      </c>
+      <c r="AO61" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AP61" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ61" s="2" t="n">
+        <v>2.505</v>
+      </c>
+      <c r="AR61" s="2" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="AS61" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="AT61" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU61" s="2" t="n">
+        <v>2.505</v>
+      </c>
+      <c r="AV61" s="2" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="AW61" s="2" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="AX61" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AY61" s="2" t="n">
+        <v>2.505</v>
+      </c>
+      <c r="AZ61" s="2" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="BA61" s="2" t="n">
+        <v>0.00398</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>10:58</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>ECHO</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="n">
+        <v>91.90000000000001</v>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21 10:57:00-04:00</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="n"/>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="n">
+        <v>0.422</v>
+      </c>
+      <c r="I62" s="2" t="inlineStr">
+        <is>
+          <t>breakeven</t>
+        </is>
+      </c>
+      <c r="J62" s="2" t="inlineStr">
+        <is>
+          <t>ema_bounce</t>
+        </is>
+      </c>
+      <c r="K62" s="2" t="n">
+        <v>88</v>
+      </c>
+      <c r="L62" s="2" t="n">
+        <v>0.0724621157594378</v>
+      </c>
+      <c r="M62" s="2" t="n">
+        <v>0.0491955090870073</v>
+      </c>
+      <c r="N62" s="2" t="n">
+        <v>1.139281437820044</v>
+      </c>
+      <c r="O62" s="2" t="n">
+        <v>0.0070404993171284</v>
+      </c>
+      <c r="P62" s="2" t="n">
+        <v>0.0080949974476731</v>
+      </c>
+      <c r="Q62" s="2" t="n">
+        <v>-0.0060079129288076</v>
+      </c>
+      <c r="R62" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S62" s="2" t="n">
+        <v>4.52882896920065</v>
+      </c>
+      <c r="T62" s="2" t="n">
+        <v>0.0025746590408104</v>
+      </c>
+      <c r="U62" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V62" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W62" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="X62" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y62" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z62" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA62" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB62" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC62" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AD62" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AE62" s="2" t="n">
+        <v>92.66</v>
+      </c>
+      <c r="AF62" s="2" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="AG62" s="2" t="n">
+        <v>0.2237</v>
+      </c>
+      <c r="AH62" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI62" s="2" t="n">
+        <v>92.66</v>
+      </c>
+      <c r="AJ62" s="2" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="AK62" s="2" t="n">
+        <v>1.2138</v>
+      </c>
+      <c r="AL62" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AM62" s="2" t="n">
+        <v>92.66</v>
+      </c>
+      <c r="AN62" s="2" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="AO62" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AP62" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AQ62" s="2" t="n">
+        <v>92.65000000000001</v>
+      </c>
+      <c r="AR62" s="2" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="AS62" s="2" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="AT62" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU62" s="2" t="n">
+        <v>92.65000000000001</v>
+      </c>
+      <c r="AV62" s="2" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="AW62" s="2" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="AX62" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AY62" s="2" t="n">
+        <v>92.65000000000001</v>
+      </c>
+      <c r="AZ62" s="2" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="BA62" s="2" t="n">
+        <v>0.00119</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>11:02</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>WULF</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="n">
+        <v>12.62</v>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21 11:01:00-04:00</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="n"/>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="n">
+        <v>-1.19</v>
+      </c>
+      <c r="I63" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="J63" s="2" t="inlineStr">
+        <is>
+          <t>ema_bounce</t>
+        </is>
+      </c>
+      <c r="K63" s="2" t="n">
+        <v>92</v>
+      </c>
+      <c r="L63" s="2" t="n">
+        <v>0.0582847457056467</v>
+      </c>
+      <c r="M63" s="2" t="n">
+        <v>0.0574520871967993</v>
+      </c>
+      <c r="N63" s="2" t="n">
+        <v>1.07277050811925</v>
+      </c>
+      <c r="O63" s="2" t="n">
+        <v>0.0066292207888425</v>
+      </c>
+      <c r="P63" s="2" t="n">
+        <v>0.0070810415324038</v>
+      </c>
+      <c r="Q63" s="2" t="n">
+        <v>-0.0147286500776616</v>
+      </c>
+      <c r="R63" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S63" s="2" t="n">
+        <v>2.542389088202698</v>
+      </c>
+      <c r="T63" s="2" t="n">
+        <v>0.0024995009966179</v>
+      </c>
+      <c r="U63" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V63" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W63" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X63" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y63" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z63" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA63" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB63" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC63" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AD63" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE63" s="2" t="n">
+        <v>12.705</v>
+      </c>
+      <c r="AF63" s="2" t="n">
+        <v>0.08500000000000001</v>
+      </c>
+      <c r="AG63" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AH63" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI63" s="2" t="n">
+        <v>12.705</v>
+      </c>
+      <c r="AJ63" s="2" t="n">
+        <v>0.08500000000000001</v>
+      </c>
+      <c r="AK63" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AL63" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM63" s="2" t="n">
+        <v>12.705</v>
+      </c>
+      <c r="AN63" s="2" t="n">
+        <v>0.08500000000000001</v>
+      </c>
+      <c r="AO63" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AP63" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ63" s="2" t="n">
+        <v>12.705</v>
+      </c>
+      <c r="AR63" s="2" t="n">
+        <v>0.08500000000000001</v>
+      </c>
+      <c r="AS63" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AT63" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU63" s="2" t="n">
+        <v>12.705</v>
+      </c>
+      <c r="AV63" s="2" t="n">
+        <v>0.08500000000000001</v>
+      </c>
+      <c r="AW63" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AX63" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY63" s="2" t="n">
+        <v>12.705</v>
+      </c>
+      <c r="AZ63" s="2" t="n">
+        <v>0.08500000000000001</v>
+      </c>
+      <c r="BA63" s="2" t="n">
+        <v>0.00079</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>11:05</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>ROIV</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="n">
+        <v>36.93</v>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21 11:04:00-04:00</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="n"/>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="n">
+        <v>-1.16</v>
+      </c>
+      <c r="I64" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="J64" s="2" t="inlineStr">
+        <is>
+          <t>ema_bounce</t>
+        </is>
+      </c>
+      <c r="K64" s="2" t="n">
+        <v>95</v>
+      </c>
+      <c r="L64" s="2" t="n">
+        <v>0.0661512455446038</v>
+      </c>
+      <c r="M64" s="2" t="n">
+        <v>0.09851095709579601</v>
+      </c>
+      <c r="N64" s="2" t="n">
+        <v>1.739997591639858</v>
+      </c>
+      <c r="O64" s="2" t="n">
+        <v>0.0071875149227798</v>
+      </c>
+      <c r="P64" s="2" t="n">
+        <v>0.008058005531157399</v>
+      </c>
+      <c r="Q64" s="2" t="n">
+        <v>-0.0297106964134189</v>
+      </c>
+      <c r="R64" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S64" s="2" t="n">
+        <v>3.617114875589066</v>
+      </c>
+      <c r="T64" s="2" t="n">
+        <v>0.0025095802697039</v>
+      </c>
+      <c r="U64" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V64" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="W64" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="X64" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y64" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z64" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA64" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB64" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC64" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AD64" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE64" s="2" t="n">
+        <v>37.245</v>
+      </c>
+      <c r="AF64" s="2" t="n">
+        <v>0.315</v>
+      </c>
+      <c r="AG64" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AH64" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI64" s="2" t="n">
+        <v>37.245</v>
+      </c>
+      <c r="AJ64" s="2" t="n">
+        <v>0.315</v>
+      </c>
+      <c r="AK64" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AL64" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM64" s="2" t="n">
+        <v>37.245</v>
+      </c>
+      <c r="AN64" s="2" t="n">
+        <v>0.315</v>
+      </c>
+      <c r="AO64" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AP64" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ64" s="2" t="n">
+        <v>37.23</v>
+      </c>
+      <c r="AR64" s="2" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="AS64" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AT64" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU64" s="2" t="n">
+        <v>37.23</v>
+      </c>
+      <c r="AV64" s="2" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="AW64" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AX64" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY64" s="2" t="n">
+        <v>37.23</v>
+      </c>
+      <c r="AZ64" s="2" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="BA64" s="2" t="n">
+        <v>0.00107</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>11:07</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>GLXY</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="n">
+        <v>16.96</v>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21 11:06:00-04:00</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="n"/>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="n">
+        <v>-1.187</v>
+      </c>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="J65" s="2" t="inlineStr">
+        <is>
+          <t>ema_bounce</t>
+        </is>
+      </c>
+      <c r="K65" s="2" t="n">
+        <v>97</v>
+      </c>
+      <c r="L65" s="2" t="n">
+        <v>0.084390856877571</v>
+      </c>
+      <c r="M65" s="2" t="n">
+        <v>0.0431472268591475</v>
+      </c>
+      <c r="N65" s="2" t="n">
+        <v>1.108535437773315</v>
+      </c>
+      <c r="O65" s="2" t="n">
+        <v>0.0265209055041564</v>
+      </c>
+      <c r="P65" s="2" t="n">
+        <v>0.0076067964556573</v>
+      </c>
+      <c r="Q65" s="2" t="n">
+        <v>-0.0121386759383659</v>
+      </c>
+      <c r="R65" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S65" s="2" t="n">
+        <v>2.838493506055989</v>
+      </c>
+      <c r="T65" s="2" t="n">
+        <v>0.0026006111848979</v>
+      </c>
+      <c r="U65" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V65" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W65" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X65" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y65" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z65" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA65" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB65" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC65" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AD65" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AE65" s="2" t="n">
+        <v>17.09</v>
+      </c>
+      <c r="AF65" s="2" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="AG65" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AH65" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI65" s="2" t="n">
+        <v>17.09</v>
+      </c>
+      <c r="AJ65" s="2" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="AK65" s="2" t="n">
+        <v>0.6731</v>
+      </c>
+      <c r="AL65" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AM65" s="2" t="n">
+        <v>17.09</v>
+      </c>
+      <c r="AN65" s="2" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="AO65" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AP65" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AQ65" s="2" t="n">
+        <v>17.09</v>
+      </c>
+      <c r="AR65" s="2" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="AS65" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AT65" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU65" s="2" t="n">
+        <v>17.09</v>
+      </c>
+      <c r="AV65" s="2" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="AW65" s="2" t="n">
+        <v>0.6731</v>
+      </c>
+      <c r="AX65" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AY65" s="2" t="n">
+        <v>17.09</v>
+      </c>
+      <c r="AZ65" s="2" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="BA65" s="2" t="n">
+        <v>0.00117</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>11:08</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>APLD</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="n">
+        <v>20.54</v>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21 11:07:00-04:00</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="n"/>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="n">
+        <v>-1.133</v>
+      </c>
+      <c r="I66" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="J66" s="2" t="inlineStr">
+        <is>
+          <t>ema_bounce</t>
+        </is>
+      </c>
+      <c r="K66" s="2" t="n">
+        <v>98</v>
+      </c>
+      <c r="L66" s="2" t="n">
+        <v>0.072684981489443</v>
+      </c>
+      <c r="M66" s="2" t="n">
+        <v>0.0437143981732868</v>
+      </c>
+      <c r="N66" s="2" t="n">
+        <v>0.938732228796364</v>
+      </c>
+      <c r="O66" s="2" t="n">
+        <v>0.0186441061903501</v>
+      </c>
+      <c r="P66" s="2" t="n">
+        <v>0.009404417873718899</v>
+      </c>
+      <c r="Q66" s="2" t="n">
+        <v>-0.0031249340910153</v>
+      </c>
+      <c r="R66" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S66" s="2" t="n">
+        <v>3.031823123134156</v>
+      </c>
+      <c r="T66" s="2" t="n">
+        <v>0.0026916421000919</v>
+      </c>
+      <c r="U66" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V66" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W66" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X66" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y66" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z66" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA66" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB66" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC66" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AD66" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE66" s="2" t="n">
+        <v>20.735</v>
+      </c>
+      <c r="AF66" s="2" t="n">
+        <v>0.195</v>
+      </c>
+      <c r="AG66" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AH66" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI66" s="2" t="n">
+        <v>20.735</v>
+      </c>
+      <c r="AJ66" s="2" t="n">
+        <v>0.195</v>
+      </c>
+      <c r="AK66" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AL66" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM66" s="2" t="n">
+        <v>20.735</v>
+      </c>
+      <c r="AN66" s="2" t="n">
+        <v>0.195</v>
+      </c>
+      <c r="AO66" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AP66" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ66" s="2" t="n">
+        <v>20.735</v>
+      </c>
+      <c r="AR66" s="2" t="n">
+        <v>0.195</v>
+      </c>
+      <c r="AS66" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AT66" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU66" s="2" t="n">
+        <v>20.735</v>
+      </c>
+      <c r="AV66" s="2" t="n">
+        <v>0.195</v>
+      </c>
+      <c r="AW66" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AX66" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY66" s="2" t="n">
+        <v>20.735</v>
+      </c>
+      <c r="AZ66" s="2" t="n">
+        <v>0.195</v>
+      </c>
+      <c r="BA66" s="2" t="n">
+        <v>0.00048</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>11:08</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>WULF</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="n">
+        <v>12.64</v>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21 11:07:00-04:00</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="n"/>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="n">
+        <v>-1.333</v>
+      </c>
+      <c r="I67" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="J67" s="2" t="inlineStr">
+        <is>
+          <t>vwap_pullback</t>
+        </is>
+      </c>
+      <c r="K67" s="2" t="n">
+        <v>98</v>
+      </c>
+      <c r="L67" s="2" t="n">
+        <v>0.0553705203313672</v>
+      </c>
+      <c r="M67" s="2" t="n">
+        <v>0.0574520871967993</v>
+      </c>
+      <c r="N67" s="2" t="n">
+        <v>1.045453496421826</v>
+      </c>
+      <c r="O67" s="2" t="n">
+        <v>0.0037727243227259</v>
+      </c>
+      <c r="P67" s="2" t="n">
+        <v>0.0027613562294418</v>
+      </c>
+      <c r="Q67" s="2" t="n">
+        <v>-0.0174418166239485</v>
+      </c>
+      <c r="R67" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S67" s="2" t="n">
+        <v>2.539631564525362</v>
+      </c>
+      <c r="T67" s="2" t="n">
+        <v>0.0026916421000919</v>
+      </c>
+      <c r="U67" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V67" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W67" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X67" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y67" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z67" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA67" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB67" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC67" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AD67" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE67" s="2" t="n">
+        <v>12.68</v>
+      </c>
+      <c r="AF67" s="2" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="AG67" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AH67" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI67" s="2" t="n">
+        <v>12.68</v>
+      </c>
+      <c r="AJ67" s="2" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="AK67" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AL67" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM67" s="2" t="n">
+        <v>12.68</v>
+      </c>
+      <c r="AN67" s="2" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="AO67" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AP67" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ67" s="2" t="n">
+        <v>12.675</v>
+      </c>
+      <c r="AR67" s="2" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="AS67" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AT67" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU67" s="2" t="n">
+        <v>12.675</v>
+      </c>
+      <c r="AV67" s="2" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="AW67" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AX67" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY67" s="2" t="n">
+        <v>12.675</v>
+      </c>
+      <c r="AZ67" s="2" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="BA67" s="2" t="n">
+        <v>0.00079</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>11:11</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>APPN</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="n">
+        <v>47.82</v>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21 11:10:00-04:00</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="n"/>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I68" s="2" t="inlineStr">
+        <is>
+          <t>target</t>
+        </is>
+      </c>
+      <c r="J68" s="2" t="inlineStr">
+        <is>
+          <t>ema_bounce</t>
+        </is>
+      </c>
+      <c r="K68" s="2" t="n">
+        <v>101</v>
+      </c>
+      <c r="L68" s="2" t="n">
+        <v>0.08043140790959639</v>
+      </c>
+      <c r="M68" s="2" t="n">
+        <v>-0.0024712828533421</v>
+      </c>
+      <c r="N68" s="2" t="n">
+        <v>1.228273048924955</v>
+      </c>
+      <c r="O68" s="2" t="n">
+        <v>0.0223354420107861</v>
+      </c>
+      <c r="P68" s="2" t="n">
+        <v>0.0056144760185316</v>
+      </c>
+      <c r="Q68" s="2" t="n">
+        <v>-0.0074283211416306</v>
+      </c>
+      <c r="R68" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S68" s="2" t="n">
+        <v>3.873074258462536</v>
+      </c>
+      <c r="T68" s="2" t="n">
+        <v>0.0029777505998953</v>
+      </c>
+      <c r="U68" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V68" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W68" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X68" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y68" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z68" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA68" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB68" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC68" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AD68" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AE68" s="2" t="n">
+        <v>48.085</v>
+      </c>
+      <c r="AF68" s="2" t="n">
+        <v>0.265</v>
+      </c>
+      <c r="AG68" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="AH68" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI68" s="2" t="n">
+        <v>48.085</v>
+      </c>
+      <c r="AJ68" s="2" t="n">
+        <v>0.265</v>
+      </c>
+      <c r="AK68" s="2" t="n">
+        <v>0.5189</v>
+      </c>
+      <c r="AL68" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AM68" s="2" t="n">
+        <v>48.085</v>
+      </c>
+      <c r="AN68" s="2" t="n">
+        <v>0.265</v>
+      </c>
+      <c r="AO68" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AP68" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AQ68" s="2" t="n">
+        <v>48.085</v>
+      </c>
+      <c r="AR68" s="2" t="n">
+        <v>0.265</v>
+      </c>
+      <c r="AS68" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="AT68" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU68" s="2" t="n">
+        <v>48.085</v>
+      </c>
+      <c r="AV68" s="2" t="n">
+        <v>0.265</v>
+      </c>
+      <c r="AW68" s="2" t="n">
+        <v>0.5189</v>
+      </c>
+      <c r="AX68" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AY68" s="2" t="n">
+        <v>48.085</v>
+      </c>
+      <c r="AZ68" s="2" t="n">
+        <v>0.265</v>
+      </c>
+      <c r="BA68" s="2" t="n">
+        <v>0.00312</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>11:50</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>WFRD</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="n">
+        <v>83.61</v>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21 11:49:00-04:00</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="n"/>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I69" s="2" t="inlineStr">
+        <is>
+          <t>target</t>
+        </is>
+      </c>
+      <c r="J69" s="2" t="inlineStr">
+        <is>
+          <t>ema_bounce</t>
+        </is>
+      </c>
+      <c r="K69" s="2" t="n">
+        <v>140</v>
+      </c>
+      <c r="L69" s="2" t="n">
+        <v>0.0618856048492717</v>
+      </c>
+      <c r="M69" s="2" t="n">
+        <v>0.0470129005432313</v>
+      </c>
+      <c r="N69" s="2" t="n">
+        <v>1.108754458497237</v>
+      </c>
+      <c r="O69" s="2" t="n">
+        <v>0.0033566988206361</v>
+      </c>
+      <c r="P69" s="2" t="n">
+        <v>0.0075964391691394</v>
+      </c>
+      <c r="Q69" s="2" t="n">
+        <v>-0.0143316583327226</v>
+      </c>
+      <c r="R69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S69" s="2" t="n">
+        <v>4.433788569232471</v>
+      </c>
+      <c r="T69" s="2" t="n">
+        <v>0.0049151932343474</v>
+      </c>
+      <c r="U69" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V69" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="W69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB69" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC69" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AD69" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE69" s="2" t="n">
+        <v>84.31</v>
+      </c>
+      <c r="AF69" s="2" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AG69" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="AH69" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI69" s="2" t="n">
+        <v>84.31</v>
+      </c>
+      <c r="AJ69" s="2" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AK69" s="2" t="n">
+        <v>1.2357</v>
+      </c>
+      <c r="AL69" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AM69" s="2" t="n">
+        <v>84.31</v>
+      </c>
+      <c r="AN69" s="2" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AO69" s="2" t="n"/>
+      <c r="AP69" s="2" t="n"/>
+      <c r="AQ69" s="2" t="n"/>
+      <c r="AR69" s="2" t="n"/>
+      <c r="AS69" s="2" t="n"/>
+      <c r="AT69" s="2" t="n"/>
+      <c r="AU69" s="2" t="n"/>
+      <c r="AV69" s="2" t="n"/>
+      <c r="AW69" s="2" t="n"/>
+      <c r="AX69" s="2" t="n"/>
+      <c r="AY69" s="2" t="n"/>
+      <c r="AZ69" s="2" t="n"/>
+      <c r="BA69" s="2" t="n">
+        <v>0.00474</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>AHT</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="n">
+        <v>2.46</v>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21 12:14:00-04:00</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="n"/>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="n">
+        <v>-1.364</v>
+      </c>
+      <c r="I70" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="J70" s="2" t="inlineStr">
+        <is>
+          <t>vwap_pullback</t>
+        </is>
+      </c>
+      <c r="K70" s="2" t="n">
+        <v>165</v>
+      </c>
+      <c r="L70" s="2" t="n">
+        <v>0.3959777053316788</v>
+      </c>
+      <c r="M70" s="2" t="n">
+        <v>0.3351956177865058</v>
+      </c>
+      <c r="N70" s="2" t="n">
+        <v>7.863419779725414</v>
+      </c>
+      <c r="O70" s="2" t="n">
+        <v>0.0139315907860309</v>
+      </c>
+      <c r="P70" s="2" t="n">
+        <v>0.01552746865747</v>
+      </c>
+      <c r="Q70" s="2" t="n">
+        <v>-0.1107472988701674</v>
+      </c>
+      <c r="R70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S70" s="2" t="n">
+        <v>0.9158106323613781</v>
+      </c>
+      <c r="T70" s="2" t="n">
+        <v>0.0046031325904565</v>
+      </c>
+      <c r="U70" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC70" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AD70" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE70" s="2" t="n">
+        <v>2.495</v>
+      </c>
+      <c r="AF70" s="2" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="AG70" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AH70" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI70" s="2" t="n">
+        <v>2.495</v>
+      </c>
+      <c r="AJ70" s="2" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="AK70" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AL70" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM70" s="2" t="n">
+        <v>2.495</v>
+      </c>
+      <c r="AN70" s="2" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="AO70" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AP70" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ70" s="2" t="n">
+        <v>2.495</v>
+      </c>
+      <c r="AR70" s="2" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="AS70" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AT70" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU70" s="2" t="n">
+        <v>2.495</v>
+      </c>
+      <c r="AV70" s="2" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="AW70" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AX70" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY70" s="2" t="n">
+        <v>2.495</v>
+      </c>
+      <c r="AZ70" s="2" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="BA70" s="2" t="n">
+        <v>0.00401</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>WGO</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="n">
+        <v>24.88</v>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21 12:29:00-04:00</t>
+        </is>
+      </c>
+      <c r="F71" s="2" t="n"/>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="n">
+        <v>0.951</v>
+      </c>
+      <c r="I71" s="2" t="inlineStr">
+        <is>
+          <t>time</t>
+        </is>
+      </c>
+      <c r="J71" s="2" t="inlineStr">
+        <is>
+          <t>ema_bounce</t>
+        </is>
+      </c>
+      <c r="K71" s="2" t="n">
+        <v>180</v>
+      </c>
+      <c r="L71" s="2" t="n">
+        <v>0.0854553101301944</v>
+      </c>
+      <c r="M71" s="2" t="n">
+        <v>0.06905482849379641</v>
+      </c>
+      <c r="N71" s="2" t="n">
+        <v>1.455040430641148</v>
+      </c>
+      <c r="O71" s="2" t="n">
+        <v>0.0144071910290453</v>
+      </c>
+      <c r="P71" s="2" t="n">
+        <v>0.0107355714761658</v>
+      </c>
+      <c r="Q71" s="2" t="n">
+        <v>-0.0007946149266209</v>
+      </c>
+      <c r="R71" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S71" s="2" t="n">
+        <v>3.224857881377966</v>
+      </c>
+      <c r="T71" s="2" t="n">
+        <v>0.0041870252771503</v>
+      </c>
+      <c r="U71" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V71" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="W71" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X71" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y71" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z71" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA71" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB71" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC71" s="2" t="n">
+        <v>1.1328</v>
+      </c>
+      <c r="AD71" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AE71" s="2" t="n">
+        <v>25.2</v>
+      </c>
+      <c r="AF71" s="2" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="AG71" s="2" t="n">
+        <v>1.2656</v>
+      </c>
+      <c r="AH71" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI71" s="2" t="n">
+        <v>25.2</v>
+      </c>
+      <c r="AJ71" s="2" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="AK71" s="2" t="n">
+        <v>1.1328</v>
+      </c>
+      <c r="AL71" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AM71" s="2" t="n">
+        <v>25.2</v>
+      </c>
+      <c r="AN71" s="2" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="AO71" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AP71" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AQ71" s="2" t="n">
+        <v>25.14</v>
+      </c>
+      <c r="AR71" s="2" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="AS71" s="2" t="n">
+        <v>1.7885</v>
+      </c>
+      <c r="AT71" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU71" s="2" t="n">
+        <v>25.14</v>
+      </c>
+      <c r="AV71" s="2" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="AW71" s="2" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="AX71" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AY71" s="2" t="n">
+        <v>25.14</v>
+      </c>
+      <c r="AZ71" s="2" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="BA71" s="2" t="n">
+        <v>0.00317</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>12:36</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>APLD</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21 12:35:00-04:00</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="n"/>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I72" s="2" t="inlineStr">
+        <is>
+          <t>target</t>
+        </is>
+      </c>
+      <c r="J72" s="2" t="inlineStr">
+        <is>
+          <t>vwap_pullback</t>
+        </is>
+      </c>
+      <c r="K72" s="2" t="n">
+        <v>186</v>
+      </c>
+      <c r="L72" s="2" t="n">
+        <v>0.0623383304946763</v>
+      </c>
+      <c r="M72" s="2" t="n">
+        <v>0.0437143981732868</v>
+      </c>
+      <c r="N72" s="2" t="n">
+        <v>0.7666863290969826</v>
+      </c>
+      <c r="O72" s="2" t="n">
+        <v>0.0034848122242043</v>
+      </c>
+      <c r="P72" s="2" t="n">
+        <v>0.0017043996918519</v>
+      </c>
+      <c r="Q72" s="2" t="n">
+        <v>-0.0169937555102198</v>
+      </c>
+      <c r="R72" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S72" s="2" t="n">
+        <v>3.022130739977896</v>
+      </c>
+      <c r="T72" s="2" t="n">
+        <v>0.0041349622602651</v>
+      </c>
+      <c r="U72" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V72" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W72" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X72" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y72" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z72" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA72" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB72" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC72" s="2" t="n"/>
+      <c r="AD72" s="2" t="n"/>
+      <c r="AE72" s="2" t="n"/>
+      <c r="AF72" s="2" t="n"/>
+      <c r="AG72" s="2" t="n"/>
+      <c r="AH72" s="2" t="n"/>
+      <c r="AI72" s="2" t="n"/>
+      <c r="AJ72" s="2" t="n"/>
+      <c r="AK72" s="2" t="n"/>
+      <c r="AL72" s="2" t="n"/>
+      <c r="AM72" s="2" t="n"/>
+      <c r="AN72" s="2" t="n"/>
+      <c r="AO72" s="2" t="n"/>
+      <c r="AP72" s="2" t="n"/>
+      <c r="AQ72" s="2" t="n"/>
+      <c r="AR72" s="2" t="n"/>
+      <c r="AS72" s="2" t="n"/>
+      <c r="AT72" s="2" t="n"/>
+      <c r="AU72" s="2" t="n"/>
+      <c r="AV72" s="2" t="n"/>
+      <c r="AW72" s="2" t="n"/>
+      <c r="AX72" s="2" t="n"/>
+      <c r="AY72" s="2" t="n"/>
+      <c r="AZ72" s="2" t="n"/>
+      <c r="BA72" s="2" t="n">
+        <v>0.00049</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>APLD</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="n">
+        <v>20.73</v>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21 12:59:00-04:00</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="n"/>
+      <c r="G73" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H73" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I73" s="2" t="inlineStr">
+        <is>
+          <t>target</t>
+        </is>
+      </c>
+      <c r="J73" s="2" t="inlineStr">
+        <is>
+          <t>afternoon_hod</t>
+        </is>
+      </c>
+      <c r="K73" s="2" t="n">
+        <v>210</v>
+      </c>
+      <c r="L73" s="2" t="n">
+        <v>0.0845835610623408</v>
+      </c>
+      <c r="M73" s="2" t="n">
+        <v>0.0437143981732868</v>
+      </c>
+      <c r="N73" s="2" t="n">
+        <v>0.7475614000747192</v>
+      </c>
+      <c r="O73" s="2" t="n">
+        <v>0.0230579191886173</v>
+      </c>
+      <c r="P73" s="2" t="n">
+        <v>0.0112091653173149</v>
+      </c>
+      <c r="Q73" s="2" t="n">
+        <v>-0.0004767689487467</v>
+      </c>
+      <c r="R73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S73" s="2" t="n">
+        <v>3.042854387900946</v>
+      </c>
+      <c r="T73" s="2" t="n">
+        <v>0.0056953448440748</v>
+      </c>
+      <c r="U73" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X73" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC73" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AD73" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE73" s="2" t="n">
+        <v>20.965</v>
+      </c>
+      <c r="AF73" s="2" t="n">
+        <v>0.235</v>
+      </c>
+      <c r="AG73" s="2" t="n">
+        <v>-0.2128</v>
+      </c>
+      <c r="AH73" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI73" s="2" t="n">
+        <v>20.965</v>
+      </c>
+      <c r="AJ73" s="2" t="n">
+        <v>0.235</v>
+      </c>
+      <c r="AK73" s="2" t="n">
+        <v>0.8298</v>
+      </c>
+      <c r="AL73" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AM73" s="2" t="n">
+        <v>20.965</v>
+      </c>
+      <c r="AN73" s="2" t="n">
+        <v>0.235</v>
+      </c>
+      <c r="AO73" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AP73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ73" s="2" t="n">
+        <v>20.965</v>
+      </c>
+      <c r="AR73" s="2" t="n">
+        <v>0.235</v>
+      </c>
+      <c r="AS73" s="2" t="n">
+        <v>-0.2128</v>
+      </c>
+      <c r="AT73" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU73" s="2" t="n">
+        <v>20.965</v>
+      </c>
+      <c r="AV73" s="2" t="n">
+        <v>0.235</v>
+      </c>
+      <c r="AW73" s="2" t="n">
+        <v>0.8298</v>
+      </c>
+      <c r="AX73" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AY73" s="2" t="n">
+        <v>20.965</v>
+      </c>
+      <c r="AZ73" s="2" t="n">
+        <v>0.235</v>
+      </c>
+      <c r="BA73" s="2" t="n">
+        <v>0.00048</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>13:04</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>ECHO</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="n">
+        <v>92.7</v>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21 13:03:00-04:00</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="n"/>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H74" s="2" t="n">
+        <v>-1.25</v>
+      </c>
+      <c r="I74" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="J74" s="2" t="inlineStr">
+        <is>
+          <t>vwap_pullback</t>
+        </is>
+      </c>
+      <c r="K74" s="2" t="n">
+        <v>214</v>
+      </c>
+      <c r="L74" s="2" t="n">
+        <v>0.0779025744239096</v>
+      </c>
+      <c r="M74" s="2" t="n">
+        <v>0.0491955090870073</v>
+      </c>
+      <c r="N74" s="2" t="n">
+        <v>0.9461370068748308</v>
+      </c>
+      <c r="O74" s="2" t="n">
+        <v>0.005763189504971</v>
+      </c>
+      <c r="P74" s="2" t="n">
+        <v>0.0045103386403996</v>
+      </c>
+      <c r="Q74" s="2" t="n">
+        <v>-0.0091508893342481</v>
+      </c>
+      <c r="R74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S74" s="2" t="n">
+        <v>4.533889013478209</v>
+      </c>
+      <c r="T74" s="2" t="n">
+        <v>0.0057213763525174</v>
+      </c>
+      <c r="U74" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W74" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="X74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC74" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AD74" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE74" s="2" t="n">
+        <v>93.12</v>
+      </c>
+      <c r="AF74" s="2" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="AG74" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AH74" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI74" s="2" t="n">
+        <v>93.12</v>
+      </c>
+      <c r="AJ74" s="2" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="AK74" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AL74" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM74" s="2" t="n">
+        <v>93.12</v>
+      </c>
+      <c r="AN74" s="2" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="AO74" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AP74" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ74" s="2" t="n">
+        <v>93.12</v>
+      </c>
+      <c r="AR74" s="2" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="AS74" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AT74" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU74" s="2" t="n">
+        <v>93.12</v>
+      </c>
+      <c r="AV74" s="2" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="AW74" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AX74" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY74" s="2" t="n">
+        <v>93.12</v>
+      </c>
+      <c r="AZ74" s="2" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="BA74" s="2" t="n">
+        <v>0.00086</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>GLXY</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="n">
+        <v>17.24</v>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21 13:14:00-04:00</t>
+        </is>
+      </c>
+      <c r="F75" s="2" t="n"/>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H75" s="2" t="n">
+        <v>-1.167</v>
+      </c>
+      <c r="I75" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="J75" s="2" t="inlineStr">
+        <is>
+          <t>afternoon_hod</t>
+        </is>
+      </c>
+      <c r="K75" s="2" t="n">
+        <v>225</v>
+      </c>
+      <c r="L75" s="2" t="n">
+        <v>0.1027918089059383</v>
+      </c>
+      <c r="M75" s="2" t="n">
+        <v>0.0431472268591475</v>
+      </c>
+      <c r="N75" s="2" t="n">
+        <v>0.9883670990163382</v>
+      </c>
+      <c r="O75" s="2" t="n">
+        <v>0.0324595567687253</v>
+      </c>
+      <c r="P75" s="2" t="n">
+        <v>0.008055188004993399</v>
+      </c>
+      <c r="Q75" s="2" t="n">
+        <v>-0.0008623912964816</v>
+      </c>
+      <c r="R75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S75" s="2" t="n">
+        <v>2.855320071549938</v>
+      </c>
+      <c r="T75" s="2" t="n">
+        <v>0.0062414509708839</v>
+      </c>
+      <c r="U75" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC75" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AD75" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE75" s="2" t="n">
+        <v>17.39</v>
+      </c>
+      <c r="AF75" s="2" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="AG75" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AH75" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI75" s="2" t="n">
+        <v>17.39</v>
+      </c>
+      <c r="AJ75" s="2" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="AK75" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AL75" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM75" s="2" t="n">
+        <v>17.39</v>
+      </c>
+      <c r="AN75" s="2" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="AO75" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AP75" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ75" s="2" t="n">
+        <v>17.37</v>
+      </c>
+      <c r="AR75" s="2" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="AS75" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AT75" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU75" s="2" t="n">
+        <v>17.37</v>
+      </c>
+      <c r="AV75" s="2" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="AW75" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AX75" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY75" s="2" t="n">
+        <v>17.37</v>
+      </c>
+      <c r="AZ75" s="2" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="BA75" s="2" t="n">
+        <v>0.00173</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>13:56</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>WULF</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="n">
+        <v>12.88</v>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21 13:55:00-04:00</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="n"/>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H76" s="2" t="n">
+        <v>-1.16</v>
+      </c>
+      <c r="I76" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="J76" s="2" t="inlineStr">
+        <is>
+          <t>afternoon_hod</t>
+        </is>
+      </c>
+      <c r="K76" s="2" t="n">
+        <v>266</v>
+      </c>
+      <c r="L76" s="2" t="n">
+        <v>0.0811822988521446</v>
+      </c>
+      <c r="M76" s="2" t="n">
+        <v>0.0574520871967993</v>
+      </c>
+      <c r="N76" s="2" t="n">
+        <v>0.777384282148076</v>
+      </c>
+      <c r="O76" s="2" t="n">
+        <v>0.0238100863698085</v>
+      </c>
+      <c r="P76" s="2" t="n">
+        <v>0.008086227143121299</v>
+      </c>
+      <c r="Q76" s="2" t="n">
+        <v>-0.0003849202870684</v>
+      </c>
+      <c r="R76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S76" s="2" t="n">
+        <v>2.563794818674761</v>
+      </c>
+      <c r="T76" s="2" t="n">
+        <v>0.0064755758181571</v>
+      </c>
+      <c r="U76" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC76" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AD76" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE76" s="2" t="n">
+        <v>12.985</v>
+      </c>
+      <c r="AF76" s="2" t="n">
+        <v>0.105</v>
+      </c>
+      <c r="AG76" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AH76" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI76" s="2" t="n">
+        <v>12.985</v>
+      </c>
+      <c r="AJ76" s="2" t="n">
+        <v>0.105</v>
+      </c>
+      <c r="AK76" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AL76" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM76" s="2" t="n">
+        <v>12.985</v>
+      </c>
+      <c r="AN76" s="2" t="n">
+        <v>0.105</v>
+      </c>
+      <c r="AO76" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AP76" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ76" s="2" t="n">
+        <v>12.985</v>
+      </c>
+      <c r="AR76" s="2" t="n">
+        <v>0.105</v>
+      </c>
+      <c r="AS76" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AT76" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU76" s="2" t="n">
+        <v>12.985</v>
+      </c>
+      <c r="AV76" s="2" t="n">
+        <v>0.105</v>
+      </c>
+      <c r="AW76" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AX76" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY76" s="2" t="n">
+        <v>12.985</v>
+      </c>
+      <c r="AZ76" s="2" t="n">
+        <v>0.105</v>
+      </c>
+      <c r="BA76" s="2" t="n">
+        <v>0.00077</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>14:28</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>APPN</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="n">
+        <v>48.56</v>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21 14:27:00-04:00</t>
+        </is>
+      </c>
+      <c r="F77" s="2" t="n"/>
+      <c r="G77" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H77" s="2" t="n">
+        <v>0.344</v>
+      </c>
+      <c r="I77" s="2" t="inlineStr">
+        <is>
+          <t>time</t>
+        </is>
+      </c>
+      <c r="J77" s="2" t="inlineStr">
+        <is>
+          <t>afternoon_hod</t>
+        </is>
+      </c>
+      <c r="K77" s="2" t="n">
+        <v>298</v>
+      </c>
+      <c r="L77" s="2" t="n">
+        <v>0.1006516181953267</v>
+      </c>
+      <c r="M77" s="2" t="n">
+        <v>-0.0024712828533421</v>
+      </c>
+      <c r="N77" s="2" t="n">
+        <v>0.9943872786280572</v>
+      </c>
+      <c r="O77" s="2" t="n">
+        <v>0.0264639110825528</v>
+      </c>
+      <c r="P77" s="2" t="n">
+        <v>0.0087773354507925</v>
+      </c>
+      <c r="Q77" s="2" t="n">
+        <v>-0.0042682740084597</v>
+      </c>
+      <c r="R77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S77" s="2" t="n">
+        <v>3.891616229911899</v>
+      </c>
+      <c r="T77" s="2" t="n">
+        <v>0.0069045401569747</v>
+      </c>
+      <c r="U77" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC77" s="2" t="n">
+        <v>0.7595</v>
+      </c>
+      <c r="AD77" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE77" s="2" t="n">
+        <v>48.955</v>
+      </c>
+      <c r="AF77" s="2" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="AG77" s="2" t="n">
+        <v>0.7595</v>
+      </c>
+      <c r="AH77" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI77" s="2" t="n">
+        <v>48.955</v>
+      </c>
+      <c r="AJ77" s="2" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="AK77" s="2" t="n">
+        <v>0.7595</v>
+      </c>
+      <c r="AL77" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM77" s="2" t="n">
+        <v>48.955</v>
+      </c>
+      <c r="AN77" s="2" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="AO77" s="2" t="n">
+        <v>0.7595</v>
+      </c>
+      <c r="AP77" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ77" s="2" t="n">
+        <v>48.955</v>
+      </c>
+      <c r="AR77" s="2" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="AS77" s="2" t="n">
+        <v>0.7595</v>
+      </c>
+      <c r="AT77" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU77" s="2" t="n">
+        <v>48.955</v>
+      </c>
+      <c r="AV77" s="2" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="AW77" s="2" t="n">
+        <v>0.7595</v>
+      </c>
+      <c r="AX77" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY77" s="2" t="n">
+        <v>48.955</v>
+      </c>
+      <c r="AZ77" s="2" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="BA77" s="2" t="n">
+        <v>0.00184</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>15:09</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>WGO</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="n">
+        <v>24.89</v>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21 15:08:00-04:00</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="n"/>
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H78" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I78" s="2" t="inlineStr">
+        <is>
+          <t>target</t>
+        </is>
+      </c>
+      <c r="J78" s="2" t="inlineStr">
+        <is>
+          <t>vwap_pullback</t>
+        </is>
+      </c>
+      <c r="K78" s="2" t="n">
+        <v>339</v>
+      </c>
+      <c r="L78" s="2" t="n">
+        <v>0.0811393679143788</v>
+      </c>
+      <c r="M78" s="2" t="n">
+        <v>0.06905482849379641</v>
+      </c>
+      <c r="N78" s="2" t="n">
+        <v>1.254994889364698</v>
+      </c>
+      <c r="O78" s="2" t="n">
+        <v>0.0050503391567211</v>
+      </c>
+      <c r="P78" s="2" t="n">
+        <v>0.00638719528677</v>
+      </c>
+      <c r="Q78" s="2" t="n">
+        <v>-0.0172616923502748</v>
+      </c>
+      <c r="R78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S78" s="2" t="n">
+        <v>3.220873797074209</v>
+      </c>
+      <c r="T78" s="2" t="n">
+        <v>0.0030297342524254</v>
+      </c>
+      <c r="U78" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V78" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="W78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC78" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AD78" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE78" s="2" t="n">
+        <v>24.99</v>
+      </c>
+      <c r="AF78" s="2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AG78" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="AH78" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI78" s="2" t="n">
+        <v>24.99</v>
+      </c>
+      <c r="AJ78" s="2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AK78" s="2" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="AL78" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AM78" s="2" t="n">
+        <v>24.99</v>
+      </c>
+      <c r="AN78" s="2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AO78" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AP78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ78" s="2" t="n">
+        <v>24.99</v>
+      </c>
+      <c r="AR78" s="2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AS78" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="AT78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU78" s="2" t="n">
+        <v>24.99</v>
+      </c>
+      <c r="AV78" s="2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AW78" s="2" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="AX78" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AY78" s="2" t="n">
+        <v>24.99</v>
+      </c>
+      <c r="AZ78" s="2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="BA78" s="2" t="n">
+        <v>0.0032</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>15:12</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>GLXY</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="n">
+        <v>16.99</v>
+      </c>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21 15:11:00-04:00</t>
+        </is>
+      </c>
+      <c r="F79" s="2" t="n"/>
+      <c r="G79" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H79" s="2" t="n">
+        <v>-1.333</v>
+      </c>
+      <c r="I79" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="J79" s="2" t="inlineStr">
+        <is>
+          <t>vwap_pullback</t>
+        </is>
+      </c>
+      <c r="K79" s="2" t="n">
+        <v>342</v>
+      </c>
+      <c r="L79" s="2" t="n">
+        <v>0.0818527277566059</v>
+      </c>
+      <c r="M79" s="2" t="n">
+        <v>0.0431472268591475</v>
+      </c>
+      <c r="N79" s="2" t="n">
+        <v>0.9393046002706378</v>
+      </c>
+      <c r="O79" s="2" t="n">
+        <v>0.0055503568021033</v>
+      </c>
+      <c r="P79" s="2" t="n">
+        <v>0.0035190169938618</v>
+      </c>
+      <c r="Q79" s="2" t="n">
+        <v>-0.0226426176367813</v>
+      </c>
+      <c r="R79" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S79" s="2" t="n">
+        <v>2.836150158982343</v>
+      </c>
+      <c r="T79" s="2" t="n">
+        <v>0.0027702921759047</v>
+      </c>
+      <c r="U79" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V79" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W79" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X79" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y79" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z79" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA79" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB79" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC79" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AD79" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AE79" s="2" t="n">
+        <v>17.05</v>
+      </c>
+      <c r="AF79" s="2" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="AG79" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AH79" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI79" s="2" t="n">
+        <v>17.05</v>
+      </c>
+      <c r="AJ79" s="2" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="AK79" s="2" t="n">
+        <v>0.7917</v>
+      </c>
+      <c r="AL79" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AM79" s="2" t="n">
+        <v>17.05</v>
+      </c>
+      <c r="AN79" s="2" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="AO79" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AP79" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AQ79" s="2" t="n">
+        <v>17.05</v>
+      </c>
+      <c r="AR79" s="2" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="AS79" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AT79" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU79" s="2" t="n">
+        <v>17.05</v>
+      </c>
+      <c r="AV79" s="2" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="AW79" s="2" t="n">
+        <v>0.7917</v>
+      </c>
+      <c r="AX79" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AY79" s="2" t="n">
+        <v>17.05</v>
+      </c>
+      <c r="AZ79" s="2" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="BA79" s="2" t="n">
+        <v>0.00117</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>APPN</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="n">
+        <v>48.6</v>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21 15:29:00-04:00</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="n"/>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H80" s="2" t="n"/>
+      <c r="I80" s="2" t="n"/>
+      <c r="J80" s="2" t="inlineStr">
+        <is>
+          <t>eod_squeeze</t>
+        </is>
+      </c>
+      <c r="K80" s="2" t="n">
+        <v>360</v>
+      </c>
+      <c r="L80" s="2" t="n">
+        <v>0.099977554049617</v>
+      </c>
+      <c r="M80" s="2" t="n">
+        <v>-0.0024712828533421</v>
+      </c>
+      <c r="N80" s="2" t="n">
+        <v>0.9707696671333648</v>
+      </c>
+      <c r="O80" s="2" t="n">
+        <v>0.0220802581012165</v>
+      </c>
+      <c r="P80" s="2" t="n">
+        <v>0.0073529226144701</v>
+      </c>
+      <c r="Q80" s="2" t="n">
+        <v>-0.0058883434624841</v>
+      </c>
+      <c r="R80" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S80" s="2" t="n">
+        <v>3.891003619504574</v>
+      </c>
+      <c r="T80" s="2" t="n">
+        <v>0.0054417757298246</v>
+      </c>
+      <c r="U80" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V80" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W80" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X80" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y80" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z80" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA80" s="2" t="n"/>
+      <c r="AB80" s="2" t="n"/>
+      <c r="AC80" s="2" t="n"/>
+      <c r="AD80" s="2" t="n"/>
+      <c r="AE80" s="2" t="n"/>
+      <c r="AF80" s="2" t="n"/>
+      <c r="AG80" s="2" t="n"/>
+      <c r="AH80" s="2" t="n"/>
+      <c r="AI80" s="2" t="n"/>
+      <c r="AJ80" s="2" t="n"/>
+      <c r="AK80" s="2" t="n"/>
+      <c r="AL80" s="2" t="n"/>
+      <c r="AM80" s="2" t="n"/>
+      <c r="AN80" s="2" t="n"/>
+      <c r="AO80" s="2" t="n"/>
+      <c r="AP80" s="2" t="n"/>
+      <c r="AQ80" s="2" t="n"/>
+      <c r="AR80" s="2" t="n"/>
+      <c r="AS80" s="2" t="n"/>
+      <c r="AT80" s="2" t="n"/>
+      <c r="AU80" s="2" t="n"/>
+      <c r="AV80" s="2" t="n"/>
+      <c r="AW80" s="2" t="n"/>
+      <c r="AX80" s="2" t="n"/>
+      <c r="AY80" s="2" t="n"/>
+      <c r="AZ80" s="2" t="n"/>
+      <c r="BA80" s="2" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>WGO</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="n">
+        <v>24.88</v>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21 15:29:00-04:00</t>
+        </is>
+      </c>
+      <c r="F81" s="2" t="n"/>
+      <c r="G81" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H81" s="2" t="n"/>
+      <c r="I81" s="2" t="n"/>
+      <c r="J81" s="2" t="inlineStr">
+        <is>
+          <t>eod_squeeze</t>
+        </is>
+      </c>
+      <c r="K81" s="2" t="n">
+        <v>360</v>
+      </c>
+      <c r="L81" s="2" t="n">
+        <v>0.0927923872011555</v>
+      </c>
+      <c r="M81" s="2" t="n">
+        <v>0.06905482849379641</v>
+      </c>
+      <c r="N81" s="2" t="n">
+        <v>1.256409448164708</v>
+      </c>
+      <c r="O81" s="2" t="n">
+        <v>0.0154591800975607</v>
+      </c>
+      <c r="P81" s="2" t="n">
+        <v>0.0173775552972918</v>
+      </c>
+      <c r="Q81" s="2" t="n">
+        <v>-0.0066692851243791</v>
+      </c>
+      <c r="R81" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S81" s="2" t="n">
+        <v>3.23159458522322</v>
+      </c>
+      <c r="T81" s="2" t="n">
+        <v>0.0054417757298246</v>
+      </c>
+      <c r="U81" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V81" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="W81" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X81" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y81" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z81" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA81" s="2" t="n"/>
+      <c r="AB81" s="2" t="n"/>
+      <c r="AC81" s="2" t="n"/>
+      <c r="AD81" s="2" t="n"/>
+      <c r="AE81" s="2" t="n"/>
+      <c r="AF81" s="2" t="n"/>
+      <c r="AG81" s="2" t="n"/>
+      <c r="AH81" s="2" t="n"/>
+      <c r="AI81" s="2" t="n"/>
+      <c r="AJ81" s="2" t="n"/>
+      <c r="AK81" s="2" t="n"/>
+      <c r="AL81" s="2" t="n"/>
+      <c r="AM81" s="2" t="n"/>
+      <c r="AN81" s="2" t="n"/>
+      <c r="AO81" s="2" t="n"/>
+      <c r="AP81" s="2" t="n"/>
+      <c r="AQ81" s="2" t="n"/>
+      <c r="AR81" s="2" t="n"/>
+      <c r="AS81" s="2" t="n"/>
+      <c r="AT81" s="2" t="n"/>
+      <c r="AU81" s="2" t="n"/>
+      <c r="AV81" s="2" t="n"/>
+      <c r="AW81" s="2" t="n"/>
+      <c r="AX81" s="2" t="n"/>
+      <c r="AY81" s="2" t="n"/>
+      <c r="AZ81" s="2" t="n"/>
+      <c r="BA81" s="2" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>WULF</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="n">
+        <v>12.75</v>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21 15:29:00-04:00</t>
+        </is>
+      </c>
+      <c r="F82" s="2" t="n"/>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H82" s="2" t="n"/>
+      <c r="I82" s="2" t="n"/>
+      <c r="J82" s="2" t="inlineStr">
+        <is>
+          <t>eod_squeeze</t>
+        </is>
+      </c>
+      <c r="K82" s="2" t="n">
+        <v>360</v>
+      </c>
+      <c r="L82" s="2" t="n">
+        <v>0.0761865066124329</v>
+      </c>
+      <c r="M82" s="2" t="n">
+        <v>0.0574520871967993</v>
+      </c>
+      <c r="N82" s="2" t="n">
+        <v>0.7602620672487318</v>
+      </c>
+      <c r="O82" s="2" t="n">
+        <v>0.0144347739743151</v>
+      </c>
+      <c r="P82" s="2" t="n">
+        <v>0.013539666394768</v>
+      </c>
+      <c r="Q82" s="2" t="n">
+        <v>-0.0099578790809662</v>
+      </c>
+      <c r="R82" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S82" s="2" t="n">
+        <v>2.559163435151542</v>
+      </c>
+      <c r="T82" s="2" t="n">
+        <v>0.0054417757298246</v>
+      </c>
+      <c r="U82" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V82" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W82" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X82" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y82" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z82" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA82" s="2" t="n"/>
+      <c r="AB82" s="2" t="n"/>
+      <c r="AC82" s="2" t="n"/>
+      <c r="AD82" s="2" t="n"/>
+      <c r="AE82" s="2" t="n"/>
+      <c r="AF82" s="2" t="n"/>
+      <c r="AG82" s="2" t="n"/>
+      <c r="AH82" s="2" t="n"/>
+      <c r="AI82" s="2" t="n"/>
+      <c r="AJ82" s="2" t="n"/>
+      <c r="AK82" s="2" t="n"/>
+      <c r="AL82" s="2" t="n"/>
+      <c r="AM82" s="2" t="n"/>
+      <c r="AN82" s="2" t="n"/>
+      <c r="AO82" s="2" t="n"/>
+      <c r="AP82" s="2" t="n"/>
+      <c r="AQ82" s="2" t="n"/>
+      <c r="AR82" s="2" t="n"/>
+      <c r="AS82" s="2" t="n"/>
+      <c r="AT82" s="2" t="n"/>
+      <c r="AU82" s="2" t="n"/>
+      <c r="AV82" s="2" t="n"/>
+      <c r="AW82" s="2" t="n"/>
+      <c r="AX82" s="2" t="n"/>
+      <c r="AY82" s="2" t="n"/>
+      <c r="AZ82" s="2" t="n"/>
+      <c r="BA82" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -11922,7 +16259,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:J27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12786,6 +17123,206 @@
         <v>-3.12</v>
       </c>
       <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="n">
+        <v>350</v>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>eod_squeeze</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>TLK</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="F23" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="H23" s="2" t="n">
+        <v>11.64</v>
+      </c>
+      <c r="I23" s="2" t="n">
+        <v>4.64</v>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>vwap_pullback</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>WULF</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="n">
+        <v>-1.2</v>
+      </c>
+      <c r="F24" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H24" s="2" t="n">
+        <v>12.69</v>
+      </c>
+      <c r="I24" s="2" t="n">
+        <v>-0.75</v>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>250</v>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>ema_bounce</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>AHT</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>3.76</v>
+      </c>
+      <c r="F25" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="G25" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="H25" s="2" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="I25" s="2" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>ema_bounce</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>AHT</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F26" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="H26" s="2" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="I26" s="2" t="n">
+        <v>3.73</v>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="n">
+        <v>550</v>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>afternoon_hod</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>APLD</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="F27" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="G27" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H27" s="2" t="n">
+        <v>20.945</v>
+      </c>
+      <c r="I27" s="2" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
         <is>
           <t>closed</t>
         </is>

</xml_diff>

<commit_message>
bot session end 2026-10-26 16:02
</commit_message>
<xml_diff>
--- a/reports/Paper Bot Live.xlsx
+++ b/reports/Paper Bot Live.xlsx
@@ -864,7 +864,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q39"/>
+  <dimension ref="A1:Q44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3269,6 +3269,311 @@
       <c r="Q39" s="2" t="inlineStr">
         <is>
           <t>15-min ORB: closed above 15-min high 13.18, above VWAP | news: [Newswire] Hesai Group to Report Third Quarter 2026 Financia</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="n">
+        <v>350</v>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>bull_flag</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>EAF</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="F40" s="2" t="n">
+        <v>10.29</v>
+      </c>
+      <c r="G40" s="2" t="n">
+        <v>10.05</v>
+      </c>
+      <c r="H40" s="2" t="n">
+        <v>10.53</v>
+      </c>
+      <c r="I40" s="2" t="n">
+        <v>10.77</v>
+      </c>
+      <c r="J40" s="2" t="n">
+        <v>10.02</v>
+      </c>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="L40" s="2" t="n">
+        <v>-3.78</v>
+      </c>
+      <c r="M40" s="2" t="n">
+        <v>-1.08</v>
+      </c>
+      <c r="N40" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O40" s="2" t="n"/>
+      <c r="P40" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q40" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bull flag: 3.2% pole, 1.0% flag on light vol, broke 10.16 | news: [Google News] Where GrafTech International Goes After A 50% </t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>orb15</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>CORT</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="F41" s="2" t="n">
+        <v>91.56999999999999</v>
+      </c>
+      <c r="G41" s="2" t="n">
+        <v>88.56</v>
+      </c>
+      <c r="H41" s="2" t="n">
+        <v>94.58</v>
+      </c>
+      <c r="I41" s="2" t="n">
+        <v>97.59</v>
+      </c>
+      <c r="J41" s="2" t="n">
+        <v>88.43000000000001</v>
+      </c>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="L41" s="2" t="n">
+        <v>-9.42</v>
+      </c>
+      <c r="M41" s="2" t="n">
+        <v>-0.9399999999999999</v>
+      </c>
+      <c r="N41" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O41" s="2" t="n"/>
+      <c r="P41" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q41" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15-min ORB: closed above 15-min high 91.12, above VWAP | news: [Benzinga] Corcept Therapeutics Announces Results From Part </t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="n">
+        <v>250</v>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>orb15</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>MLCO</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="F42" s="2" t="n">
+        <v>3.98</v>
+      </c>
+      <c r="G42" s="2" t="n">
+        <v>3.84</v>
+      </c>
+      <c r="H42" s="2" t="n">
+        <v>4.12</v>
+      </c>
+      <c r="I42" s="2" t="n">
+        <v>4.26</v>
+      </c>
+      <c r="J42" s="2" t="n">
+        <v>3.86</v>
+      </c>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>time</t>
+        </is>
+      </c>
+      <c r="L42" s="2" t="n">
+        <v>-2.04</v>
+      </c>
+      <c r="M42" s="2" t="n">
+        <v>-0.82</v>
+      </c>
+      <c r="N42" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O42" s="2" t="n"/>
+      <c r="P42" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q42" s="2" t="inlineStr">
+        <is>
+          <t>15-min ORB: closed above 15-min high 3.94, above VWAP | news: [Google News] EPrivateClient - Jersey makes changes to relia</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>orb5</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>BWMX</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F43" s="2" t="n">
+        <v>17.04</v>
+      </c>
+      <c r="G43" s="2" t="n">
+        <v>16.43</v>
+      </c>
+      <c r="H43" s="2" t="n">
+        <v>17.65</v>
+      </c>
+      <c r="I43" s="2" t="n">
+        <v>18.26</v>
+      </c>
+      <c r="J43" s="2" t="n">
+        <v>16.63</v>
+      </c>
+      <c r="K43" s="2" t="inlineStr">
+        <is>
+          <t>time</t>
+        </is>
+      </c>
+      <c r="L43" s="2" t="n">
+        <v>-2.46</v>
+      </c>
+      <c r="M43" s="2" t="n">
+        <v>-0.61</v>
+      </c>
+      <c r="N43" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O43" s="2" t="n"/>
+      <c r="P43" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q43" s="2" t="inlineStr">
+        <is>
+          <t>5-min ORB: green first 5 min, closed above range high 16.90 | news: [Google News] Betterware de México, S.A.P.I. de C.V. Just Mi</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="n">
+        <v>550</v>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>pm_high_break</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>RRC</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="F44" s="2" t="n">
+        <v>53.02</v>
+      </c>
+      <c r="G44" s="2" t="n">
+        <v>51.63</v>
+      </c>
+      <c r="H44" s="2" t="n">
+        <v>54.41</v>
+      </c>
+      <c r="I44" s="2" t="n">
+        <v>55.8</v>
+      </c>
+      <c r="J44" s="2" t="n">
+        <v>53.3</v>
+      </c>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
+          <t>time</t>
+        </is>
+      </c>
+      <c r="L44" s="2" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="M44" s="2" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="N44" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O44" s="2" t="n"/>
+      <c r="P44" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q44" s="2" t="inlineStr">
+        <is>
+          <t>Premarket-high break: closed above PM high 52.78, above VWAP | news: [Benzinga] EQT, Range Resources Mega-Merger Set to Create US</t>
         </is>
       </c>
     </row>
@@ -3283,7 +3588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BA171"/>
+  <dimension ref="A1:BA193"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31101,8 +31406,14 @@
           <t>off</t>
         </is>
       </c>
-      <c r="H166" s="2" t="n"/>
-      <c r="I166" s="2" t="n"/>
+      <c r="H166" s="2" t="n">
+        <v>-1.364</v>
+      </c>
+      <c r="I166" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
       <c r="J166" s="2" t="inlineStr">
         <is>
           <t>eod_squeeze</t>
@@ -31156,33 +31467,87 @@
       <c r="Z166" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA166" s="2" t="n"/>
-      <c r="AB166" s="2" t="n"/>
-      <c r="AC166" s="2" t="n"/>
-      <c r="AD166" s="2" t="n"/>
-      <c r="AE166" s="2" t="n"/>
-      <c r="AF166" s="2" t="n"/>
-      <c r="AG166" s="2" t="n"/>
-      <c r="AH166" s="2" t="n"/>
-      <c r="AI166" s="2" t="n"/>
-      <c r="AJ166" s="2" t="n"/>
-      <c r="AK166" s="2" t="n"/>
-      <c r="AL166" s="2" t="n"/>
-      <c r="AM166" s="2" t="n"/>
-      <c r="AN166" s="2" t="n"/>
-      <c r="AO166" s="2" t="n"/>
-      <c r="AP166" s="2" t="n"/>
-      <c r="AQ166" s="2" t="n"/>
-      <c r="AR166" s="2" t="n"/>
-      <c r="AS166" s="2" t="n"/>
-      <c r="AT166" s="2" t="n"/>
-      <c r="AU166" s="2" t="n"/>
-      <c r="AV166" s="2" t="n"/>
-      <c r="AW166" s="2" t="n"/>
-      <c r="AX166" s="2" t="n"/>
-      <c r="AY166" s="2" t="n"/>
-      <c r="AZ166" s="2" t="n"/>
-      <c r="BA166" s="2" t="n"/>
+      <c r="AA166" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB166" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC166" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AD166" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE166" s="2" t="n">
+        <v>79.84</v>
+      </c>
+      <c r="AF166" s="2" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="AG166" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AH166" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI166" s="2" t="n">
+        <v>79.84</v>
+      </c>
+      <c r="AJ166" s="2" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="AK166" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AL166" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM166" s="2" t="n">
+        <v>79.84</v>
+      </c>
+      <c r="AN166" s="2" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="AO166" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AP166" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ166" s="2" t="n">
+        <v>79.815</v>
+      </c>
+      <c r="AR166" s="2" t="n">
+        <v>0.185</v>
+      </c>
+      <c r="AS166" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AT166" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU166" s="2" t="n">
+        <v>79.815</v>
+      </c>
+      <c r="AV166" s="2" t="n">
+        <v>0.185</v>
+      </c>
+      <c r="AW166" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AX166" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY166" s="2" t="n">
+        <v>79.815</v>
+      </c>
+      <c r="AZ166" s="2" t="n">
+        <v>0.185</v>
+      </c>
+      <c r="BA166" s="2" t="n">
+        <v>0.00063</v>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
@@ -31214,8 +31579,14 @@
           <t>off</t>
         </is>
       </c>
-      <c r="H167" s="2" t="n"/>
-      <c r="I167" s="2" t="n"/>
+      <c r="H167" s="2" t="n">
+        <v>-0.138</v>
+      </c>
+      <c r="I167" s="2" t="inlineStr">
+        <is>
+          <t>next open</t>
+        </is>
+      </c>
       <c r="J167" s="2" t="inlineStr">
         <is>
           <t>eod_squeeze</t>
@@ -31269,33 +31640,87 @@
       <c r="Z167" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA167" s="2" t="n"/>
-      <c r="AB167" s="2" t="n"/>
-      <c r="AC167" s="2" t="n"/>
-      <c r="AD167" s="2" t="n"/>
-      <c r="AE167" s="2" t="n"/>
-      <c r="AF167" s="2" t="n"/>
-      <c r="AG167" s="2" t="n"/>
-      <c r="AH167" s="2" t="n"/>
-      <c r="AI167" s="2" t="n"/>
-      <c r="AJ167" s="2" t="n"/>
-      <c r="AK167" s="2" t="n"/>
-      <c r="AL167" s="2" t="n"/>
-      <c r="AM167" s="2" t="n"/>
-      <c r="AN167" s="2" t="n"/>
-      <c r="AO167" s="2" t="n"/>
-      <c r="AP167" s="2" t="n"/>
-      <c r="AQ167" s="2" t="n"/>
-      <c r="AR167" s="2" t="n"/>
-      <c r="AS167" s="2" t="n"/>
-      <c r="AT167" s="2" t="n"/>
-      <c r="AU167" s="2" t="n"/>
-      <c r="AV167" s="2" t="n"/>
-      <c r="AW167" s="2" t="n"/>
-      <c r="AX167" s="2" t="n"/>
-      <c r="AY167" s="2" t="n"/>
-      <c r="AZ167" s="2" t="n"/>
-      <c r="BA167" s="2" t="n"/>
+      <c r="AA167" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB167" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC167" s="2" t="n">
+        <v>0.8444</v>
+      </c>
+      <c r="AD167" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AE167" s="2" t="n">
+        <v>1.395</v>
+      </c>
+      <c r="AF167" s="2" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="AG167" s="2" t="n">
+        <v>0.6889</v>
+      </c>
+      <c r="AH167" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI167" s="2" t="n">
+        <v>1.395</v>
+      </c>
+      <c r="AJ167" s="2" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="AK167" s="2" t="n">
+        <v>0.8444</v>
+      </c>
+      <c r="AL167" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AM167" s="2" t="n">
+        <v>1.395</v>
+      </c>
+      <c r="AN167" s="2" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="AO167" s="2" t="n">
+        <v>0.8444</v>
+      </c>
+      <c r="AP167" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AQ167" s="2" t="n">
+        <v>1.395</v>
+      </c>
+      <c r="AR167" s="2" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="AS167" s="2" t="n">
+        <v>0.6889</v>
+      </c>
+      <c r="AT167" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU167" s="2" t="n">
+        <v>1.395</v>
+      </c>
+      <c r="AV167" s="2" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="AW167" s="2" t="n">
+        <v>0.8444</v>
+      </c>
+      <c r="AX167" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AY167" s="2" t="n">
+        <v>1.395</v>
+      </c>
+      <c r="AZ167" s="2" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="BA167" s="2" t="n">
+        <v>0.00717</v>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
@@ -31327,8 +31752,14 @@
           <t>off</t>
         </is>
       </c>
-      <c r="H168" s="2" t="n"/>
-      <c r="I168" s="2" t="n"/>
+      <c r="H168" s="2" t="n">
+        <v>-2.024</v>
+      </c>
+      <c r="I168" s="2" t="inlineStr">
+        <is>
+          <t>next open</t>
+        </is>
+      </c>
       <c r="J168" s="2" t="inlineStr">
         <is>
           <t>eod_squeeze</t>
@@ -31382,33 +31813,87 @@
       <c r="Z168" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA168" s="2" t="n"/>
-      <c r="AB168" s="2" t="n"/>
-      <c r="AC168" s="2" t="n"/>
-      <c r="AD168" s="2" t="n"/>
-      <c r="AE168" s="2" t="n"/>
-      <c r="AF168" s="2" t="n"/>
-      <c r="AG168" s="2" t="n"/>
-      <c r="AH168" s="2" t="n"/>
-      <c r="AI168" s="2" t="n"/>
-      <c r="AJ168" s="2" t="n"/>
-      <c r="AK168" s="2" t="n"/>
-      <c r="AL168" s="2" t="n"/>
-      <c r="AM168" s="2" t="n"/>
-      <c r="AN168" s="2" t="n"/>
-      <c r="AO168" s="2" t="n"/>
-      <c r="AP168" s="2" t="n"/>
-      <c r="AQ168" s="2" t="n"/>
-      <c r="AR168" s="2" t="n"/>
-      <c r="AS168" s="2" t="n"/>
-      <c r="AT168" s="2" t="n"/>
-      <c r="AU168" s="2" t="n"/>
-      <c r="AV168" s="2" t="n"/>
-      <c r="AW168" s="2" t="n"/>
-      <c r="AX168" s="2" t="n"/>
-      <c r="AY168" s="2" t="n"/>
-      <c r="AZ168" s="2" t="n"/>
-      <c r="BA168" s="2" t="n"/>
+      <c r="AA168" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB168" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC168" s="2" t="n">
+        <v>-2.0286</v>
+      </c>
+      <c r="AD168" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE168" s="2" t="n">
+        <v>47.77</v>
+      </c>
+      <c r="AF168" s="2" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="AG168" s="2" t="n">
+        <v>-2.0286</v>
+      </c>
+      <c r="AH168" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI168" s="2" t="n">
+        <v>47.77</v>
+      </c>
+      <c r="AJ168" s="2" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="AK168" s="2" t="n">
+        <v>-2.0286</v>
+      </c>
+      <c r="AL168" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM168" s="2" t="n">
+        <v>47.77</v>
+      </c>
+      <c r="AN168" s="2" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="AO168" s="2" t="n">
+        <v>-2.0588</v>
+      </c>
+      <c r="AP168" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ168" s="2" t="n">
+        <v>47.76</v>
+      </c>
+      <c r="AR168" s="2" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="AS168" s="2" t="n">
+        <v>-2.0588</v>
+      </c>
+      <c r="AT168" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU168" s="2" t="n">
+        <v>47.76</v>
+      </c>
+      <c r="AV168" s="2" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="AW168" s="2" t="n">
+        <v>-2.0588</v>
+      </c>
+      <c r="AX168" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY168" s="2" t="n">
+        <v>47.76</v>
+      </c>
+      <c r="AZ168" s="2" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="BA168" s="2" t="n">
+        <v>0.00105</v>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
@@ -31440,8 +31925,14 @@
           <t>off</t>
         </is>
       </c>
-      <c r="H169" s="2" t="n"/>
-      <c r="I169" s="2" t="n"/>
+      <c r="H169" s="2" t="n">
+        <v>-10.089</v>
+      </c>
+      <c r="I169" s="2" t="inlineStr">
+        <is>
+          <t>next open</t>
+        </is>
+      </c>
       <c r="J169" s="2" t="inlineStr">
         <is>
           <t>eod_squeeze</t>
@@ -31495,33 +31986,87 @@
       <c r="Z169" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA169" s="2" t="n"/>
-      <c r="AB169" s="2" t="n"/>
-      <c r="AC169" s="2" t="n"/>
-      <c r="AD169" s="2" t="n"/>
-      <c r="AE169" s="2" t="n"/>
-      <c r="AF169" s="2" t="n"/>
-      <c r="AG169" s="2" t="n"/>
-      <c r="AH169" s="2" t="n"/>
-      <c r="AI169" s="2" t="n"/>
-      <c r="AJ169" s="2" t="n"/>
-      <c r="AK169" s="2" t="n"/>
-      <c r="AL169" s="2" t="n"/>
-      <c r="AM169" s="2" t="n"/>
-      <c r="AN169" s="2" t="n"/>
-      <c r="AO169" s="2" t="n"/>
-      <c r="AP169" s="2" t="n"/>
-      <c r="AQ169" s="2" t="n"/>
-      <c r="AR169" s="2" t="n"/>
-      <c r="AS169" s="2" t="n"/>
-      <c r="AT169" s="2" t="n"/>
-      <c r="AU169" s="2" t="n"/>
-      <c r="AV169" s="2" t="n"/>
-      <c r="AW169" s="2" t="n"/>
-      <c r="AX169" s="2" t="n"/>
-      <c r="AY169" s="2" t="n"/>
-      <c r="AZ169" s="2" t="n"/>
-      <c r="BA169" s="2" t="n"/>
+      <c r="AA169" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB169" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC169" s="2" t="n">
+        <v>-14.7114</v>
+      </c>
+      <c r="AD169" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE169" s="2" t="n">
+        <v>4.415</v>
+      </c>
+      <c r="AF169" s="2" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="AG169" s="2" t="n">
+        <v>-14.7114</v>
+      </c>
+      <c r="AH169" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI169" s="2" t="n">
+        <v>4.415</v>
+      </c>
+      <c r="AJ169" s="2" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="AK169" s="2" t="n">
+        <v>-14.7114</v>
+      </c>
+      <c r="AL169" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM169" s="2" t="n">
+        <v>4.415</v>
+      </c>
+      <c r="AN169" s="2" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="AO169" s="2" t="n">
+        <v>-14.7114</v>
+      </c>
+      <c r="AP169" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ169" s="2" t="n">
+        <v>4.415</v>
+      </c>
+      <c r="AR169" s="2" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="AS169" s="2" t="n">
+        <v>-14.7114</v>
+      </c>
+      <c r="AT169" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU169" s="2" t="n">
+        <v>4.415</v>
+      </c>
+      <c r="AV169" s="2" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="AW169" s="2" t="n">
+        <v>-14.7114</v>
+      </c>
+      <c r="AX169" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY169" s="2" t="n">
+        <v>4.415</v>
+      </c>
+      <c r="AZ169" s="2" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="BA169" s="2" t="n">
+        <v>0.00227</v>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
@@ -31553,8 +32098,14 @@
           <t>off</t>
         </is>
       </c>
-      <c r="H170" s="2" t="n"/>
-      <c r="I170" s="2" t="n"/>
+      <c r="H170" s="2" t="n">
+        <v>0.433</v>
+      </c>
+      <c r="I170" s="2" t="inlineStr">
+        <is>
+          <t>breakeven</t>
+        </is>
+      </c>
       <c r="J170" s="2" t="inlineStr">
         <is>
           <t>eod_squeeze</t>
@@ -31608,33 +32159,87 @@
       <c r="Z170" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA170" s="2" t="n"/>
-      <c r="AB170" s="2" t="n"/>
-      <c r="AC170" s="2" t="n"/>
-      <c r="AD170" s="2" t="n"/>
-      <c r="AE170" s="2" t="n"/>
-      <c r="AF170" s="2" t="n"/>
-      <c r="AG170" s="2" t="n"/>
-      <c r="AH170" s="2" t="n"/>
-      <c r="AI170" s="2" t="n"/>
-      <c r="AJ170" s="2" t="n"/>
-      <c r="AK170" s="2" t="n"/>
-      <c r="AL170" s="2" t="n"/>
-      <c r="AM170" s="2" t="n"/>
-      <c r="AN170" s="2" t="n"/>
-      <c r="AO170" s="2" t="n"/>
-      <c r="AP170" s="2" t="n"/>
-      <c r="AQ170" s="2" t="n"/>
-      <c r="AR170" s="2" t="n"/>
-      <c r="AS170" s="2" t="n"/>
-      <c r="AT170" s="2" t="n"/>
-      <c r="AU170" s="2" t="n"/>
-      <c r="AV170" s="2" t="n"/>
-      <c r="AW170" s="2" t="n"/>
-      <c r="AX170" s="2" t="n"/>
-      <c r="AY170" s="2" t="n"/>
-      <c r="AZ170" s="2" t="n"/>
-      <c r="BA170" s="2" t="n"/>
+      <c r="AA170" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB170" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC170" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AD170" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AE170" s="2" t="n">
+        <v>46.315</v>
+      </c>
+      <c r="AF170" s="2" t="n">
+        <v>0.455</v>
+      </c>
+      <c r="AG170" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AH170" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI170" s="2" t="n">
+        <v>46.315</v>
+      </c>
+      <c r="AJ170" s="2" t="n">
+        <v>0.455</v>
+      </c>
+      <c r="AK170" s="2" t="n">
+        <v>0.8022</v>
+      </c>
+      <c r="AL170" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AM170" s="2" t="n">
+        <v>46.315</v>
+      </c>
+      <c r="AN170" s="2" t="n">
+        <v>0.455</v>
+      </c>
+      <c r="AO170" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AP170" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AQ170" s="2" t="n">
+        <v>46.315</v>
+      </c>
+      <c r="AR170" s="2" t="n">
+        <v>0.455</v>
+      </c>
+      <c r="AS170" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AT170" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU170" s="2" t="n">
+        <v>46.315</v>
+      </c>
+      <c r="AV170" s="2" t="n">
+        <v>0.455</v>
+      </c>
+      <c r="AW170" s="2" t="n">
+        <v>0.8022</v>
+      </c>
+      <c r="AX170" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AY170" s="2" t="n">
+        <v>46.315</v>
+      </c>
+      <c r="AZ170" s="2" t="n">
+        <v>0.455</v>
+      </c>
+      <c r="BA170" s="2" t="n">
+        <v>0.00108</v>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
@@ -31666,8 +32271,14 @@
           <t>off</t>
         </is>
       </c>
-      <c r="H171" s="2" t="n"/>
-      <c r="I171" s="2" t="n"/>
+      <c r="H171" s="2" t="n">
+        <v>-0.826</v>
+      </c>
+      <c r="I171" s="2" t="inlineStr">
+        <is>
+          <t>next open</t>
+        </is>
+      </c>
       <c r="J171" s="2" t="inlineStr">
         <is>
           <t>eod_squeeze</t>
@@ -31721,33 +32332,3607 @@
       <c r="Z171" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA171" s="2" t="n"/>
-      <c r="AB171" s="2" t="n"/>
-      <c r="AC171" s="2" t="n"/>
-      <c r="AD171" s="2" t="n"/>
-      <c r="AE171" s="2" t="n"/>
-      <c r="AF171" s="2" t="n"/>
-      <c r="AG171" s="2" t="n"/>
-      <c r="AH171" s="2" t="n"/>
-      <c r="AI171" s="2" t="n"/>
-      <c r="AJ171" s="2" t="n"/>
-      <c r="AK171" s="2" t="n"/>
-      <c r="AL171" s="2" t="n"/>
-      <c r="AM171" s="2" t="n"/>
-      <c r="AN171" s="2" t="n"/>
-      <c r="AO171" s="2" t="n"/>
-      <c r="AP171" s="2" t="n"/>
-      <c r="AQ171" s="2" t="n"/>
-      <c r="AR171" s="2" t="n"/>
-      <c r="AS171" s="2" t="n"/>
-      <c r="AT171" s="2" t="n"/>
-      <c r="AU171" s="2" t="n"/>
-      <c r="AV171" s="2" t="n"/>
-      <c r="AW171" s="2" t="n"/>
-      <c r="AX171" s="2" t="n"/>
-      <c r="AY171" s="2" t="n"/>
-      <c r="AZ171" s="2" t="n"/>
-      <c r="BA171" s="2" t="n"/>
+      <c r="AA171" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB171" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC171" s="2" t="n">
+        <v>-0.5789</v>
+      </c>
+      <c r="AD171" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE171" s="2" t="n">
+        <v>9.355</v>
+      </c>
+      <c r="AF171" s="2" t="n">
+        <v>0.095</v>
+      </c>
+      <c r="AG171" s="2" t="n">
+        <v>-0.5789</v>
+      </c>
+      <c r="AH171" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI171" s="2" t="n">
+        <v>9.355</v>
+      </c>
+      <c r="AJ171" s="2" t="n">
+        <v>0.095</v>
+      </c>
+      <c r="AK171" s="2" t="n">
+        <v>-0.5789</v>
+      </c>
+      <c r="AL171" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM171" s="2" t="n">
+        <v>9.355</v>
+      </c>
+      <c r="AN171" s="2" t="n">
+        <v>0.095</v>
+      </c>
+      <c r="AO171" s="2" t="n">
+        <v>-0.5789</v>
+      </c>
+      <c r="AP171" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ171" s="2" t="n">
+        <v>9.355</v>
+      </c>
+      <c r="AR171" s="2" t="n">
+        <v>0.095</v>
+      </c>
+      <c r="AS171" s="2" t="n">
+        <v>-0.5789</v>
+      </c>
+      <c r="AT171" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU171" s="2" t="n">
+        <v>9.355</v>
+      </c>
+      <c r="AV171" s="2" t="n">
+        <v>0.095</v>
+      </c>
+      <c r="AW171" s="2" t="n">
+        <v>-0.5789</v>
+      </c>
+      <c r="AX171" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY171" s="2" t="n">
+        <v>9.355</v>
+      </c>
+      <c r="AZ171" s="2" t="n">
+        <v>0.095</v>
+      </c>
+      <c r="BA171" s="2" t="n">
+        <v>0.00107</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B172" s="2" t="inlineStr">
+        <is>
+          <t>09:48</t>
+        </is>
+      </c>
+      <c r="C172" s="2" t="inlineStr">
+        <is>
+          <t>CORT</t>
+        </is>
+      </c>
+      <c r="D172" s="2" t="n">
+        <v>88.56</v>
+      </c>
+      <c r="E172" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26 09:47:00-04:00</t>
+        </is>
+      </c>
+      <c r="F172" s="2" t="n"/>
+      <c r="G172" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H172" s="2" t="n">
+        <v>-1.043</v>
+      </c>
+      <c r="I172" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="J172" s="2" t="inlineStr">
+        <is>
+          <t>orb15</t>
+        </is>
+      </c>
+      <c r="K172" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="L172" s="2" t="n">
+        <v>0.0620195307522533</v>
+      </c>
+      <c r="M172" s="2" t="n">
+        <v>0.002795223178004402</v>
+      </c>
+      <c r="N172" s="2" t="n">
+        <v>1.645299068053378</v>
+      </c>
+      <c r="O172" s="2" t="n">
+        <v>0.02000658251783816</v>
+      </c>
+      <c r="P172" s="2" t="n">
+        <v>0.02878760354088921</v>
+      </c>
+      <c r="Q172" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R172" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S172" s="2" t="n">
+        <v>4.512890383094586</v>
+      </c>
+      <c r="T172" s="2" t="n">
+        <v>0.003921262179805707</v>
+      </c>
+      <c r="U172" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V172" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="W172" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="X172" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y172" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z172" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA172" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB172" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC172" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AD172" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE172" s="2" t="n">
+        <v>91.435</v>
+      </c>
+      <c r="AF172" s="2" t="n">
+        <v>2.875</v>
+      </c>
+      <c r="AG172" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AH172" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI172" s="2" t="n">
+        <v>91.435</v>
+      </c>
+      <c r="AJ172" s="2" t="n">
+        <v>2.875</v>
+      </c>
+      <c r="AK172" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AL172" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM172" s="2" t="n">
+        <v>91.435</v>
+      </c>
+      <c r="AN172" s="2" t="n">
+        <v>2.875</v>
+      </c>
+      <c r="AO172" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AP172" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ172" s="2" t="n">
+        <v>91.185</v>
+      </c>
+      <c r="AR172" s="2" t="n">
+        <v>2.625</v>
+      </c>
+      <c r="AS172" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AT172" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU172" s="2" t="n">
+        <v>91.185</v>
+      </c>
+      <c r="AV172" s="2" t="n">
+        <v>2.625</v>
+      </c>
+      <c r="AW172" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AX172" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY172" s="2" t="n">
+        <v>91.185</v>
+      </c>
+      <c r="AZ172" s="2" t="n">
+        <v>2.625</v>
+      </c>
+      <c r="BA172" s="2" t="n">
+        <v>0.00691</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B173" s="2" t="inlineStr">
+        <is>
+          <t>09:51</t>
+        </is>
+      </c>
+      <c r="C173" s="2" t="inlineStr">
+        <is>
+          <t>RRC</t>
+        </is>
+      </c>
+      <c r="D173" s="2" t="n">
+        <v>51.28</v>
+      </c>
+      <c r="E173" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26 09:50:00-04:00</t>
+        </is>
+      </c>
+      <c r="F173" s="2" t="n"/>
+      <c r="G173" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H173" s="2" t="n">
+        <v>0.208</v>
+      </c>
+      <c r="I173" s="2" t="inlineStr">
+        <is>
+          <t>time</t>
+        </is>
+      </c>
+      <c r="J173" s="2" t="inlineStr">
+        <is>
+          <t>orb5</t>
+        </is>
+      </c>
+      <c r="K173" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="L173" s="2" t="n">
+        <v>0.1614674516741468</v>
+      </c>
+      <c r="M173" s="2" t="n">
+        <v>0.1161028074311174</v>
+      </c>
+      <c r="N173" s="2" t="n">
+        <v>3.463741271091359</v>
+      </c>
+      <c r="O173" s="2" t="n">
+        <v>0.02214554056517049</v>
+      </c>
+      <c r="P173" s="2" t="n">
+        <v>0.03007374624564008</v>
+      </c>
+      <c r="Q173" s="2" t="n">
+        <v>-0.0005482018481800521</v>
+      </c>
+      <c r="R173" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S173" s="2" t="n">
+        <v>3.967836050044687</v>
+      </c>
+      <c r="T173" s="2" t="n">
+        <v>0.004135054292916829</v>
+      </c>
+      <c r="U173" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V173" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W173" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X173" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y173" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z173" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA173" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB173" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC173" s="2" t="n">
+        <v>0.3192</v>
+      </c>
+      <c r="AD173" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE173" s="2" t="n">
+        <v>52.87</v>
+      </c>
+      <c r="AF173" s="2" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="AG173" s="2" t="n">
+        <v>0.3192</v>
+      </c>
+      <c r="AH173" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI173" s="2" t="n">
+        <v>52.87</v>
+      </c>
+      <c r="AJ173" s="2" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="AK173" s="2" t="n">
+        <v>0.3192</v>
+      </c>
+      <c r="AL173" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM173" s="2" t="n">
+        <v>52.87</v>
+      </c>
+      <c r="AN173" s="2" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="AO173" s="2" t="n">
+        <v>0.3192</v>
+      </c>
+      <c r="AP173" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ173" s="2" t="n">
+        <v>52.87</v>
+      </c>
+      <c r="AR173" s="2" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="AS173" s="2" t="n">
+        <v>0.3192</v>
+      </c>
+      <c r="AT173" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU173" s="2" t="n">
+        <v>52.87</v>
+      </c>
+      <c r="AV173" s="2" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="AW173" s="2" t="n">
+        <v>0.3192</v>
+      </c>
+      <c r="AX173" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY173" s="2" t="n">
+        <v>52.87</v>
+      </c>
+      <c r="AZ173" s="2" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="BA173" s="2" t="n">
+        <v>0.00076</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B174" s="2" t="inlineStr">
+        <is>
+          <t>09:51</t>
+        </is>
+      </c>
+      <c r="C174" s="2" t="inlineStr">
+        <is>
+          <t>RRC</t>
+        </is>
+      </c>
+      <c r="D174" s="2" t="n">
+        <v>51.4</v>
+      </c>
+      <c r="E174" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26 09:50:00-04:00</t>
+        </is>
+      </c>
+      <c r="F174" s="2" t="n"/>
+      <c r="G174" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H174" s="2" t="n">
+        <v>0.224</v>
+      </c>
+      <c r="I174" s="2" t="inlineStr">
+        <is>
+          <t>time</t>
+        </is>
+      </c>
+      <c r="J174" s="2" t="inlineStr">
+        <is>
+          <t>orb15</t>
+        </is>
+      </c>
+      <c r="K174" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="L174" s="2" t="n">
+        <v>0.1614674516741468</v>
+      </c>
+      <c r="M174" s="2" t="n">
+        <v>0.1161028074311174</v>
+      </c>
+      <c r="N174" s="2" t="n">
+        <v>3.463741271091359</v>
+      </c>
+      <c r="O174" s="2" t="n">
+        <v>0.02214554056517049</v>
+      </c>
+      <c r="P174" s="2" t="n">
+        <v>0.02780402802312603</v>
+      </c>
+      <c r="Q174" s="2" t="n">
+        <v>-0.0005482018481800521</v>
+      </c>
+      <c r="R174" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S174" s="2" t="n">
+        <v>3.967836050044687</v>
+      </c>
+      <c r="T174" s="2" t="n">
+        <v>0.004135054292916829</v>
+      </c>
+      <c r="U174" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V174" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W174" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X174" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y174" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z174" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA174" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB174" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC174" s="2" t="n">
+        <v>0.3452</v>
+      </c>
+      <c r="AD174" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE174" s="2" t="n">
+        <v>52.87</v>
+      </c>
+      <c r="AF174" s="2" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="AG174" s="2" t="n">
+        <v>0.3452</v>
+      </c>
+      <c r="AH174" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI174" s="2" t="n">
+        <v>52.87</v>
+      </c>
+      <c r="AJ174" s="2" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="AK174" s="2" t="n">
+        <v>0.3452</v>
+      </c>
+      <c r="AL174" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM174" s="2" t="n">
+        <v>52.87</v>
+      </c>
+      <c r="AN174" s="2" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="AO174" s="2" t="n">
+        <v>0.3452</v>
+      </c>
+      <c r="AP174" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ174" s="2" t="n">
+        <v>52.87</v>
+      </c>
+      <c r="AR174" s="2" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="AS174" s="2" t="n">
+        <v>0.3452</v>
+      </c>
+      <c r="AT174" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU174" s="2" t="n">
+        <v>52.87</v>
+      </c>
+      <c r="AV174" s="2" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="AW174" s="2" t="n">
+        <v>0.3452</v>
+      </c>
+      <c r="AX174" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY174" s="2" t="n">
+        <v>52.87</v>
+      </c>
+      <c r="AZ174" s="2" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="BA174" s="2" t="n">
+        <v>0.00076</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B175" s="2" t="inlineStr">
+        <is>
+          <t>09:51</t>
+        </is>
+      </c>
+      <c r="C175" s="2" t="inlineStr">
+        <is>
+          <t>RRC</t>
+        </is>
+      </c>
+      <c r="D175" s="2" t="n">
+        <v>51.63</v>
+      </c>
+      <c r="E175" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26 09:50:00-04:00</t>
+        </is>
+      </c>
+      <c r="F175" s="2" t="n"/>
+      <c r="G175" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H175" s="2" t="n">
+        <v>0.263</v>
+      </c>
+      <c r="I175" s="2" t="inlineStr">
+        <is>
+          <t>time</t>
+        </is>
+      </c>
+      <c r="J175" s="2" t="inlineStr">
+        <is>
+          <t>pm_high_break</t>
+        </is>
+      </c>
+      <c r="K175" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="L175" s="2" t="n">
+        <v>0.1614674516741468</v>
+      </c>
+      <c r="M175" s="2" t="n">
+        <v>0.1161028074311174</v>
+      </c>
+      <c r="N175" s="2" t="n">
+        <v>3.463741271091359</v>
+      </c>
+      <c r="O175" s="2" t="n">
+        <v>0.02214554056517049</v>
+      </c>
+      <c r="P175" s="2" t="n">
+        <v>0.02345373476330725</v>
+      </c>
+      <c r="Q175" s="2" t="n">
+        <v>-0.0005482018481800521</v>
+      </c>
+      <c r="R175" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S175" s="2" t="n">
+        <v>3.967836050044687</v>
+      </c>
+      <c r="T175" s="2" t="n">
+        <v>0.004135054292916829</v>
+      </c>
+      <c r="U175" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V175" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W175" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X175" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y175" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z175" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA175" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB175" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC175" s="2" t="n">
+        <v>0.4093</v>
+      </c>
+      <c r="AD175" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE175" s="2" t="n">
+        <v>52.87</v>
+      </c>
+      <c r="AF175" s="2" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="AG175" s="2" t="n">
+        <v>0.4093</v>
+      </c>
+      <c r="AH175" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI175" s="2" t="n">
+        <v>52.87</v>
+      </c>
+      <c r="AJ175" s="2" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="AK175" s="2" t="n">
+        <v>0.4093</v>
+      </c>
+      <c r="AL175" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM175" s="2" t="n">
+        <v>52.87</v>
+      </c>
+      <c r="AN175" s="2" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="AO175" s="2" t="n">
+        <v>0.4093</v>
+      </c>
+      <c r="AP175" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ175" s="2" t="n">
+        <v>52.87</v>
+      </c>
+      <c r="AR175" s="2" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="AS175" s="2" t="n">
+        <v>0.4093</v>
+      </c>
+      <c r="AT175" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU175" s="2" t="n">
+        <v>52.87</v>
+      </c>
+      <c r="AV175" s="2" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="AW175" s="2" t="n">
+        <v>0.4093</v>
+      </c>
+      <c r="AX175" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY175" s="2" t="n">
+        <v>52.87</v>
+      </c>
+      <c r="AZ175" s="2" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="BA175" s="2" t="n">
+        <v>0.00076</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B176" s="2" t="inlineStr">
+        <is>
+          <t>09:53</t>
+        </is>
+      </c>
+      <c r="C176" s="2" t="inlineStr">
+        <is>
+          <t>BWMX</t>
+        </is>
+      </c>
+      <c r="D176" s="2" t="n">
+        <v>16.43</v>
+      </c>
+      <c r="E176" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26 09:52:00-04:00</t>
+        </is>
+      </c>
+      <c r="F176" s="2" t="n"/>
+      <c r="G176" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H176" s="2" t="n">
+        <v>-0.639</v>
+      </c>
+      <c r="I176" s="2" t="inlineStr">
+        <is>
+          <t>time</t>
+        </is>
+      </c>
+      <c r="J176" s="2" t="inlineStr">
+        <is>
+          <t>orb5</t>
+        </is>
+      </c>
+      <c r="K176" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="L176" s="2" t="n">
+        <v>0.08659399411523605</v>
+      </c>
+      <c r="M176" s="2" t="n">
+        <v>0.06542658420656622</v>
+      </c>
+      <c r="N176" s="2" t="n">
+        <v>2.682873388415721</v>
+      </c>
+      <c r="O176" s="2" t="n">
+        <v>0.01399564768118866</v>
+      </c>
+      <c r="P176" s="2" t="n">
+        <v>0.03010628795626476</v>
+      </c>
+      <c r="Q176" s="2" t="n">
+        <v>-0.007615651030504655</v>
+      </c>
+      <c r="R176" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S176" s="2" t="n">
+        <v>2.829677720750332</v>
+      </c>
+      <c r="T176" s="2" t="n">
+        <v>0.004842367268186543</v>
+      </c>
+      <c r="U176" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V176" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="W176" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X176" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y176" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z176" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA176" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB176" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC176" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AD176" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AE176" s="2" t="n">
+        <v>16.94</v>
+      </c>
+      <c r="AF176" s="2" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="AG176" s="2" t="n">
+        <v>-0.5784</v>
+      </c>
+      <c r="AH176" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI176" s="2" t="n">
+        <v>16.94</v>
+      </c>
+      <c r="AJ176" s="2" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="AK176" s="2" t="n">
+        <v>0.8235</v>
+      </c>
+      <c r="AL176" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AM176" s="2" t="n">
+        <v>16.94</v>
+      </c>
+      <c r="AN176" s="2" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="AO176" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AP176" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AQ176" s="2" t="n">
+        <v>16.94</v>
+      </c>
+      <c r="AR176" s="2" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="AS176" s="2" t="n">
+        <v>-0.5784</v>
+      </c>
+      <c r="AT176" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU176" s="2" t="n">
+        <v>16.94</v>
+      </c>
+      <c r="AV176" s="2" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="AW176" s="2" t="n">
+        <v>0.8235</v>
+      </c>
+      <c r="AX176" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AY176" s="2" t="n">
+        <v>16.94</v>
+      </c>
+      <c r="AZ176" s="2" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="BA176" s="2" t="n">
+        <v>0.01353</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B177" s="2" t="inlineStr">
+        <is>
+          <t>09:55</t>
+        </is>
+      </c>
+      <c r="C177" s="2" t="inlineStr">
+        <is>
+          <t>MLCO</t>
+        </is>
+      </c>
+      <c r="D177" s="2" t="n">
+        <v>3.84</v>
+      </c>
+      <c r="E177" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26 09:54:00-04:00</t>
+        </is>
+      </c>
+      <c r="F177" s="2" t="n"/>
+      <c r="G177" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H177" s="2" t="n">
+        <v>-0.829</v>
+      </c>
+      <c r="I177" s="2" t="inlineStr">
+        <is>
+          <t>time</t>
+        </is>
+      </c>
+      <c r="J177" s="2" t="inlineStr">
+        <is>
+          <t>orb15</t>
+        </is>
+      </c>
+      <c r="K177" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="L177" s="2" t="n">
+        <v>0.05898124061266796</v>
+      </c>
+      <c r="M177" s="2" t="n">
+        <v>0.01072385030790524</v>
+      </c>
+      <c r="N177" s="2" t="n">
+        <v>1.416064361519773</v>
+      </c>
+      <c r="O177" s="2" t="n">
+        <v>0.02066411134925517</v>
+      </c>
+      <c r="P177" s="2" t="n">
+        <v>0.02784811300147201</v>
+      </c>
+      <c r="Q177" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R177" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S177" s="2" t="n">
+        <v>1.373715590984857</v>
+      </c>
+      <c r="T177" s="2" t="n">
+        <v>0.005131813840557609</v>
+      </c>
+      <c r="U177" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V177" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W177" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X177" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y177" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z177" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA177" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB177" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC177" s="2" t="n">
+        <v>-0.6443</v>
+      </c>
+      <c r="AD177" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE177" s="2" t="n">
+        <v>3.9665</v>
+      </c>
+      <c r="AF177" s="2" t="n">
+        <v>0.1265</v>
+      </c>
+      <c r="AG177" s="2" t="n">
+        <v>-0.6443</v>
+      </c>
+      <c r="AH177" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI177" s="2" t="n">
+        <v>3.9665</v>
+      </c>
+      <c r="AJ177" s="2" t="n">
+        <v>0.1265</v>
+      </c>
+      <c r="AK177" s="2" t="n">
+        <v>-0.6443</v>
+      </c>
+      <c r="AL177" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM177" s="2" t="n">
+        <v>3.9665</v>
+      </c>
+      <c r="AN177" s="2" t="n">
+        <v>0.1265</v>
+      </c>
+      <c r="AO177" s="2" t="n">
+        <v>-0.5755</v>
+      </c>
+      <c r="AP177" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ177" s="2" t="n">
+        <v>3.946</v>
+      </c>
+      <c r="AR177" s="2" t="n">
+        <v>0.106</v>
+      </c>
+      <c r="AS177" s="2" t="n">
+        <v>-0.5755</v>
+      </c>
+      <c r="AT177" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU177" s="2" t="n">
+        <v>3.946</v>
+      </c>
+      <c r="AV177" s="2" t="n">
+        <v>0.106</v>
+      </c>
+      <c r="AW177" s="2" t="n">
+        <v>-0.5755</v>
+      </c>
+      <c r="AX177" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY177" s="2" t="n">
+        <v>3.946</v>
+      </c>
+      <c r="AZ177" s="2" t="n">
+        <v>0.106</v>
+      </c>
+      <c r="BA177" s="2" t="n">
+        <v>0.00252</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B178" s="2" t="inlineStr">
+        <is>
+          <t>09:56</t>
+        </is>
+      </c>
+      <c r="C178" s="2" t="inlineStr">
+        <is>
+          <t>BWMX</t>
+        </is>
+      </c>
+      <c r="D178" s="2" t="n">
+        <v>16.68</v>
+      </c>
+      <c r="E178" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26 09:55:00-04:00</t>
+        </is>
+      </c>
+      <c r="F178" s="2" t="n"/>
+      <c r="G178" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H178" s="2" t="n">
+        <v>-1.071</v>
+      </c>
+      <c r="I178" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="J178" s="2" t="inlineStr">
+        <is>
+          <t>orb15</t>
+        </is>
+      </c>
+      <c r="K178" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="L178" s="2" t="n">
+        <v>0.09653618640387096</v>
+      </c>
+      <c r="M178" s="2" t="n">
+        <v>0.06542658420656622</v>
+      </c>
+      <c r="N178" s="2" t="n">
+        <v>2.604121511266614</v>
+      </c>
+      <c r="O178" s="2" t="n">
+        <v>0.02292279163854838</v>
+      </c>
+      <c r="P178" s="2" t="n">
+        <v>0.02427606493264366</v>
+      </c>
+      <c r="Q178" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R178" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S178" s="2" t="n">
+        <v>2.838785982924811</v>
+      </c>
+      <c r="T178" s="2" t="n">
+        <v>0.005592326228453404</v>
+      </c>
+      <c r="U178" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V178" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="W178" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X178" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y178" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z178" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA178" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB178" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC178" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AD178" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE178" s="2" t="n">
+        <v>17.07</v>
+      </c>
+      <c r="AF178" s="2" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="AG178" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AH178" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI178" s="2" t="n">
+        <v>17.07</v>
+      </c>
+      <c r="AJ178" s="2" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="AK178" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AL178" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM178" s="2" t="n">
+        <v>17.07</v>
+      </c>
+      <c r="AN178" s="2" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="AO178" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AP178" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ178" s="2" t="n">
+        <v>17.07</v>
+      </c>
+      <c r="AR178" s="2" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="AS178" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AT178" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU178" s="2" t="n">
+        <v>17.07</v>
+      </c>
+      <c r="AV178" s="2" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="AW178" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AX178" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY178" s="2" t="n">
+        <v>17.07</v>
+      </c>
+      <c r="AZ178" s="2" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="BA178" s="2" t="n">
+        <v>0.00586</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B179" s="2" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="C179" s="2" t="inlineStr">
+        <is>
+          <t>RRC</t>
+        </is>
+      </c>
+      <c r="D179" s="2" t="n">
+        <v>52.46</v>
+      </c>
+      <c r="E179" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26 09:59:00-04:00</t>
+        </is>
+      </c>
+      <c r="F179" s="2" t="n"/>
+      <c r="G179" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H179" s="2" t="n">
+        <v>-1.1</v>
+      </c>
+      <c r="I179" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="J179" s="2" t="inlineStr">
+        <is>
+          <t>bull_flag</t>
+        </is>
+      </c>
+      <c r="K179" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="L179" s="2" t="n">
+        <v>0.1680579445134187</v>
+      </c>
+      <c r="M179" s="2" t="n">
+        <v>0.1161028074311174</v>
+      </c>
+      <c r="N179" s="2" t="n">
+        <v>3.326273929797391</v>
+      </c>
+      <c r="O179" s="2" t="n">
+        <v>0.02384568736697346</v>
+      </c>
+      <c r="P179" s="2" t="n">
+        <v>0.01335336079360627</v>
+      </c>
+      <c r="Q179" s="2" t="n">
+        <v>-0.0007517556138996184</v>
+      </c>
+      <c r="R179" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S179" s="2" t="n">
+        <v>3.973494293078506</v>
+      </c>
+      <c r="T179" s="2" t="n">
+        <v>0.003789629845700304</v>
+      </c>
+      <c r="U179" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V179" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W179" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X179" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y179" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z179" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA179" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB179" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC179" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AD179" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE179" s="2" t="n">
+        <v>53.18</v>
+      </c>
+      <c r="AF179" s="2" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="AG179" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AH179" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI179" s="2" t="n">
+        <v>53.18</v>
+      </c>
+      <c r="AJ179" s="2" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="AK179" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AL179" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM179" s="2" t="n">
+        <v>53.18</v>
+      </c>
+      <c r="AN179" s="2" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="AO179" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AP179" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ179" s="2" t="n">
+        <v>53.17</v>
+      </c>
+      <c r="AR179" s="2" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="AS179" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AT179" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU179" s="2" t="n">
+        <v>53.17</v>
+      </c>
+      <c r="AV179" s="2" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="AW179" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AX179" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY179" s="2" t="n">
+        <v>53.17</v>
+      </c>
+      <c r="AZ179" s="2" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="BA179" s="2" t="n">
+        <v>0.00056</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B180" s="2" t="inlineStr">
+        <is>
+          <t>10:01</t>
+        </is>
+      </c>
+      <c r="C180" s="2" t="inlineStr">
+        <is>
+          <t>RRC</t>
+        </is>
+      </c>
+      <c r="D180" s="2" t="n">
+        <v>51.97</v>
+      </c>
+      <c r="E180" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26 10:00:00-04:00</t>
+        </is>
+      </c>
+      <c r="F180" s="2" t="n"/>
+      <c r="G180" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H180" s="2" t="n">
+        <v>-0.059</v>
+      </c>
+      <c r="I180" s="2" t="inlineStr">
+        <is>
+          <t>time</t>
+        </is>
+      </c>
+      <c r="J180" s="2" t="inlineStr">
+        <is>
+          <t>vwap_pullback</t>
+        </is>
+      </c>
+      <c r="K180" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="L180" s="2" t="n">
+        <v>0.1705843433998488</v>
+      </c>
+      <c r="M180" s="2" t="n">
+        <v>0.1161028074311174</v>
+      </c>
+      <c r="N180" s="2" t="n">
+        <v>3.303193779805128</v>
+      </c>
+      <c r="O180" s="2" t="n">
+        <v>0.0258179085421042</v>
+      </c>
+      <c r="P180" s="2" t="n">
+        <v>0.02467861220189111</v>
+      </c>
+      <c r="Q180" s="2" t="n">
+        <v>-9.384627564867909e-05</v>
+      </c>
+      <c r="R180" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S180" s="2" t="n">
+        <v>3.975654862809301</v>
+      </c>
+      <c r="T180" s="2" t="n">
+        <v>0.004842367268186543</v>
+      </c>
+      <c r="U180" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V180" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W180" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X180" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y180" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z180" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA180" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB180" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC180" s="2" t="n">
+        <v>0.0583</v>
+      </c>
+      <c r="AD180" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE180" s="2" t="n">
+        <v>53.3</v>
+      </c>
+      <c r="AF180" s="2" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="AG180" s="2" t="n">
+        <v>0.0583</v>
+      </c>
+      <c r="AH180" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI180" s="2" t="n">
+        <v>53.3</v>
+      </c>
+      <c r="AJ180" s="2" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="AK180" s="2" t="n">
+        <v>0.0583</v>
+      </c>
+      <c r="AL180" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM180" s="2" t="n">
+        <v>53.3</v>
+      </c>
+      <c r="AN180" s="2" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="AO180" s="2" t="n">
+        <v>0.0703</v>
+      </c>
+      <c r="AP180" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ180" s="2" t="n">
+        <v>53.285</v>
+      </c>
+      <c r="AR180" s="2" t="n">
+        <v>1.315</v>
+      </c>
+      <c r="AS180" s="2" t="n">
+        <v>0.0703</v>
+      </c>
+      <c r="AT180" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU180" s="2" t="n">
+        <v>53.285</v>
+      </c>
+      <c r="AV180" s="2" t="n">
+        <v>1.315</v>
+      </c>
+      <c r="AW180" s="2" t="n">
+        <v>0.0703</v>
+      </c>
+      <c r="AX180" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY180" s="2" t="n">
+        <v>53.285</v>
+      </c>
+      <c r="AZ180" s="2" t="n">
+        <v>1.315</v>
+      </c>
+      <c r="BA180" s="2" t="n">
+        <v>0.00056</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B181" s="2" t="inlineStr">
+        <is>
+          <t>10:05</t>
+        </is>
+      </c>
+      <c r="C181" s="2" t="inlineStr">
+        <is>
+          <t>CORT</t>
+        </is>
+      </c>
+      <c r="D181" s="2" t="n">
+        <v>90.06999999999999</v>
+      </c>
+      <c r="E181" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26 10:04:00-04:00</t>
+        </is>
+      </c>
+      <c r="F181" s="2" t="n"/>
+      <c r="G181" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H181" s="2" t="n"/>
+      <c r="I181" s="2" t="n"/>
+      <c r="J181" s="2" t="inlineStr">
+        <is>
+          <t>vwap_pullback</t>
+        </is>
+      </c>
+      <c r="K181" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="L181" s="2" t="n">
+        <v>0.05095504273118467</v>
+      </c>
+      <c r="M181" s="2" t="n">
+        <v>0.002795223178004402</v>
+      </c>
+      <c r="N181" s="2" t="n">
+        <v>1.55359037437974</v>
+      </c>
+      <c r="O181" s="2" t="n">
+        <v>0.002227835160107716</v>
+      </c>
+      <c r="P181" s="2" t="n">
+        <v>0.001828565514883377</v>
+      </c>
+      <c r="Q181" s="2" t="n">
+        <v>-0.01624418521184179</v>
+      </c>
+      <c r="R181" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S181" s="2" t="n">
+        <v>4.502417385177284</v>
+      </c>
+      <c r="T181" s="2" t="n">
+        <v>0.004987090554372076</v>
+      </c>
+      <c r="U181" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V181" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="W181" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="X181" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y181" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z181" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA181" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB181" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC181" s="2" t="n"/>
+      <c r="AD181" s="2" t="n"/>
+      <c r="AE181" s="2" t="n"/>
+      <c r="AF181" s="2" t="n"/>
+      <c r="AG181" s="2" t="n"/>
+      <c r="AH181" s="2" t="n"/>
+      <c r="AI181" s="2" t="n"/>
+      <c r="AJ181" s="2" t="n"/>
+      <c r="AK181" s="2" t="n"/>
+      <c r="AL181" s="2" t="n"/>
+      <c r="AM181" s="2" t="n"/>
+      <c r="AN181" s="2" t="n"/>
+      <c r="AO181" s="2" t="n"/>
+      <c r="AP181" s="2" t="n"/>
+      <c r="AQ181" s="2" t="n"/>
+      <c r="AR181" s="2" t="n"/>
+      <c r="AS181" s="2" t="n"/>
+      <c r="AT181" s="2" t="n"/>
+      <c r="AU181" s="2" t="n"/>
+      <c r="AV181" s="2" t="n"/>
+      <c r="AW181" s="2" t="n"/>
+      <c r="AX181" s="2" t="n"/>
+      <c r="AY181" s="2" t="n"/>
+      <c r="AZ181" s="2" t="n"/>
+      <c r="BA181" s="2" t="n">
+        <v>0.00477</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B182" s="2" t="inlineStr">
+        <is>
+          <t>10:11</t>
+        </is>
+      </c>
+      <c r="C182" s="2" t="inlineStr">
+        <is>
+          <t>EAF</t>
+        </is>
+      </c>
+      <c r="D182" s="2" t="n">
+        <v>10.05</v>
+      </c>
+      <c r="E182" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26 10:10:00-04:00</t>
+        </is>
+      </c>
+      <c r="F182" s="2" t="n"/>
+      <c r="G182" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H182" s="2" t="n">
+        <v>-1.144</v>
+      </c>
+      <c r="I182" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="J182" s="2" t="inlineStr">
+        <is>
+          <t>bull_flag</t>
+        </is>
+      </c>
+      <c r="K182" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="L182" s="2" t="n">
+        <v>0.2056404175008981</v>
+      </c>
+      <c r="M182" s="2" t="n">
+        <v>0.03407755041754346</v>
+      </c>
+      <c r="N182" s="2" t="n">
+        <v>1.817857295002203</v>
+      </c>
+      <c r="O182" s="2" t="n">
+        <v>0.04825944069406329</v>
+      </c>
+      <c r="P182" s="2" t="n">
+        <v>0.02046785810888054</v>
+      </c>
+      <c r="Q182" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R182" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S182" s="2" t="n">
+        <v>2.328252862050794</v>
+      </c>
+      <c r="T182" s="2" t="n">
+        <v>0.005473945471606845</v>
+      </c>
+      <c r="U182" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V182" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W182" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X182" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y182" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z182" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA182" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB182" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC182" s="2" t="n">
+        <v>-1.0647</v>
+      </c>
+      <c r="AD182" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE182" s="2" t="n">
+        <v>10.2665</v>
+      </c>
+      <c r="AF182" s="2" t="n">
+        <v>0.2165</v>
+      </c>
+      <c r="AG182" s="2" t="n">
+        <v>-1.0647</v>
+      </c>
+      <c r="AH182" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI182" s="2" t="n">
+        <v>10.2665</v>
+      </c>
+      <c r="AJ182" s="2" t="n">
+        <v>0.2165</v>
+      </c>
+      <c r="AK182" s="2" t="n">
+        <v>-1.0647</v>
+      </c>
+      <c r="AL182" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM182" s="2" t="n">
+        <v>10.2665</v>
+      </c>
+      <c r="AN182" s="2" t="n">
+        <v>0.2165</v>
+      </c>
+      <c r="AO182" s="2" t="n"/>
+      <c r="AP182" s="2" t="n"/>
+      <c r="AQ182" s="2" t="n"/>
+      <c r="AR182" s="2" t="n"/>
+      <c r="AS182" s="2" t="n"/>
+      <c r="AT182" s="2" t="n"/>
+      <c r="AU182" s="2" t="n"/>
+      <c r="AV182" s="2" t="n"/>
+      <c r="AW182" s="2" t="n"/>
+      <c r="AX182" s="2" t="n"/>
+      <c r="AY182" s="2" t="n"/>
+      <c r="AZ182" s="2" t="n"/>
+      <c r="BA182" s="2" t="n">
+        <v>0.00489</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B183" s="2" t="inlineStr">
+        <is>
+          <t>10:12</t>
+        </is>
+      </c>
+      <c r="C183" s="2" t="inlineStr">
+        <is>
+          <t>LU</t>
+        </is>
+      </c>
+      <c r="D183" s="2" t="n">
+        <v>8.449999999999999</v>
+      </c>
+      <c r="E183" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26 10:11:00-04:00</t>
+        </is>
+      </c>
+      <c r="F183" s="2" t="n"/>
+      <c r="G183" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H183" s="2" t="n">
+        <v>-1.071</v>
+      </c>
+      <c r="I183" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="J183" s="2" t="inlineStr">
+        <is>
+          <t>failed_breakdown</t>
+        </is>
+      </c>
+      <c r="K183" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="L183" s="2" t="n">
+        <v>0.08428031255431723</v>
+      </c>
+      <c r="M183" s="2" t="n">
+        <v>0.1178659751621098</v>
+      </c>
+      <c r="N183" s="2" t="n">
+        <v>1.723891825146658</v>
+      </c>
+      <c r="O183" s="2" t="n">
+        <v>0.002908591995585574</v>
+      </c>
+      <c r="P183" s="2" t="n">
+        <v>0.03310331281059654</v>
+      </c>
+      <c r="Q183" s="2" t="n">
+        <v>-0.0300444448207865</v>
+      </c>
+      <c r="R183" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S183" s="2" t="n">
+        <v>2.167830069086014</v>
+      </c>
+      <c r="T183" s="2" t="n">
+        <v>0.005460774206937247</v>
+      </c>
+      <c r="U183" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V183" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W183" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X183" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y183" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z183" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA183" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB183" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC183" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AD183" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE183" s="2" t="n">
+        <v>8.712999999999999</v>
+      </c>
+      <c r="AF183" s="2" t="n">
+        <v>0.263</v>
+      </c>
+      <c r="AG183" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AH183" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI183" s="2" t="n">
+        <v>8.712999999999999</v>
+      </c>
+      <c r="AJ183" s="2" t="n">
+        <v>0.263</v>
+      </c>
+      <c r="AK183" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AL183" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM183" s="2" t="n">
+        <v>8.712999999999999</v>
+      </c>
+      <c r="AN183" s="2" t="n">
+        <v>0.263</v>
+      </c>
+      <c r="AO183" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AP183" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ183" s="2" t="n">
+        <v>8.712999999999999</v>
+      </c>
+      <c r="AR183" s="2" t="n">
+        <v>0.263</v>
+      </c>
+      <c r="AS183" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AT183" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU183" s="2" t="n">
+        <v>8.712999999999999</v>
+      </c>
+      <c r="AV183" s="2" t="n">
+        <v>0.263</v>
+      </c>
+      <c r="AW183" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AX183" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY183" s="2" t="n">
+        <v>8.712999999999999</v>
+      </c>
+      <c r="AZ183" s="2" t="n">
+        <v>0.263</v>
+      </c>
+      <c r="BA183" s="2" t="n">
+        <v>0.0046</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B184" s="2" t="inlineStr">
+        <is>
+          <t>10:16</t>
+        </is>
+      </c>
+      <c r="C184" s="2" t="inlineStr">
+        <is>
+          <t>FUN</t>
+        </is>
+      </c>
+      <c r="D184" s="2" t="n">
+        <v>7.08</v>
+      </c>
+      <c r="E184" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26 10:15:00-04:00</t>
+        </is>
+      </c>
+      <c r="F184" s="2" t="n"/>
+      <c r="G184" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H184" s="2" t="n">
+        <v>-1.133</v>
+      </c>
+      <c r="I184" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="J184" s="2" t="inlineStr">
+        <is>
+          <t>bull_flag</t>
+        </is>
+      </c>
+      <c r="K184" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="L184" s="2" t="n">
+        <v>0.06646969136380299</v>
+      </c>
+      <c r="M184" s="2" t="n">
+        <v>-0.01033975950643906</v>
+      </c>
+      <c r="N184" s="2" t="n">
+        <v>0.7201696580534914</v>
+      </c>
+      <c r="O184" s="2" t="n">
+        <v>0.03651768772269892</v>
+      </c>
+      <c r="P184" s="2" t="n">
+        <v>0.01939055322159976</v>
+      </c>
+      <c r="Q184" s="2" t="n">
+        <v>-0.0006920573711997058</v>
+      </c>
+      <c r="R184" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S184" s="2" t="n">
+        <v>1.976854923845406</v>
+      </c>
+      <c r="T184" s="2" t="n">
+        <v>0.006500260052164641</v>
+      </c>
+      <c r="U184" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V184" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W184" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X184" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y184" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z184" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA184" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB184" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC184" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AD184" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE184" s="2" t="n">
+        <v>7.21</v>
+      </c>
+      <c r="AF184" s="2" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="AG184" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AH184" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI184" s="2" t="n">
+        <v>7.21</v>
+      </c>
+      <c r="AJ184" s="2" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="AK184" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AL184" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM184" s="2" t="n">
+        <v>7.21</v>
+      </c>
+      <c r="AN184" s="2" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="AO184" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AP184" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ184" s="2" t="n">
+        <v>7.21</v>
+      </c>
+      <c r="AR184" s="2" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="AS184" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AT184" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU184" s="2" t="n">
+        <v>7.21</v>
+      </c>
+      <c r="AV184" s="2" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="AW184" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AX184" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY184" s="2" t="n">
+        <v>7.21</v>
+      </c>
+      <c r="AZ184" s="2" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="BA184" s="2" t="n">
+        <v>0.00277</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B185" s="2" t="inlineStr">
+        <is>
+          <t>10:18</t>
+        </is>
+      </c>
+      <c r="C185" s="2" t="inlineStr">
+        <is>
+          <t>WGS</t>
+        </is>
+      </c>
+      <c r="D185" s="2" t="n">
+        <v>61.14</v>
+      </c>
+      <c r="E185" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26 10:17:00-04:00</t>
+        </is>
+      </c>
+      <c r="F185" s="2" t="n"/>
+      <c r="G185" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H185" s="2" t="n">
+        <v>-1.162</v>
+      </c>
+      <c r="I185" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="J185" s="2" t="inlineStr">
+        <is>
+          <t>bull_flag</t>
+        </is>
+      </c>
+      <c r="K185" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="L185" s="2" t="n">
+        <v>0.104185188159343</v>
+      </c>
+      <c r="M185" s="2" t="n">
+        <v>0.0331254985771825</v>
+      </c>
+      <c r="N185" s="2" t="n">
+        <v>1.149831571205187</v>
+      </c>
+      <c r="O185" s="2" t="n">
+        <v>0.01936109462953683</v>
+      </c>
+      <c r="P185" s="2" t="n">
+        <v>0.01387096774193547</v>
+      </c>
+      <c r="Q185" s="2" t="n">
+        <v>-0.0157168066691008</v>
+      </c>
+      <c r="R185" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S185" s="2" t="n">
+        <v>4.127134385045092</v>
+      </c>
+      <c r="T185" s="2" t="n">
+        <v>0.006724010926367097</v>
+      </c>
+      <c r="U185" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V185" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W185" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X185" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y185" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z185" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA185" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB185" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC185" s="2" t="n">
+        <v>-1.0646</v>
+      </c>
+      <c r="AD185" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE185" s="2" t="n">
+        <v>61.9135</v>
+      </c>
+      <c r="AF185" s="2" t="n">
+        <v>0.7735</v>
+      </c>
+      <c r="AG185" s="2" t="n">
+        <v>-1.0646</v>
+      </c>
+      <c r="AH185" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI185" s="2" t="n">
+        <v>61.9135</v>
+      </c>
+      <c r="AJ185" s="2" t="n">
+        <v>0.7735</v>
+      </c>
+      <c r="AK185" s="2" t="n">
+        <v>-1.0646</v>
+      </c>
+      <c r="AL185" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM185" s="2" t="n">
+        <v>61.9135</v>
+      </c>
+      <c r="AN185" s="2" t="n">
+        <v>0.7735</v>
+      </c>
+      <c r="AO185" s="2" t="n">
+        <v>-1.0646</v>
+      </c>
+      <c r="AP185" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ185" s="2" t="n">
+        <v>61.9135</v>
+      </c>
+      <c r="AR185" s="2" t="n">
+        <v>0.7735</v>
+      </c>
+      <c r="AS185" s="2" t="n">
+        <v>-1.0646</v>
+      </c>
+      <c r="AT185" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU185" s="2" t="n">
+        <v>61.9135</v>
+      </c>
+      <c r="AV185" s="2" t="n">
+        <v>0.7735</v>
+      </c>
+      <c r="AW185" s="2" t="n">
+        <v>-1.0646</v>
+      </c>
+      <c r="AX185" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY185" s="2" t="n">
+        <v>61.9135</v>
+      </c>
+      <c r="AZ185" s="2" t="n">
+        <v>0.7735</v>
+      </c>
+      <c r="BA185" s="2" t="n"/>
+    </row>
+    <row r="186">
+      <c r="A186" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B186" s="2" t="inlineStr">
+        <is>
+          <t>10:28</t>
+        </is>
+      </c>
+      <c r="C186" s="2" t="inlineStr">
+        <is>
+          <t>ORKA</t>
+        </is>
+      </c>
+      <c r="D186" s="2" t="n">
+        <v>88.95999999999999</v>
+      </c>
+      <c r="E186" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26 10:27:00-04:00</t>
+        </is>
+      </c>
+      <c r="F186" s="2" t="n"/>
+      <c r="G186" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H186" s="2" t="n">
+        <v>-1.222</v>
+      </c>
+      <c r="I186" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="J186" s="2" t="inlineStr">
+        <is>
+          <t>ema_bounce</t>
+        </is>
+      </c>
+      <c r="K186" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="L186" s="2" t="n">
+        <v>0.120024890006788</v>
+      </c>
+      <c r="M186" s="2" t="n">
+        <v>0.02283221205509034</v>
+      </c>
+      <c r="N186" s="2" t="n">
+        <v>1.404396649159392</v>
+      </c>
+      <c r="O186" s="2" t="n">
+        <v>0.01355336678127106</v>
+      </c>
+      <c r="P186" s="2" t="n">
+        <v>0.009023021870960206</v>
+      </c>
+      <c r="Q186" s="2" t="n">
+        <v>-0.01976419689669096</v>
+      </c>
+      <c r="R186" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S186" s="2" t="n">
+        <v>4.49725080637377</v>
+      </c>
+      <c r="T186" s="2" t="n">
+        <v>0.006171299685785003</v>
+      </c>
+      <c r="U186" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V186" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="W186" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="X186" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y186" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z186" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA186" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB186" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC186" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AD186" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE186" s="2" t="n">
+        <v>89.41500000000001</v>
+      </c>
+      <c r="AF186" s="2" t="n">
+        <v>0.455</v>
+      </c>
+      <c r="AG186" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AH186" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI186" s="2" t="n">
+        <v>89.41500000000001</v>
+      </c>
+      <c r="AJ186" s="2" t="n">
+        <v>0.455</v>
+      </c>
+      <c r="AK186" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AL186" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM186" s="2" t="n">
+        <v>89.41500000000001</v>
+      </c>
+      <c r="AN186" s="2" t="n">
+        <v>0.455</v>
+      </c>
+      <c r="AO186" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AP186" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ186" s="2" t="n">
+        <v>89.41500000000001</v>
+      </c>
+      <c r="AR186" s="2" t="n">
+        <v>0.455</v>
+      </c>
+      <c r="AS186" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AT186" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU186" s="2" t="n">
+        <v>89.41500000000001</v>
+      </c>
+      <c r="AV186" s="2" t="n">
+        <v>0.455</v>
+      </c>
+      <c r="AW186" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AX186" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY186" s="2" t="n">
+        <v>89.41500000000001</v>
+      </c>
+      <c r="AZ186" s="2" t="n">
+        <v>0.455</v>
+      </c>
+      <c r="BA186" s="2" t="n">
+        <v>0.007939999999999999</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B187" s="2" t="inlineStr">
+        <is>
+          <t>14:54</t>
+        </is>
+      </c>
+      <c r="C187" s="2" t="inlineStr">
+        <is>
+          <t>RRC</t>
+        </is>
+      </c>
+      <c r="D187" s="2" t="n">
+        <v>53.17</v>
+      </c>
+      <c r="E187" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26 14:53:00-04:00</t>
+        </is>
+      </c>
+      <c r="F187" s="2" t="n"/>
+      <c r="G187" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H187" s="2" t="n">
+        <v>-1.195</v>
+      </c>
+      <c r="I187" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="J187" s="2" t="inlineStr">
+        <is>
+          <t>ema_bounce</t>
+        </is>
+      </c>
+      <c r="K187" s="2" t="n">
+        <v>324</v>
+      </c>
+      <c r="L187" s="2" t="n">
+        <v>0.1750878985183271</v>
+      </c>
+      <c r="M187" s="2" t="n">
+        <v>0.1161028074311174</v>
+      </c>
+      <c r="N187" s="2" t="n">
+        <v>2.2519033723006</v>
+      </c>
+      <c r="O187" s="2" t="n">
+        <v>0.01757123318532017</v>
+      </c>
+      <c r="P187" s="2" t="n">
+        <v>0.005982457813150838</v>
+      </c>
+      <c r="Q187" s="2" t="n">
+        <v>-0.001493336136142442</v>
+      </c>
+      <c r="R187" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S187" s="2" t="n">
+        <v>3.979494751922235</v>
+      </c>
+      <c r="T187" s="2" t="n">
+        <v>0.006895076741891826</v>
+      </c>
+      <c r="U187" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V187" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W187" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X187" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y187" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z187" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA187" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB187" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC187" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AD187" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE187" s="2" t="n">
+        <v>53.5</v>
+      </c>
+      <c r="AF187" s="2" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="AG187" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AH187" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI187" s="2" t="n">
+        <v>53.5</v>
+      </c>
+      <c r="AJ187" s="2" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="AK187" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AL187" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM187" s="2" t="n">
+        <v>53.5</v>
+      </c>
+      <c r="AN187" s="2" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="AO187" s="2" t="n"/>
+      <c r="AP187" s="2" t="n"/>
+      <c r="AQ187" s="2" t="n"/>
+      <c r="AR187" s="2" t="n"/>
+      <c r="AS187" s="2" t="n"/>
+      <c r="AT187" s="2" t="n"/>
+      <c r="AU187" s="2" t="n"/>
+      <c r="AV187" s="2" t="n"/>
+      <c r="AW187" s="2" t="n"/>
+      <c r="AX187" s="2" t="n"/>
+      <c r="AY187" s="2" t="n"/>
+      <c r="AZ187" s="2" t="n"/>
+      <c r="BA187" s="2" t="n">
+        <v>0.00019</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B188" s="2" t="inlineStr">
+        <is>
+          <t>14:54</t>
+        </is>
+      </c>
+      <c r="C188" s="2" t="inlineStr">
+        <is>
+          <t>SGRY</t>
+        </is>
+      </c>
+      <c r="D188" s="2" t="n">
+        <v>23.06</v>
+      </c>
+      <c r="E188" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26 14:53:00-04:00</t>
+        </is>
+      </c>
+      <c r="F188" s="2" t="n"/>
+      <c r="G188" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H188" s="2" t="n">
+        <v>0.061</v>
+      </c>
+      <c r="I188" s="2" t="inlineStr">
+        <is>
+          <t>time</t>
+        </is>
+      </c>
+      <c r="J188" s="2" t="inlineStr">
+        <is>
+          <t>ema_bounce</t>
+        </is>
+      </c>
+      <c r="K188" s="2" t="n">
+        <v>324</v>
+      </c>
+      <c r="L188" s="2" t="n">
+        <v>0.4726983933221727</v>
+      </c>
+      <c r="M188" s="2" t="n">
+        <v>0.4622222658187625</v>
+      </c>
+      <c r="N188" s="2" t="n">
+        <v>3.638482627395722</v>
+      </c>
+      <c r="O188" s="2" t="n">
+        <v>0.006791416851420262</v>
+      </c>
+      <c r="P188" s="2" t="n">
+        <v>0.005820206794585307</v>
+      </c>
+      <c r="Q188" s="2" t="n">
+        <v>-0.003646918750202732</v>
+      </c>
+      <c r="R188" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S188" s="2" t="n">
+        <v>3.143936725046743</v>
+      </c>
+      <c r="T188" s="2" t="n">
+        <v>0.006895076741891826</v>
+      </c>
+      <c r="U188" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V188" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W188" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X188" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y188" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z188" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA188" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB188" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC188" s="2" t="n">
+        <v>0.5185</v>
+      </c>
+      <c r="AD188" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE188" s="2" t="n">
+        <v>23.195</v>
+      </c>
+      <c r="AF188" s="2" t="n">
+        <v>0.135</v>
+      </c>
+      <c r="AG188" s="2" t="n">
+        <v>0.5185</v>
+      </c>
+      <c r="AH188" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI188" s="2" t="n">
+        <v>23.195</v>
+      </c>
+      <c r="AJ188" s="2" t="n">
+        <v>0.135</v>
+      </c>
+      <c r="AK188" s="2" t="n">
+        <v>0.5185</v>
+      </c>
+      <c r="AL188" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM188" s="2" t="n">
+        <v>23.195</v>
+      </c>
+      <c r="AN188" s="2" t="n">
+        <v>0.135</v>
+      </c>
+      <c r="AO188" s="2" t="n">
+        <v>0.5185</v>
+      </c>
+      <c r="AP188" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ188" s="2" t="n">
+        <v>23.195</v>
+      </c>
+      <c r="AR188" s="2" t="n">
+        <v>0.135</v>
+      </c>
+      <c r="AS188" s="2" t="n">
+        <v>0.5185</v>
+      </c>
+      <c r="AT188" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU188" s="2" t="n">
+        <v>23.195</v>
+      </c>
+      <c r="AV188" s="2" t="n">
+        <v>0.135</v>
+      </c>
+      <c r="AW188" s="2" t="n">
+        <v>0.5185</v>
+      </c>
+      <c r="AX188" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY188" s="2" t="n">
+        <v>23.195</v>
+      </c>
+      <c r="AZ188" s="2" t="n">
+        <v>0.135</v>
+      </c>
+      <c r="BA188" s="2" t="n"/>
+    </row>
+    <row r="189">
+      <c r="A189" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B189" s="2" t="inlineStr">
+        <is>
+          <t>14:56</t>
+        </is>
+      </c>
+      <c r="C189" s="2" t="inlineStr">
+        <is>
+          <t>LQDA</t>
+        </is>
+      </c>
+      <c r="D189" s="2" t="n">
+        <v>44.15</v>
+      </c>
+      <c r="E189" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26 14:55:00-04:00</t>
+        </is>
+      </c>
+      <c r="F189" s="2" t="n"/>
+      <c r="G189" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H189" s="2" t="n">
+        <v>-1.169</v>
+      </c>
+      <c r="I189" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="J189" s="2" t="inlineStr">
+        <is>
+          <t>ema_bounce</t>
+        </is>
+      </c>
+      <c r="K189" s="2" t="n">
+        <v>326</v>
+      </c>
+      <c r="L189" s="2" t="n">
+        <v>0.04337628154593531</v>
+      </c>
+      <c r="M189" s="2" t="n">
+        <v>0.002813573917739509</v>
+      </c>
+      <c r="N189" s="2" t="n">
+        <v>0.3896937488550453</v>
+      </c>
+      <c r="O189" s="2" t="n">
+        <v>0.004703027740371679</v>
+      </c>
+      <c r="P189" s="2" t="n">
+        <v>0.007865168539325874</v>
+      </c>
+      <c r="Q189" s="2" t="n">
+        <v>-0.02668419046652781</v>
+      </c>
+      <c r="R189" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S189" s="2" t="n">
+        <v>3.795489189172195</v>
+      </c>
+      <c r="T189" s="2" t="n">
+        <v>0.006770030040121</v>
+      </c>
+      <c r="U189" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V189" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W189" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X189" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y189" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z189" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA189" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB189" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC189" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AD189" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE189" s="2" t="n">
+        <v>44.495</v>
+      </c>
+      <c r="AF189" s="2" t="n">
+        <v>0.345</v>
+      </c>
+      <c r="AG189" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AH189" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI189" s="2" t="n">
+        <v>44.495</v>
+      </c>
+      <c r="AJ189" s="2" t="n">
+        <v>0.345</v>
+      </c>
+      <c r="AK189" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AL189" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM189" s="2" t="n">
+        <v>44.495</v>
+      </c>
+      <c r="AN189" s="2" t="n">
+        <v>0.345</v>
+      </c>
+      <c r="AO189" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AP189" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ189" s="2" t="n">
+        <v>44.495</v>
+      </c>
+      <c r="AR189" s="2" t="n">
+        <v>0.345</v>
+      </c>
+      <c r="AS189" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AT189" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU189" s="2" t="n">
+        <v>44.495</v>
+      </c>
+      <c r="AV189" s="2" t="n">
+        <v>0.345</v>
+      </c>
+      <c r="AW189" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AX189" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY189" s="2" t="n">
+        <v>44.495</v>
+      </c>
+      <c r="AZ189" s="2" t="n">
+        <v>0.345</v>
+      </c>
+      <c r="BA189" s="2" t="n">
+        <v>0.00157</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B190" s="2" t="inlineStr">
+        <is>
+          <t>14:57</t>
+        </is>
+      </c>
+      <c r="C190" s="2" t="inlineStr">
+        <is>
+          <t>RRC</t>
+        </is>
+      </c>
+      <c r="D190" s="2" t="n">
+        <v>53.34</v>
+      </c>
+      <c r="E190" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26 14:56:00-04:00</t>
+        </is>
+      </c>
+      <c r="F190" s="2" t="n"/>
+      <c r="G190" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H190" s="2" t="n">
+        <v>-1.235</v>
+      </c>
+      <c r="I190" s="2" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="J190" s="2" t="inlineStr">
+        <is>
+          <t>afternoon_hod</t>
+        </is>
+      </c>
+      <c r="K190" s="2" t="n">
+        <v>327</v>
+      </c>
+      <c r="L190" s="2" t="n">
+        <v>0.1775043483106851</v>
+      </c>
+      <c r="M190" s="2" t="n">
+        <v>0.1161028074311174</v>
+      </c>
+      <c r="N190" s="2" t="n">
+        <v>2.249088733348406</v>
+      </c>
+      <c r="O190" s="2" t="n">
+        <v>0.01954759665499672</v>
+      </c>
+      <c r="P190" s="2" t="n">
+        <v>0.004850717938856316</v>
+      </c>
+      <c r="Q190" s="2" t="n">
+        <v>-0.0009301052993533343</v>
+      </c>
+      <c r="R190" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S190" s="2" t="n">
+        <v>3.981549039608866</v>
+      </c>
+      <c r="T190" s="2" t="n">
+        <v>0.00655294511084259</v>
+      </c>
+      <c r="U190" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V190" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W190" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X190" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y190" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z190" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA190" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB190" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC190" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AD190" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE190" s="2" t="n">
+        <v>53.6</v>
+      </c>
+      <c r="AF190" s="2" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="AG190" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AH190" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI190" s="2" t="n">
+        <v>53.6</v>
+      </c>
+      <c r="AJ190" s="2" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="AK190" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AL190" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM190" s="2" t="n">
+        <v>53.6</v>
+      </c>
+      <c r="AN190" s="2" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="AO190" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AP190" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ190" s="2" t="n">
+        <v>53.6</v>
+      </c>
+      <c r="AR190" s="2" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="AS190" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AT190" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU190" s="2" t="n">
+        <v>53.6</v>
+      </c>
+      <c r="AV190" s="2" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="AW190" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AX190" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY190" s="2" t="n">
+        <v>53.6</v>
+      </c>
+      <c r="AZ190" s="2" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="BA190" s="2" t="n">
+        <v>0.00037</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B191" s="2" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="C191" s="2" t="inlineStr">
+        <is>
+          <t>SGRY</t>
+        </is>
+      </c>
+      <c r="D191" s="2" t="n">
+        <v>23.17</v>
+      </c>
+      <c r="E191" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26 15:29:00-04:00</t>
+        </is>
+      </c>
+      <c r="F191" s="2" t="n"/>
+      <c r="G191" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H191" s="2" t="n"/>
+      <c r="I191" s="2" t="n"/>
+      <c r="J191" s="2" t="inlineStr">
+        <is>
+          <t>eod_squeeze</t>
+        </is>
+      </c>
+      <c r="K191" s="2" t="n">
+        <v>360</v>
+      </c>
+      <c r="L191" s="2" t="n">
+        <v>0.4752381339905754</v>
+      </c>
+      <c r="M191" s="2" t="n">
+        <v>0.4622222658187625</v>
+      </c>
+      <c r="N191" s="2" t="n">
+        <v>3.550366544529863</v>
+      </c>
+      <c r="O191" s="2" t="n">
+        <v>0.008413839157334513</v>
+      </c>
+      <c r="P191" s="2" t="n">
+        <v>0.002797529961010717</v>
+      </c>
+      <c r="Q191" s="2" t="n">
+        <v>-0.00192865895443417</v>
+      </c>
+      <c r="R191" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S191" s="2" t="n">
+        <v>3.145659788805569</v>
+      </c>
+      <c r="T191" s="2" t="n">
+        <v>0.007145089832843787</v>
+      </c>
+      <c r="U191" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V191" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W191" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X191" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y191" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z191" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA191" s="2" t="n"/>
+      <c r="AB191" s="2" t="n"/>
+      <c r="AC191" s="2" t="n"/>
+      <c r="AD191" s="2" t="n"/>
+      <c r="AE191" s="2" t="n"/>
+      <c r="AF191" s="2" t="n"/>
+      <c r="AG191" s="2" t="n"/>
+      <c r="AH191" s="2" t="n"/>
+      <c r="AI191" s="2" t="n"/>
+      <c r="AJ191" s="2" t="n"/>
+      <c r="AK191" s="2" t="n"/>
+      <c r="AL191" s="2" t="n"/>
+      <c r="AM191" s="2" t="n"/>
+      <c r="AN191" s="2" t="n"/>
+      <c r="AO191" s="2" t="n"/>
+      <c r="AP191" s="2" t="n"/>
+      <c r="AQ191" s="2" t="n"/>
+      <c r="AR191" s="2" t="n"/>
+      <c r="AS191" s="2" t="n"/>
+      <c r="AT191" s="2" t="n"/>
+      <c r="AU191" s="2" t="n"/>
+      <c r="AV191" s="2" t="n"/>
+      <c r="AW191" s="2" t="n"/>
+      <c r="AX191" s="2" t="n"/>
+      <c r="AY191" s="2" t="n"/>
+      <c r="AZ191" s="2" t="n"/>
+      <c r="BA191" s="2" t="n"/>
+    </row>
+    <row r="192">
+      <c r="A192" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B192" s="2" t="inlineStr">
+        <is>
+          <t>15:34</t>
+        </is>
+      </c>
+      <c r="C192" s="2" t="inlineStr">
+        <is>
+          <t>RRC</t>
+        </is>
+      </c>
+      <c r="D192" s="2" t="n">
+        <v>52.77</v>
+      </c>
+      <c r="E192" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26 15:33:00-04:00</t>
+        </is>
+      </c>
+      <c r="F192" s="2" t="n"/>
+      <c r="G192" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H192" s="2" t="n"/>
+      <c r="I192" s="2" t="n"/>
+      <c r="J192" s="2" t="inlineStr">
+        <is>
+          <t>eod_squeeze</t>
+        </is>
+      </c>
+      <c r="K192" s="2" t="n">
+        <v>364</v>
+      </c>
+      <c r="L192" s="2" t="n">
+        <v>0.1673989203702904</v>
+      </c>
+      <c r="M192" s="2" t="n">
+        <v>0.1161028074311174</v>
+      </c>
+      <c r="N192" s="2" t="n">
+        <v>2.255532732504951</v>
+      </c>
+      <c r="O192" s="2" t="n">
+        <v>0.009491641027011388</v>
+      </c>
+      <c r="P192" s="2" t="n">
+        <v>0.006962728526498807</v>
+      </c>
+      <c r="Q192" s="2" t="n">
+        <v>-0.009506097329456065</v>
+      </c>
+      <c r="R192" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S192" s="2" t="n">
+        <v>3.97292992884594</v>
+      </c>
+      <c r="T192" s="2" t="n">
+        <v>0.007460878934553827</v>
+      </c>
+      <c r="U192" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V192" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W192" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X192" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y192" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z192" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA192" s="2" t="n"/>
+      <c r="AB192" s="2" t="n"/>
+      <c r="AC192" s="2" t="n"/>
+      <c r="AD192" s="2" t="n"/>
+      <c r="AE192" s="2" t="n"/>
+      <c r="AF192" s="2" t="n"/>
+      <c r="AG192" s="2" t="n"/>
+      <c r="AH192" s="2" t="n"/>
+      <c r="AI192" s="2" t="n"/>
+      <c r="AJ192" s="2" t="n"/>
+      <c r="AK192" s="2" t="n"/>
+      <c r="AL192" s="2" t="n"/>
+      <c r="AM192" s="2" t="n"/>
+      <c r="AN192" s="2" t="n"/>
+      <c r="AO192" s="2" t="n"/>
+      <c r="AP192" s="2" t="n"/>
+      <c r="AQ192" s="2" t="n"/>
+      <c r="AR192" s="2" t="n"/>
+      <c r="AS192" s="2" t="n"/>
+      <c r="AT192" s="2" t="n"/>
+      <c r="AU192" s="2" t="n"/>
+      <c r="AV192" s="2" t="n"/>
+      <c r="AW192" s="2" t="n"/>
+      <c r="AX192" s="2" t="n"/>
+      <c r="AY192" s="2" t="n"/>
+      <c r="AZ192" s="2" t="n"/>
+      <c r="BA192" s="2" t="n"/>
+    </row>
+    <row r="193">
+      <c r="A193" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B193" s="2" t="inlineStr">
+        <is>
+          <t>15:35</t>
+        </is>
+      </c>
+      <c r="C193" s="2" t="inlineStr">
+        <is>
+          <t>HHH</t>
+        </is>
+      </c>
+      <c r="D193" s="2" t="n">
+        <v>73.84</v>
+      </c>
+      <c r="E193" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26 15:34:00-04:00</t>
+        </is>
+      </c>
+      <c r="F193" s="2" t="n"/>
+      <c r="G193" s="2" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H193" s="2" t="n"/>
+      <c r="I193" s="2" t="n"/>
+      <c r="J193" s="2" t="inlineStr">
+        <is>
+          <t>eod_squeeze</t>
+        </is>
+      </c>
+      <c r="K193" s="2" t="n">
+        <v>365</v>
+      </c>
+      <c r="L193" s="2" t="n">
+        <v>0.0564894742837565</v>
+      </c>
+      <c r="M193" s="2" t="n">
+        <v>0.0423137358227399</v>
+      </c>
+      <c r="N193" s="2" t="n">
+        <v>1.552916954684296</v>
+      </c>
+      <c r="O193" s="2" t="n">
+        <v>0.008070308029459294</v>
+      </c>
+      <c r="P193" s="2" t="n">
+        <v>0.004247842822226776</v>
+      </c>
+      <c r="Q193" s="2" t="n">
+        <v>-0.009946631927966298</v>
+      </c>
+      <c r="R193" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S193" s="2" t="n">
+        <v>4.306157480732418</v>
+      </c>
+      <c r="T193" s="2" t="n">
+        <v>0.007579259691400386</v>
+      </c>
+      <c r="U193" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V193" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W193" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X193" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y193" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z193" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA193" s="2" t="n"/>
+      <c r="AB193" s="2" t="n"/>
+      <c r="AC193" s="2" t="n"/>
+      <c r="AD193" s="2" t="n"/>
+      <c r="AE193" s="2" t="n"/>
+      <c r="AF193" s="2" t="n"/>
+      <c r="AG193" s="2" t="n"/>
+      <c r="AH193" s="2" t="n"/>
+      <c r="AI193" s="2" t="n"/>
+      <c r="AJ193" s="2" t="n"/>
+      <c r="AK193" s="2" t="n"/>
+      <c r="AL193" s="2" t="n"/>
+      <c r="AM193" s="2" t="n"/>
+      <c r="AN193" s="2" t="n"/>
+      <c r="AO193" s="2" t="n"/>
+      <c r="AP193" s="2" t="n"/>
+      <c r="AQ193" s="2" t="n"/>
+      <c r="AR193" s="2" t="n"/>
+      <c r="AS193" s="2" t="n"/>
+      <c r="AT193" s="2" t="n"/>
+      <c r="AU193" s="2" t="n"/>
+      <c r="AV193" s="2" t="n"/>
+      <c r="AW193" s="2" t="n"/>
+      <c r="AX193" s="2" t="n"/>
+      <c r="AY193" s="2" t="n"/>
+      <c r="AZ193" s="2" t="n"/>
+      <c r="BA193" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -31760,7 +35945,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J39"/>
+  <dimension ref="A1:J44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -33288,6 +37473,194 @@
       <c r="J39" s="2" t="inlineStr">
         <is>
           <t>closed</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="n">
+        <v>350</v>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>bull_flag</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>EAF</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="n">
+        <v>-3.78</v>
+      </c>
+      <c r="F40" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="G40" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="H40" s="2" t="n">
+        <v>10.26</v>
+      </c>
+      <c r="I40" s="2" t="n">
+        <v>-3.27</v>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>orb15</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>CORT</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="n">
+        <v>-9.42</v>
+      </c>
+      <c r="F41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" s="2" t="n"/>
+      <c r="I41" s="2" t="n"/>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>no fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="n">
+        <v>250</v>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>orb15</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>MLCO</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="n">
+        <v>-2.04</v>
+      </c>
+      <c r="F42" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="G42" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H42" s="2" t="n">
+        <v>3.97</v>
+      </c>
+      <c r="I42" s="2" t="n"/>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>partially open</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>orb5</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>BWMX</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="n">
+        <v>-2.46</v>
+      </c>
+      <c r="F43" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G43" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" s="2" t="n"/>
+      <c r="I43" s="2" t="n"/>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>no fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="n">
+        <v>550</v>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>pm_high_break</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>RRC</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="F44" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="G44" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H44" s="2" t="n">
+        <v>52.885</v>
+      </c>
+      <c r="I44" s="2" t="n"/>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>partially open</t>
         </is>
       </c>
     </row>

</xml_diff>